<commit_message>
BOM: CNC tab — a listing link on every line, Link column visible
- 44 of 46 lines now carry a candidate listing (AliExpress, Amazon.ca, Home Depot, grblHAL); the 2 Have lines need none
- Vendor/ref updated with the listing IDs; notes expanded on the router, collet, VFD spindle and wiring lines
- Link column moved out of the hidden group so it shows at the right of the tab

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZTgn2wDHFLcnBAkTFZVua
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4437" uniqueCount="1109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4463" uniqueCount="1149">
   <si>
     <t xml:space="preserve">07K ZN6 Turbo Swap — Cost Summary</t>
   </si>
@@ -2832,7 +2832,7 @@
     <t xml:space="preserve">07K ZN6 — CNC mill BOM (HTMCNC-style, 450 x 750 x 110 mm work area)</t>
   </si>
   <si>
-    <t xml:space="preserve">Same rules as the BOM tab. Blue column H = your real price (CAD). Lines with NO price are undecided: fill D/E with an estimate or H with the real price once you pick a listing. Decided so far (Oct 4, 2026): motor/driver/supply kit (Amazon), extrusion (Amazon). Have: Arduino UNO, filament. Candidate AliExpress listings are in the Link column; prices for those are NOT entered on purpose.</t>
+    <t xml:space="preserve">Same rules as the BOM tab. Blue column H = your real price (CAD). Lines with NO price are undecided: fill D/E with an estimate or H with the real price once you pick a listing. Decided so far (Oct 4, 2026): motor/driver/supply kit (Amazon), extrusion (Amazon). Have: Arduino UNO, filament. Every line has a candidate listing in the Link column at the far right (click to open); columns L–W with the notes are grouped — click the + above them to expand.</t>
   </si>
   <si>
     <t xml:space="preserve">2040 T-slot extrusion, 1000 mm, black — VEVOR 5-pack</t>
@@ -2928,10 +2928,13 @@
     <t xml:space="preserve">Socket-head bolt kit (author's list)</t>
   </si>
   <si>
-    <t xml:space="preserve">M3x12 ×10, M3x16 ×5, M3x30 ×5, M4x10 ×5, M4x12 ×5, M4x14 ×60, M4x25 ×10, M5x12 ×50, M5x16 ×40, M5x20 ×40, M5x30 ×40, M5x50 ×25, M5x60 ×35, M5x70 ×5. Cheapest as an assorted M4/M5 kit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amazon / AliExpress</t>
+    <t xml:space="preserve">Pick the sizes from the list; 304 DIN912. Or an assorted M4/M5 kit on Amazon.ca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 32968483467</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/32968483467.html</t>
   </si>
   <si>
     <t xml:space="preserve">HGR15 linear rail 1000 mm + 2 HGH15CA blocks (Y)</t>
@@ -3033,10 +3036,13 @@
     <t xml:space="preserve">M12x1 locknut (ballscrew end)</t>
   </si>
   <si>
-    <t xml:space="preserve">Also included in BK12 support kits.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress</t>
+    <t xml:space="preserve">BK12 lock nut listing; M12x1 for the 1605 screw end.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 4000909595284</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/4000909595284.html</t>
   </si>
   <si>
     <t xml:space="preserve">C19</t>
@@ -3126,6 +3132,15 @@
     <t xml:space="preserve">E-stop button, NC</t>
   </si>
   <si>
+    <t xml:space="preserve">22 mm metal, 2NO 2NC, latching.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005001806206333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005001806206333.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">C25</t>
   </si>
   <si>
@@ -3135,25 +3150,40 @@
     <t xml:space="preserve">Wiring</t>
   </si>
   <si>
-    <t xml:space="preserve">Author used double-shielded; ground the shield at the box only.</t>
+    <t xml:space="preserve">Pick the 4-core 22AWG shielded option. Author used double-shielded; ground the shield at the box only.</t>
   </si>
   <si>
     <t xml:space="preserve">m</t>
   </si>
   <si>
+    <t xml:space="preserve">AliExpress 4000564582198</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/4000564582198.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">C26</t>
   </si>
   <si>
     <t xml:space="preserve">Shielded 2-wire cable, limit switches</t>
   </si>
   <si>
+    <t xml:space="preserve">Same listing, 2-core 24AWG shielded.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C27</t>
   </si>
   <si>
     <t xml:space="preserve">Drag chain 10x20 + end mounts</t>
   </si>
   <si>
-    <t xml:space="preserve">X and Y runs.</t>
+    <t xml:space="preserve">Open bridge type, 10x20, 1 m lengths. X and Y runs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005001795469984</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005001795469984.html</t>
   </si>
   <si>
     <t xml:space="preserve">C28</t>
@@ -3162,6 +3192,15 @@
     <t xml:space="preserve">Terminal blocks, ferrules, USB cable, hookup wire</t>
   </si>
   <si>
+    <t xml:space="preserve">Ratchet ferrule crimper + ferrule kit. Terminal strips and USB cable from Amazon.ca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005007097035466</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005007097035466.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">C29</t>
   </si>
   <si>
@@ -3171,7 +3210,13 @@
     <t xml:space="preserve">Control box</t>
   </si>
   <si>
-    <t xml:space="preserve">Author's metal enclosure + GX16 connectors cost ~US$500; an open panel does the job.</t>
+    <t xml:space="preserve">Author's metal enclosure + GX16 connectors cost ~US$500; a plywood panel does the job.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home Depot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.homedepot.ca/search?q=plywood%201%2F2</t>
   </si>
   <si>
     <t xml:space="preserve">C30</t>
@@ -3180,7 +3225,13 @@
     <t xml:space="preserve">12 V fan + DC-DC converter for the box</t>
   </si>
   <si>
-    <t xml:space="preserve">Only if the drivers go in a closed box.</t>
+    <t xml:space="preserve">36 V → 12 V 3 A buck module. Add any 80 mm 12 V fan. Only if the drivers go in a closed box.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005007181838501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005007181838501.html</t>
   </si>
   <si>
     <t xml:space="preserve">C31</t>
@@ -3189,7 +3240,13 @@
     <t xml:space="preserve">Ethernet CNC controller (grblHAL Teensy 4.1 + breakout) — EMI fix</t>
   </si>
   <si>
-    <t xml:space="preserve">Author could not fully stop USB/EMI false alarms on Arduino+GRBL. Upgrade path, not needed to start.</t>
+    <t xml:space="preserve">Author could not fully stop USB/EMI false alarms on Arduino+GRBL. Ethernet upgrade path, not needed to start.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">grblHAL Teensy 4.1 breakout (PCBWay) + Teensy 4.1 (pjrc.com)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/phil-barrett/grblHAL-teensy-4.x</t>
   </si>
   <si>
     <t xml:space="preserve">C32</t>
@@ -3204,10 +3261,13 @@
     <t xml:space="preserve">Router</t>
   </si>
   <si>
-    <t xml:space="preserve">New vs used vs 65 mm clone. The printed mount is sized for the 65 mm Makita body; the Craftsman does not fit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home Depot / Amazon.ca / Marketplace</t>
+    <t xml:space="preserve">New vs used vs 65 mm clone. Bare RT0701C is the one to buy; the CX7 kit (B00HAQMHEO) adds bases you don't need. The printed mount is sized for the 65 mm Makita body; the Craftsman does not fit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon B00E7D3V4S (bare tool) / Home Depot.ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.ca/dp/B00E7D3V4S</t>
   </si>
   <si>
     <t xml:space="preserve">C33</t>
@@ -3216,7 +3276,13 @@
     <t xml:space="preserve">6 mm collet for RT0701C</t>
   </si>
   <si>
-    <t xml:space="preserve">Router ships with 1/4 in only.</t>
+    <t xml:space="preserve">Router ships with the 1/4 in cone (763637-1) only. Buy the genuine 6 mm cone, not a sleeve adapter (adds runout).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon.ca search; Makita part 763636-3 (verify)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.ca/makita-rt0701c-collet/s?k=makita+rt0701c+collet</t>
   </si>
   <si>
     <t xml:space="preserve">C34</t>
@@ -3228,7 +3294,13 @@
     <t xml:space="preserve">Upgrade</t>
   </si>
   <si>
-    <t xml:space="preserve">Author moved to a 2.2 kW VFD spindle for runout; do this before the gearbox adapter plate.</t>
+    <t xml:space="preserve">2.2 kW ER20 air-cooled 80 mm round + VFD. Water-cooled kit with clamp: 1005003968400625. Author moved to a 2.2 kW VFD spindle for runout; do this before the gearbox adapter plate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005008081995923</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005008081995923.html</t>
   </si>
   <si>
     <t xml:space="preserve">C35</t>
@@ -3237,7 +3309,13 @@
     <t xml:space="preserve">80 mm spindle mount (if VFD spindle)</t>
   </si>
   <si>
-    <t xml:space="preserve">Machine it on the CNC itself.</t>
+    <t xml:space="preserve">80 mm clamp if you'd rather buy it than machine it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005009168636967</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005009168636967.html</t>
   </si>
   <si>
     <t xml:space="preserve">C36</t>
@@ -3285,7 +3363,7 @@
     <t xml:space="preserve">Surface it with the machine once running.</t>
   </si>
   <si>
-    <t xml:space="preserve">Home Depot</t>
+    <t xml:space="preserve">https://www.homedepot.ca/search?q=mdf%203%2F4</t>
   </si>
   <si>
     <t xml:space="preserve">C39</t>
@@ -3294,13 +3372,28 @@
     <t xml:space="preserve">Threaded inserts M6 (or T-track) for hold-downs</t>
   </si>
   <si>
+    <t xml:space="preserve">M6 hex-drive wood inserts, 100-pack.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005011942750737</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005011942750737.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">C40</t>
   </si>
   <si>
     <t xml:space="preserve">Clamps / hold-down set</t>
   </si>
   <si>
-    <t xml:space="preserve">Print the first set; machine aluminum ones later.</t>
+    <t xml:space="preserve">Arc press-plate clamps. Print the first set; machine aluminum ones later.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005005244930679</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005005244930679.html</t>
   </si>
   <si>
     <t xml:space="preserve">C41</t>
@@ -3342,7 +3435,13 @@
     <t xml:space="preserve">Setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Tramming, squareness, collet runout. Mark Have if you own one.</t>
+    <t xml:space="preserve">0.01 mm indicator with flexible magnetic base. Tramming, squareness, collet runout. Mark Have if you own one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005007169855682</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005007169855682.html</t>
   </si>
   <si>
     <t xml:space="preserve">C44</t>
@@ -3351,13 +3450,25 @@
     <t xml:space="preserve">Z touch plate / probe</t>
   </si>
   <si>
+    <t xml:space="preserve">AliExpress 1005008660120770</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005008660120770.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">C45</t>
   </si>
   <si>
     <t xml:space="preserve">Air blast or mist setup (isopropyl / WD-40) for aluminum</t>
   </si>
   <si>
-    <t xml:space="preserve">Stops chip welding on the single-flute cutters.</t>
+    <t xml:space="preserve">Pneumatic mist sprayer, magnetic base. Stops chip welding on the single-flute cutters.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress 1005008490356061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aliexpress.com/item/1005008490356061.html</t>
   </si>
   <si>
     <t xml:space="preserve">C46</t>
@@ -3370,6 +3481,15 @@
   </si>
   <si>
     <t xml:space="preserve">Consumables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NLGI 2 lithium grease for rails and screws; zip ties and heat shrink from the same order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon.ca / Canadian Tire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.ca/s?k=white+lithium+grease</t>
   </si>
   <si>
     <t xml:space="preserve">How to use this sheet</t>
@@ -3733,7 +3853,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="18">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3878,20 +3998,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2EFDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5083,12 +5189,12 @@
       <c r="D66" s="15"/>
       <c r="E66" s="15"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="5" t="s">
         <v>18</v>
       </c>
@@ -5102,7 +5208,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="3" t="s">
         <v>67</v>
       </c>
@@ -5119,7 +5225,7 @@
         <v>349.98</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="3" t="s">
         <v>51</v>
       </c>
@@ -5136,7 +5242,7 @@
         <v>349.98</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="3" t="s">
         <v>52</v>
       </c>
@@ -5153,7 +5259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B73" s="3" t="s">
         <v>53</v>
       </c>
@@ -5170,7 +5276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="3" t="s">
         <v>68</v>
       </c>
@@ -5187,12 +5293,12 @@
         <v>349.98</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="5" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="3" t="s">
         <v>70</v>
       </c>
@@ -5201,7 +5307,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="3" t="s">
         <v>71</v>
       </c>
@@ -5210,7 +5316,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B79" s="3" t="s">
         <v>59</v>
       </c>
@@ -5219,7 +5325,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="3" t="s">
         <v>72</v>
       </c>
@@ -5228,7 +5334,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B81" s="3" t="s">
         <v>61</v>
       </c>
@@ -5237,7 +5343,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B83" s="9" t="s">
         <v>73</v>
       </c>
@@ -22605,10 +22711,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="12" min="12" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="24" min="13" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="23" min="13" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>914</v>
       </c>
@@ -23319,14 +23426,16 @@
       <c r="W13" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X13" s="26"/>
+      <c r="X13" s="26" t="s">
+        <v>949</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
         <v>798</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="C14" s="20" t="n">
         <v>2</v>
@@ -23351,13 +23460,13 @@
         <v>103</v>
       </c>
       <c r="L14" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M14" s="24" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="N14" s="19" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="O14" s="18" t="s">
         <v>106</v>
@@ -23369,7 +23478,7 @@
         <v>44</v>
       </c>
       <c r="R14" s="24" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="S14" s="18" t="s">
         <v>922</v>
@@ -23387,7 +23496,7 @@
         <v>62</v>
       </c>
       <c r="X14" s="26" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23395,7 +23504,7 @@
         <v>802</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="C15" s="20" t="n">
         <v>2</v>
@@ -23420,13 +23529,13 @@
         <v>103</v>
       </c>
       <c r="L15" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M15" s="24" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="N15" s="19" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="O15" s="18" t="s">
         <v>106</v>
@@ -23438,7 +23547,7 @@
         <v>44</v>
       </c>
       <c r="R15" s="24" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="S15" s="18" t="s">
         <v>922</v>
@@ -23456,7 +23565,7 @@
         <v>62</v>
       </c>
       <c r="X15" s="26" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23464,7 +23573,7 @@
         <v>806</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="C16" s="20" t="n">
         <v>2</v>
@@ -23489,13 +23598,13 @@
         <v>103</v>
       </c>
       <c r="L16" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M16" s="24" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="N16" s="19" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="O16" s="18" t="s">
         <v>106</v>
@@ -23507,7 +23616,7 @@
         <v>44</v>
       </c>
       <c r="R16" s="24" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="S16" s="18" t="s">
         <v>922</v>
@@ -23525,7 +23634,7 @@
         <v>62</v>
       </c>
       <c r="X16" s="26" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23533,7 +23642,7 @@
         <v>808</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="C17" s="20" t="n">
         <v>2</v>
@@ -23558,13 +23667,13 @@
         <v>103</v>
       </c>
       <c r="L17" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M17" s="24" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="N17" s="19" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="O17" s="18" t="s">
         <v>106</v>
@@ -23576,7 +23685,7 @@
         <v>44</v>
       </c>
       <c r="R17" s="24" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="S17" s="18" t="s">
         <v>922</v>
@@ -23594,7 +23703,7 @@
         <v>62</v>
       </c>
       <c r="X17" s="26" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23602,7 +23711,7 @@
         <v>813</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="C18" s="20" t="n">
         <v>1</v>
@@ -23627,10 +23736,10 @@
         <v>103</v>
       </c>
       <c r="L18" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M18" s="24" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="N18" s="19"/>
       <c r="O18" s="18" t="s">
@@ -23643,7 +23752,7 @@
         <v>44</v>
       </c>
       <c r="R18" s="24" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="S18" s="18" t="s">
         <v>922</v>
@@ -23661,7 +23770,7 @@
         <v>62</v>
       </c>
       <c r="X18" s="26" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23669,7 +23778,7 @@
         <v>816</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="C19" s="20" t="n">
         <v>1</v>
@@ -23694,13 +23803,13 @@
         <v>103</v>
       </c>
       <c r="L19" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M19" s="24" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="N19" s="19" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="O19" s="18" t="s">
         <v>106</v>
@@ -23712,7 +23821,7 @@
         <v>44</v>
       </c>
       <c r="R19" s="24" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="S19" s="18" t="s">
         <v>922</v>
@@ -23730,7 +23839,7 @@
         <v>62</v>
       </c>
       <c r="X19" s="26" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23738,7 +23847,7 @@
         <v>818</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="C20" s="20" t="n">
         <v>4</v>
@@ -23763,16 +23872,16 @@
         <v>103</v>
       </c>
       <c r="L20" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M20" s="24" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="N20" s="19" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="O20" s="18" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="P20" s="20" t="s">
         <v>6</v>
@@ -23781,7 +23890,7 @@
         <v>44</v>
       </c>
       <c r="R20" s="24" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="S20" s="18" t="s">
         <v>922</v>
@@ -23799,15 +23908,15 @@
         <v>62</v>
       </c>
       <c r="X20" s="26" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="C21" s="20" t="n">
         <v>4</v>
@@ -23832,13 +23941,13 @@
         <v>103</v>
       </c>
       <c r="L21" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M21" s="24" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="N21" s="19" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="O21" s="18" t="s">
         <v>106</v>
@@ -23850,7 +23959,7 @@
         <v>44</v>
       </c>
       <c r="R21" s="24" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="S21" s="18" t="s">
         <v>922</v>
@@ -23868,15 +23977,15 @@
         <v>62</v>
       </c>
       <c r="X21" s="26" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="C22" s="20" t="n">
         <v>4</v>
@@ -23901,13 +24010,13 @@
         <v>103</v>
       </c>
       <c r="L22" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M22" s="24" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="N22" s="19" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="O22" s="18" t="s">
         <v>106</v>
@@ -23919,7 +24028,7 @@
         <v>44</v>
       </c>
       <c r="R22" s="24" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="S22" s="18" t="s">
         <v>922</v>
@@ -23936,14 +24045,16 @@
       <c r="W22" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X22" s="26"/>
+      <c r="X22" s="26" t="s">
+        <v>985</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>985</v>
+        <v>987</v>
       </c>
       <c r="C23" s="20" t="n">
         <v>4</v>
@@ -23968,13 +24079,13 @@
         <v>103</v>
       </c>
       <c r="L23" s="24" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="M23" s="24" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
       <c r="N23" s="19" t="s">
-        <v>987</v>
+        <v>989</v>
       </c>
       <c r="O23" s="18" t="s">
         <v>106</v>
@@ -23986,7 +24097,7 @@
         <v>44</v>
       </c>
       <c r="R23" s="24" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="S23" s="18" t="s">
         <v>922</v>
@@ -24004,15 +24115,15 @@
         <v>62</v>
       </c>
       <c r="X23" s="26" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>991</v>
+        <v>993</v>
       </c>
       <c r="C24" s="20" t="n">
         <v>1</v>
@@ -24039,13 +24150,13 @@
         <v>103</v>
       </c>
       <c r="L24" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M24" s="24" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="N24" s="19" t="s">
-        <v>994</v>
+        <v>996</v>
       </c>
       <c r="O24" s="18" t="s">
         <v>160</v>
@@ -24057,7 +24168,7 @@
         <v>44</v>
       </c>
       <c r="R24" s="24" t="s">
-        <v>995</v>
+        <v>997</v>
       </c>
       <c r="S24" s="18" t="s">
         <v>922</v>
@@ -24075,15 +24186,15 @@
         <v>219</v>
       </c>
       <c r="X24" s="26" t="s">
-        <v>996</v>
+        <v>998</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
       <c r="C25" s="20" t="n">
         <v>1</v>
@@ -24108,13 +24219,13 @@
         <v>103</v>
       </c>
       <c r="L25" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M25" s="24" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="N25" s="19" t="s">
-        <v>999</v>
+        <v>1001</v>
       </c>
       <c r="O25" s="18" t="s">
         <v>106</v>
@@ -24147,10 +24258,10 @@
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>1000</v>
+        <v>1002</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
       <c r="C26" s="20" t="n">
         <v>1</v>
@@ -24175,13 +24286,13 @@
         <v>103</v>
       </c>
       <c r="L26" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M26" s="24" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="N26" s="19" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="O26" s="18" t="s">
         <v>106</v>
@@ -24193,7 +24304,7 @@
         <v>44</v>
       </c>
       <c r="R26" s="24" t="s">
-        <v>1003</v>
+        <v>1005</v>
       </c>
       <c r="S26" s="18" t="s">
         <v>922</v>
@@ -24211,15 +24322,15 @@
         <v>62</v>
       </c>
       <c r="X26" s="26" t="s">
-        <v>1004</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>1005</v>
+        <v>1007</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>1006</v>
+        <v>1008</v>
       </c>
       <c r="C27" s="20" t="n">
         <v>6</v>
@@ -24244,13 +24355,13 @@
         <v>103</v>
       </c>
       <c r="L27" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M27" s="24" t="s">
-        <v>1007</v>
+        <v>1009</v>
       </c>
       <c r="N27" s="19" t="s">
-        <v>1008</v>
+        <v>1010</v>
       </c>
       <c r="O27" s="18" t="s">
         <v>106</v>
@@ -24262,7 +24373,7 @@
         <v>44</v>
       </c>
       <c r="R27" s="24" t="s">
-        <v>1009</v>
+        <v>1011</v>
       </c>
       <c r="S27" s="18" t="s">
         <v>922</v>
@@ -24280,15 +24391,15 @@
         <v>62</v>
       </c>
       <c r="X27" s="26" t="s">
-        <v>1010</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>1011</v>
+        <v>1013</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>1012</v>
+        <v>1014</v>
       </c>
       <c r="C28" s="20" t="n">
         <v>1</v>
@@ -24313,12 +24424,14 @@
         <v>103</v>
       </c>
       <c r="L28" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M28" s="24" t="s">
-        <v>1007</v>
-      </c>
-      <c r="N28" s="19"/>
+        <v>1009</v>
+      </c>
+      <c r="N28" s="19" t="s">
+        <v>1015</v>
+      </c>
       <c r="O28" s="18" t="s">
         <v>106</v>
       </c>
@@ -24329,7 +24442,7 @@
         <v>44</v>
       </c>
       <c r="R28" s="24" t="s">
-        <v>983</v>
+        <v>1016</v>
       </c>
       <c r="S28" s="18" t="s">
         <v>922</v>
@@ -24346,14 +24459,16 @@
       <c r="W28" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X28" s="26"/>
+      <c r="X28" s="26" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>1013</v>
+        <v>1018</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="C29" s="20" t="n">
         <v>15</v>
@@ -24378,16 +24493,16 @@
         <v>103</v>
       </c>
       <c r="L29" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M29" s="24" t="s">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="N29" s="19" t="s">
-        <v>1016</v>
+        <v>1021</v>
       </c>
       <c r="O29" s="18" t="s">
-        <v>1017</v>
+        <v>1022</v>
       </c>
       <c r="P29" s="20" t="s">
         <v>6</v>
@@ -24396,7 +24511,7 @@
         <v>44</v>
       </c>
       <c r="R29" s="24" t="s">
-        <v>983</v>
+        <v>1023</v>
       </c>
       <c r="S29" s="18" t="s">
         <v>922</v>
@@ -24413,14 +24528,16 @@
       <c r="W29" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X29" s="26"/>
+      <c r="X29" s="26" t="s">
+        <v>1024</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>1018</v>
+        <v>1025</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>1019</v>
+        <v>1026</v>
       </c>
       <c r="C30" s="20" t="n">
         <v>10</v>
@@ -24445,14 +24562,16 @@
         <v>103</v>
       </c>
       <c r="L30" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M30" s="24" t="s">
-        <v>1015</v>
-      </c>
-      <c r="N30" s="19"/>
+        <v>1020</v>
+      </c>
+      <c r="N30" s="19" t="s">
+        <v>1027</v>
+      </c>
       <c r="O30" s="18" t="s">
-        <v>1017</v>
+        <v>1022</v>
       </c>
       <c r="P30" s="20" t="s">
         <v>6</v>
@@ -24461,7 +24580,7 @@
         <v>44</v>
       </c>
       <c r="R30" s="24" t="s">
-        <v>983</v>
+        <v>1023</v>
       </c>
       <c r="S30" s="18" t="s">
         <v>922</v>
@@ -24478,14 +24597,16 @@
       <c r="W30" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X30" s="26"/>
+      <c r="X30" s="26" t="s">
+        <v>1024</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>1020</v>
+        <v>1028</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>1021</v>
+        <v>1029</v>
       </c>
       <c r="C31" s="20" t="n">
         <v>2</v>
@@ -24510,16 +24631,16 @@
         <v>103</v>
       </c>
       <c r="L31" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M31" s="24" t="s">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="N31" s="19" t="s">
+        <v>1030</v>
+      </c>
+      <c r="O31" s="18" t="s">
         <v>1022</v>
-      </c>
-      <c r="O31" s="18" t="s">
-        <v>1017</v>
       </c>
       <c r="P31" s="20" t="s">
         <v>6</v>
@@ -24528,7 +24649,7 @@
         <v>44</v>
       </c>
       <c r="R31" s="24" t="s">
-        <v>983</v>
+        <v>1031</v>
       </c>
       <c r="S31" s="18" t="s">
         <v>922</v>
@@ -24545,14 +24666,16 @@
       <c r="W31" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X31" s="26"/>
+      <c r="X31" s="26" t="s">
+        <v>1032</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>1023</v>
+        <v>1033</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>1024</v>
+        <v>1034</v>
       </c>
       <c r="C32" s="20" t="n">
         <v>1</v>
@@ -24577,12 +24700,14 @@
         <v>103</v>
       </c>
       <c r="L32" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M32" s="24" t="s">
-        <v>1015</v>
-      </c>
-      <c r="N32" s="19"/>
+        <v>1020</v>
+      </c>
+      <c r="N32" s="19" t="s">
+        <v>1035</v>
+      </c>
       <c r="O32" s="18" t="s">
         <v>212</v>
       </c>
@@ -24593,7 +24718,7 @@
         <v>44</v>
       </c>
       <c r="R32" s="24" t="s">
-        <v>948</v>
+        <v>1036</v>
       </c>
       <c r="S32" s="18" t="s">
         <v>922</v>
@@ -24610,14 +24735,16 @@
       <c r="W32" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X32" s="26"/>
+      <c r="X32" s="26" t="s">
+        <v>1037</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>1025</v>
+        <v>1038</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>1026</v>
+        <v>1039</v>
       </c>
       <c r="C33" s="20" t="n">
         <v>1</v>
@@ -24642,13 +24769,13 @@
         <v>103</v>
       </c>
       <c r="L33" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M33" s="24" t="s">
-        <v>1027</v>
+        <v>1040</v>
       </c>
       <c r="N33" s="19" t="s">
-        <v>1028</v>
+        <v>1041</v>
       </c>
       <c r="O33" s="18" t="s">
         <v>106</v>
@@ -24660,7 +24787,7 @@
         <v>45</v>
       </c>
       <c r="R33" s="24" t="s">
-        <v>7</v>
+        <v>1042</v>
       </c>
       <c r="S33" s="18" t="s">
         <v>922</v>
@@ -24677,14 +24804,16 @@
       <c r="W33" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X33" s="26"/>
+      <c r="X33" s="26" t="s">
+        <v>1043</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>1029</v>
+        <v>1044</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>1030</v>
+        <v>1045</v>
       </c>
       <c r="C34" s="20" t="n">
         <v>1</v>
@@ -24709,13 +24838,13 @@
         <v>101</v>
       </c>
       <c r="L34" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M34" s="24" t="s">
-        <v>1027</v>
+        <v>1040</v>
       </c>
       <c r="N34" s="19" t="s">
-        <v>1031</v>
+        <v>1046</v>
       </c>
       <c r="O34" s="18" t="s">
         <v>106</v>
@@ -24727,7 +24856,7 @@
         <v>44</v>
       </c>
       <c r="R34" s="24" t="s">
-        <v>983</v>
+        <v>1047</v>
       </c>
       <c r="S34" s="18" t="s">
         <v>922</v>
@@ -24744,14 +24873,16 @@
       <c r="W34" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X34" s="26"/>
+      <c r="X34" s="26" t="s">
+        <v>1048</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>1032</v>
+        <v>1049</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>1033</v>
+        <v>1050</v>
       </c>
       <c r="C35" s="20" t="n">
         <v>1</v>
@@ -24776,13 +24907,13 @@
         <v>101</v>
       </c>
       <c r="L35" s="24" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="M35" s="24" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="N35" s="19" t="s">
-        <v>1034</v>
+        <v>1051</v>
       </c>
       <c r="O35" s="18" t="s">
         <v>106</v>
@@ -24794,7 +24925,7 @@
         <v>44</v>
       </c>
       <c r="R35" s="24" t="s">
-        <v>7</v>
+        <v>1052</v>
       </c>
       <c r="S35" s="18" t="s">
         <v>922</v>
@@ -24811,14 +24942,16 @@
       <c r="W35" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X35" s="26"/>
+      <c r="X35" s="26" t="s">
+        <v>1053</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>1035</v>
+        <v>1054</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>1036</v>
+        <v>1055</v>
       </c>
       <c r="C36" s="20" t="n">
         <v>1</v>
@@ -24843,13 +24976,13 @@
         <v>103</v>
       </c>
       <c r="L36" s="24" t="s">
-        <v>1037</v>
+        <v>1056</v>
       </c>
       <c r="M36" s="24" t="s">
-        <v>1038</v>
+        <v>1057</v>
       </c>
       <c r="N36" s="19" t="s">
-        <v>1039</v>
+        <v>1058</v>
       </c>
       <c r="O36" s="18" t="s">
         <v>106</v>
@@ -24861,7 +24994,7 @@
         <v>44</v>
       </c>
       <c r="R36" s="24" t="s">
-        <v>1040</v>
+        <v>1059</v>
       </c>
       <c r="S36" s="18" t="s">
         <v>922</v>
@@ -24878,14 +25011,16 @@
       <c r="W36" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X36" s="26"/>
+      <c r="X36" s="26" t="s">
+        <v>1060</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>1041</v>
+        <v>1061</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>1042</v>
+        <v>1062</v>
       </c>
       <c r="C37" s="20" t="n">
         <v>1</v>
@@ -24910,13 +25045,13 @@
         <v>103</v>
       </c>
       <c r="L37" s="24" t="s">
-        <v>1037</v>
+        <v>1056</v>
       </c>
       <c r="M37" s="24" t="s">
-        <v>1038</v>
+        <v>1057</v>
       </c>
       <c r="N37" s="19" t="s">
-        <v>1043</v>
+        <v>1063</v>
       </c>
       <c r="O37" s="18" t="s">
         <v>106</v>
@@ -24928,7 +25063,7 @@
         <v>44</v>
       </c>
       <c r="R37" s="24" t="s">
-        <v>948</v>
+        <v>1064</v>
       </c>
       <c r="S37" s="18" t="s">
         <v>922</v>
@@ -24945,14 +25080,16 @@
       <c r="W37" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X37" s="26"/>
+      <c r="X37" s="26" t="s">
+        <v>1065</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>1044</v>
+        <v>1066</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>1045</v>
+        <v>1067</v>
       </c>
       <c r="C38" s="20" t="n">
         <v>1</v>
@@ -24977,13 +25114,13 @@
         <v>101</v>
       </c>
       <c r="L38" s="24" t="s">
-        <v>1037</v>
+        <v>1056</v>
       </c>
       <c r="M38" s="24" t="s">
-        <v>1046</v>
+        <v>1068</v>
       </c>
       <c r="N38" s="19" t="s">
-        <v>1047</v>
+        <v>1069</v>
       </c>
       <c r="O38" s="18" t="s">
         <v>106</v>
@@ -24995,7 +25132,7 @@
         <v>44</v>
       </c>
       <c r="R38" s="24" t="s">
-        <v>983</v>
+        <v>1070</v>
       </c>
       <c r="S38" s="18" t="s">
         <v>922</v>
@@ -25012,14 +25149,16 @@
       <c r="W38" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X38" s="26"/>
+      <c r="X38" s="26" t="s">
+        <v>1071</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>1048</v>
+        <v>1072</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>1049</v>
+        <v>1073</v>
       </c>
       <c r="C39" s="20" t="n">
         <v>1</v>
@@ -25044,13 +25183,13 @@
         <v>101</v>
       </c>
       <c r="L39" s="24" t="s">
-        <v>1037</v>
+        <v>1056</v>
       </c>
       <c r="M39" s="24" t="s">
-        <v>1046</v>
+        <v>1068</v>
       </c>
       <c r="N39" s="19" t="s">
-        <v>1050</v>
+        <v>1074</v>
       </c>
       <c r="O39" s="18" t="s">
         <v>106</v>
@@ -25062,7 +25201,7 @@
         <v>45</v>
       </c>
       <c r="R39" s="24" t="s">
-        <v>7</v>
+        <v>1075</v>
       </c>
       <c r="S39" s="18" t="s">
         <v>922</v>
@@ -25079,14 +25218,16 @@
       <c r="W39" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X39" s="26"/>
+      <c r="X39" s="26" t="s">
+        <v>1076</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>1051</v>
+        <v>1077</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>1052</v>
+        <v>1078</v>
       </c>
       <c r="C40" s="20" t="n">
         <v>3</v>
@@ -25111,13 +25252,13 @@
         <v>103</v>
       </c>
       <c r="L40" s="24" t="s">
-        <v>1053</v>
+        <v>1079</v>
       </c>
       <c r="M40" s="24" t="s">
         <v>867</v>
       </c>
       <c r="N40" s="19" t="s">
-        <v>1054</v>
+        <v>1080</v>
       </c>
       <c r="O40" s="18" t="s">
         <v>868</v>
@@ -25150,10 +25291,10 @@
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>1055</v>
+        <v>1081</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>1056</v>
+        <v>1082</v>
       </c>
       <c r="C41" s="20" t="n">
         <v>1</v>
@@ -25178,13 +25319,13 @@
         <v>103</v>
       </c>
       <c r="L41" s="24" t="s">
-        <v>1053</v>
+        <v>1079</v>
       </c>
       <c r="M41" s="24" t="s">
-        <v>1057</v>
+        <v>1083</v>
       </c>
       <c r="N41" s="19" t="s">
-        <v>1058</v>
+        <v>1084</v>
       </c>
       <c r="O41" s="18" t="s">
         <v>106</v>
@@ -25196,7 +25337,7 @@
         <v>44</v>
       </c>
       <c r="R41" s="24" t="s">
-        <v>1059</v>
+        <v>1085</v>
       </c>
       <c r="S41" s="18" t="s">
         <v>922</v>
@@ -25214,15 +25355,15 @@
         <v>62</v>
       </c>
       <c r="X41" s="26" t="s">
-        <v>1060</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="18" t="s">
-        <v>1061</v>
+        <v>1087</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>1062</v>
+        <v>1088</v>
       </c>
       <c r="C42" s="20" t="n">
         <v>1</v>
@@ -25247,13 +25388,13 @@
         <v>103</v>
       </c>
       <c r="L42" s="24" t="s">
-        <v>1063</v>
+        <v>1089</v>
       </c>
       <c r="M42" s="24" t="s">
-        <v>1064</v>
+        <v>1090</v>
       </c>
       <c r="N42" s="19" t="s">
-        <v>1065</v>
+        <v>1091</v>
       </c>
       <c r="O42" s="18" t="s">
         <v>106</v>
@@ -25265,7 +25406,7 @@
         <v>44</v>
       </c>
       <c r="R42" s="24" t="s">
-        <v>1066</v>
+        <v>1042</v>
       </c>
       <c r="S42" s="18" t="s">
         <v>922</v>
@@ -25282,14 +25423,16 @@
       <c r="W42" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X42" s="26"/>
+      <c r="X42" s="26" t="s">
+        <v>1092</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
-        <v>1067</v>
+        <v>1093</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>1068</v>
+        <v>1094</v>
       </c>
       <c r="C43" s="20" t="n">
         <v>1</v>
@@ -25314,12 +25457,14 @@
         <v>103</v>
       </c>
       <c r="L43" s="24" t="s">
-        <v>1063</v>
+        <v>1089</v>
       </c>
       <c r="M43" s="24" t="s">
-        <v>1064</v>
-      </c>
-      <c r="N43" s="19"/>
+        <v>1090</v>
+      </c>
+      <c r="N43" s="19" t="s">
+        <v>1095</v>
+      </c>
       <c r="O43" s="18" t="s">
         <v>212</v>
       </c>
@@ -25330,7 +25475,7 @@
         <v>44</v>
       </c>
       <c r="R43" s="24" t="s">
-        <v>948</v>
+        <v>1096</v>
       </c>
       <c r="S43" s="18" t="s">
         <v>922</v>
@@ -25347,14 +25492,16 @@
       <c r="W43" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X43" s="26"/>
+      <c r="X43" s="26" t="s">
+        <v>1097</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>1069</v>
+        <v>1098</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>1070</v>
+        <v>1099</v>
       </c>
       <c r="C44" s="20" t="n">
         <v>1</v>
@@ -25379,13 +25526,13 @@
         <v>103</v>
       </c>
       <c r="L44" s="24" t="s">
-        <v>1063</v>
+        <v>1089</v>
       </c>
       <c r="M44" s="24" t="s">
-        <v>1064</v>
+        <v>1090</v>
       </c>
       <c r="N44" s="19" t="s">
-        <v>1071</v>
+        <v>1100</v>
       </c>
       <c r="O44" s="18" t="s">
         <v>140</v>
@@ -25397,7 +25544,7 @@
         <v>45</v>
       </c>
       <c r="R44" s="24" t="s">
-        <v>7</v>
+        <v>1101</v>
       </c>
       <c r="S44" s="18" t="s">
         <v>922</v>
@@ -25414,14 +25561,16 @@
       <c r="W44" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X44" s="26"/>
+      <c r="X44" s="26" t="s">
+        <v>1102</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
-        <v>1072</v>
+        <v>1103</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>1073</v>
+        <v>1104</v>
       </c>
       <c r="C45" s="20" t="n">
         <v>2</v>
@@ -25446,13 +25595,13 @@
         <v>103</v>
       </c>
       <c r="L45" s="24" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="M45" s="24" t="s">
-        <v>1075</v>
+        <v>1106</v>
       </c>
       <c r="N45" s="19" t="s">
-        <v>1076</v>
+        <v>1107</v>
       </c>
       <c r="O45" s="18" t="s">
         <v>106</v>
@@ -25464,7 +25613,7 @@
         <v>44</v>
       </c>
       <c r="R45" s="24" t="s">
-        <v>1077</v>
+        <v>1108</v>
       </c>
       <c r="S45" s="18" t="s">
         <v>922</v>
@@ -25482,15 +25631,15 @@
         <v>62</v>
       </c>
       <c r="X45" s="26" t="s">
-        <v>1078</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>1079</v>
+        <v>1110</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>1080</v>
+        <v>1111</v>
       </c>
       <c r="C46" s="20" t="n">
         <v>2</v>
@@ -25515,13 +25664,13 @@
         <v>103</v>
       </c>
       <c r="L46" s="24" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="M46" s="24" t="s">
-        <v>1075</v>
+        <v>1106</v>
       </c>
       <c r="N46" s="19" t="s">
-        <v>1081</v>
+        <v>1112</v>
       </c>
       <c r="O46" s="18" t="s">
         <v>106</v>
@@ -25533,7 +25682,7 @@
         <v>44</v>
       </c>
       <c r="R46" s="24" t="s">
-        <v>1077</v>
+        <v>1108</v>
       </c>
       <c r="S46" s="18" t="s">
         <v>922</v>
@@ -25551,15 +25700,15 @@
         <v>62</v>
       </c>
       <c r="X46" s="26" t="s">
-        <v>1078</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="s">
-        <v>1082</v>
+        <v>1113</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>1083</v>
+        <v>1114</v>
       </c>
       <c r="C47" s="20" t="n">
         <v>1</v>
@@ -25584,13 +25733,13 @@
         <v>103</v>
       </c>
       <c r="L47" s="24" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="M47" s="24" t="s">
-        <v>1084</v>
+        <v>1115</v>
       </c>
       <c r="N47" s="19" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="O47" s="18" t="s">
         <v>106</v>
@@ -25602,7 +25751,7 @@
         <v>44</v>
       </c>
       <c r="R47" s="24" t="s">
-        <v>609</v>
+        <v>1117</v>
       </c>
       <c r="S47" s="18" t="s">
         <v>922</v>
@@ -25619,14 +25768,16 @@
       <c r="W47" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X47" s="26"/>
+      <c r="X47" s="26" t="s">
+        <v>1118</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="s">
-        <v>1086</v>
+        <v>1119</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>1087</v>
+        <v>1120</v>
       </c>
       <c r="C48" s="20" t="n">
         <v>1</v>
@@ -25651,10 +25802,10 @@
         <v>103</v>
       </c>
       <c r="L48" s="24" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="M48" s="24" t="s">
-        <v>1084</v>
+        <v>1115</v>
       </c>
       <c r="N48" s="19"/>
       <c r="O48" s="18" t="s">
@@ -25667,7 +25818,7 @@
         <v>44</v>
       </c>
       <c r="R48" s="24" t="s">
-        <v>983</v>
+        <v>1121</v>
       </c>
       <c r="S48" s="18" t="s">
         <v>922</v>
@@ -25684,14 +25835,16 @@
       <c r="W48" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X48" s="26"/>
+      <c r="X48" s="26" t="s">
+        <v>1122</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="s">
-        <v>1088</v>
+        <v>1123</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>1089</v>
+        <v>1124</v>
       </c>
       <c r="C49" s="20" t="n">
         <v>1</v>
@@ -25716,13 +25869,13 @@
         <v>103</v>
       </c>
       <c r="L49" s="24" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="M49" s="24" t="s">
-        <v>1084</v>
+        <v>1115</v>
       </c>
       <c r="N49" s="19" t="s">
-        <v>1090</v>
+        <v>1125</v>
       </c>
       <c r="O49" s="18" t="s">
         <v>106</v>
@@ -25734,7 +25887,7 @@
         <v>44</v>
       </c>
       <c r="R49" s="24" t="s">
-        <v>948</v>
+        <v>1126</v>
       </c>
       <c r="S49" s="18" t="s">
         <v>922</v>
@@ -25751,14 +25904,16 @@
       <c r="W49" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X49" s="26"/>
+      <c r="X49" s="26" t="s">
+        <v>1127</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="18" t="s">
-        <v>1091</v>
+        <v>1128</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>1092</v>
+        <v>1129</v>
       </c>
       <c r="C50" s="20" t="n">
         <v>1</v>
@@ -25783,12 +25938,14 @@
         <v>103</v>
       </c>
       <c r="L50" s="24" t="s">
-        <v>1093</v>
+        <v>1130</v>
       </c>
       <c r="M50" s="24" t="s">
-        <v>1094</v>
-      </c>
-      <c r="N50" s="19"/>
+        <v>1131</v>
+      </c>
+      <c r="N50" s="19" t="s">
+        <v>1132</v>
+      </c>
       <c r="O50" s="18" t="s">
         <v>212</v>
       </c>
@@ -25799,7 +25956,7 @@
         <v>44</v>
       </c>
       <c r="R50" s="24" t="s">
-        <v>860</v>
+        <v>1133</v>
       </c>
       <c r="S50" s="18" t="s">
         <v>922</v>
@@ -25816,9 +25973,11 @@
       <c r="W50" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="X50" s="26"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="X50" s="26" t="s">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H51" s="14" t="s">
         <v>913</v>
       </c>
@@ -25847,17 +26006,17 @@
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>AND($T5&lt;&gt;"",$T5&lt;&gt;Summary!$C$11)</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$F5="Y"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J50">
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$J5="To decide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:E50">
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>AND($K5="Y",$F5&lt;&gt;"Y",$H5="",$D5="",$E5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25892,21 +26051,42 @@
     <hyperlink ref="X10" r:id="rId6" display="https://www.aliexpress.com/item/32814359094.html"/>
     <hyperlink ref="X11" r:id="rId7" display="https://www.aliexpress.com/item/1005007883028035.html"/>
     <hyperlink ref="X12" r:id="rId8" display="https://www.aliexpress.com/item/32814359094.html"/>
-    <hyperlink ref="X14" r:id="rId9" display="https://www.aliexpress.com/item/1005004825209262.html"/>
-    <hyperlink ref="X15" r:id="rId10" display="https://www.aliexpress.com/item/1005004825209262.html"/>
-    <hyperlink ref="X16" r:id="rId11" display="https://www.aliexpress.com/item/1005004825209262.html"/>
-    <hyperlink ref="X17" r:id="rId12" display="https://www.aliexpress.com/item/1005007791178337.html"/>
-    <hyperlink ref="X18" r:id="rId13" display="https://www.aliexpress.com/item/1005007791178337.html"/>
-    <hyperlink ref="X19" r:id="rId14" display="https://www.aliexpress.com/item/32995243964.html"/>
-    <hyperlink ref="X20" r:id="rId15" display="https://www.aliexpress.com/item/32794645480.html"/>
-    <hyperlink ref="X21" r:id="rId16" display="https://www.aliexpress.com/item/1005006093979302.html"/>
-    <hyperlink ref="X23" r:id="rId17" display="https://www.aliexpress.com/item/1005007121900242.html"/>
-    <hyperlink ref="X24" r:id="rId18" display="https://www.amazon.ca/dp/B0BTJTXHNN"/>
-    <hyperlink ref="X26" r:id="rId19" display="https://www.aliexpress.com/item/1005006478108991.html"/>
-    <hyperlink ref="X27" r:id="rId20" display="https://www.aliexpress.com/item/1005001599112235.html"/>
-    <hyperlink ref="X41" r:id="rId21" display="https://cults3d.com/en/3d-model/tool/diy-3d-printed-cnc-machine-htmcnc"/>
-    <hyperlink ref="X45" r:id="rId22" display="https://www.aliexpress.com/item/1005001948417279.html"/>
-    <hyperlink ref="X46" r:id="rId23" display="https://www.aliexpress.com/item/1005001948417279.html"/>
+    <hyperlink ref="X13" r:id="rId9" display="https://www.aliexpress.com/item/32968483467.html"/>
+    <hyperlink ref="X14" r:id="rId10" display="https://www.aliexpress.com/item/1005004825209262.html"/>
+    <hyperlink ref="X15" r:id="rId11" display="https://www.aliexpress.com/item/1005004825209262.html"/>
+    <hyperlink ref="X16" r:id="rId12" display="https://www.aliexpress.com/item/1005004825209262.html"/>
+    <hyperlink ref="X17" r:id="rId13" display="https://www.aliexpress.com/item/1005007791178337.html"/>
+    <hyperlink ref="X18" r:id="rId14" display="https://www.aliexpress.com/item/1005007791178337.html"/>
+    <hyperlink ref="X19" r:id="rId15" display="https://www.aliexpress.com/item/32995243964.html"/>
+    <hyperlink ref="X20" r:id="rId16" display="https://www.aliexpress.com/item/32794645480.html"/>
+    <hyperlink ref="X21" r:id="rId17" display="https://www.aliexpress.com/item/1005006093979302.html"/>
+    <hyperlink ref="X22" r:id="rId18" display="https://www.aliexpress.com/item/4000909595284.html"/>
+    <hyperlink ref="X23" r:id="rId19" display="https://www.aliexpress.com/item/1005007121900242.html"/>
+    <hyperlink ref="X24" r:id="rId20" display="https://www.amazon.ca/dp/B0BTJTXHNN"/>
+    <hyperlink ref="X26" r:id="rId21" display="https://www.aliexpress.com/item/1005006478108991.html"/>
+    <hyperlink ref="X27" r:id="rId22" display="https://www.aliexpress.com/item/1005001599112235.html"/>
+    <hyperlink ref="X28" r:id="rId23" display="https://www.aliexpress.com/item/1005001806206333.html"/>
+    <hyperlink ref="X29" r:id="rId24" display="https://www.aliexpress.com/item/4000564582198.html"/>
+    <hyperlink ref="X30" r:id="rId25" display="https://www.aliexpress.com/item/4000564582198.html"/>
+    <hyperlink ref="X31" r:id="rId26" display="https://www.aliexpress.com/item/1005001795469984.html"/>
+    <hyperlink ref="X32" r:id="rId27" display="https://www.aliexpress.com/item/1005007097035466.html"/>
+    <hyperlink ref="X33" r:id="rId28" display="https://www.homedepot.ca/search?q=plywood%201%2F2"/>
+    <hyperlink ref="X34" r:id="rId29" display="https://www.aliexpress.com/item/1005007181838501.html"/>
+    <hyperlink ref="X35" r:id="rId30" display="https://github.com/phil-barrett/grblHAL-teensy-4.x"/>
+    <hyperlink ref="X36" r:id="rId31" display="https://www.amazon.ca/dp/B00E7D3V4S"/>
+    <hyperlink ref="X37" r:id="rId32" display="https://www.amazon.ca/makita-rt0701c-collet/s?k=makita+rt0701c+collet"/>
+    <hyperlink ref="X38" r:id="rId33" display="https://www.aliexpress.com/item/1005008081995923.html"/>
+    <hyperlink ref="X39" r:id="rId34" display="https://www.aliexpress.com/item/1005009168636967.html"/>
+    <hyperlink ref="X41" r:id="rId35" display="https://cults3d.com/en/3d-model/tool/diy-3d-printed-cnc-machine-htmcnc"/>
+    <hyperlink ref="X42" r:id="rId36" display="https://www.homedepot.ca/search?q=mdf%203%2F4"/>
+    <hyperlink ref="X43" r:id="rId37" display="https://www.aliexpress.com/item/1005011942750737.html"/>
+    <hyperlink ref="X44" r:id="rId38" display="https://www.aliexpress.com/item/1005005244930679.html"/>
+    <hyperlink ref="X45" r:id="rId39" display="https://www.aliexpress.com/item/1005001948417279.html"/>
+    <hyperlink ref="X46" r:id="rId40" display="https://www.aliexpress.com/item/1005001948417279.html"/>
+    <hyperlink ref="X47" r:id="rId41" display="https://www.aliexpress.com/item/1005007169855682.html"/>
+    <hyperlink ref="X48" r:id="rId42" display="https://www.aliexpress.com/item/1005008660120770.html"/>
+    <hyperlink ref="X49" r:id="rId43" display="https://www.aliexpress.com/item/1005008490356061.html"/>
+    <hyperlink ref="X50" r:id="rId44" display="https://www.amazon.ca/s?k=white+lithium+grease"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25915,7 +26095,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId24"/>
+  <drawing r:id="rId45"/>
 </worksheet>
 </file>
 
@@ -25932,72 +26112,72 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>1095</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>1096</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>1097</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
-        <v>1098</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>1099</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>1100</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>1101</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>1102</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>1103</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>1104</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>1105</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>1106</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>1107</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>1108</v>
+        <v>1148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BOM: CNC tab — fill Est. low/high with every price found, as the number to beat
- 43 lines get per-unit CAD prices from the AliExpress/Amazon/Spool3D/Home Depot research (Basis = Listing or Estimate), with the source in the notes
- Decided lines keep their bought price; alternatives to beat noted on the extrusion lines
- Row-2 legend rewritten: D/E = found price, blue H = your cheaper real price overrides it

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZTgn2wDHFLcnBAkTFZVua
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4463" uniqueCount="1149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4467" uniqueCount="1154">
   <si>
     <t xml:space="preserve">07K ZN6 Turbo Swap — Cost Summary</t>
   </si>
@@ -2832,7 +2832,7 @@
     <t xml:space="preserve">07K ZN6 — CNC mill BOM (HTMCNC-style, 450 x 750 x 110 mm work area)</t>
   </si>
   <si>
-    <t xml:space="preserve">Same rules as the BOM tab. Blue column H = your real price (CAD). Lines with NO price are undecided: fill D/E with an estimate or H with the real price once you pick a listing. Decided so far (Oct 4, 2026): motor/driver/supply kit (Amazon), extrusion (Amazon). Have: Arduino UNO, filament. Every line has a candidate listing in the Link column at the far right (click to open); columns L–W with the notes are grouped — click the + above them to expand.</t>
+    <t xml:space="preserve">Same rules as the BOM tab. Est. low/high (D/E) = the prices I found on Oct 4–5, 2026, per unit in CAD, mostly AliExpress listing prices (Basis = Listing) or inferred from them (Basis = Estimate). That is the number to beat: when you find cheaper, type your real price in the blue column H and it overrides the estimate. Decided and bought-price lines: C01, C02, C20. Have: C21, C36. Every line has a candidate listing in the Link column at the far right; columns L–W with the notes are grouped (click the + above them).</t>
   </si>
   <si>
     <t xml:space="preserve">2040 T-slot extrusion, 1000 mm, black — VEVOR 5-pack</t>
@@ -2844,7 +2844,7 @@
     <t xml:space="preserve">Extrusion</t>
   </si>
   <si>
-    <t xml:space="preserve">Cut plan: two bars → 700 + 200 + 100; three bars stay 600. Cut 2–3 mm long, file square. Decided Oct 4: Amazon.</t>
+    <t xml:space="preserve">Cut plan: two bars → 700 + 200 + 100; three bars stay 600. Cut 2–3 mm long, file square. Decided Oct 4: Amazon. Found: To beat: Spool3D 2040 T-slot 1500 mm 31.50 / 1000 mm 21.00; AliExpress ~8–12 per 600 mm.</t>
   </si>
   <si>
     <t xml:space="preserve">pack</t>
@@ -2862,7 +2862,7 @@
     <t xml:space="preserve">2080 T-slot extrusion, 1000 mm, silver — 2-pack (Y rails)</t>
   </si>
   <si>
-    <t xml:space="preserve">Check the variant selector is on 1000 mm silver before buying. Decided Oct 4: Amazon. Alt: Spool3D 2080 V-slot 1000 mm.</t>
+    <t xml:space="preserve">Check the variant selector is on 1000 mm silver before buying. Decided Oct 4: Amazon. Alt: Spool3D 2080 V-slot 1000 mm. Found: To beat: Spool3D 2080 V-slot 1000 mm CAD 39.00 each (free ship over $140); AliExpress ~25–35 each plus shipping.</t>
   </si>
   <si>
     <t xml:space="preserve">Amazon B09MWBZRGH</t>
@@ -2874,19 +2874,22 @@
     <t xml:space="preserve">Corner bracket 28x20x28 (2028), with T-nuts + M5 bolts</t>
   </si>
   <si>
-    <t xml:space="preserve">Author's BOM: 18. Sold in 10-packs → buy 2 packs.</t>
+    <t xml:space="preserve">Author's BOM: 18. Sold in 10-packs → buy 2 packs. Found: 10-pack from CAD 5.11 (169 sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005007660268625</t>
   </si>
   <si>
+    <t xml:space="preserve">Listing</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.aliexpress.com/item/1005007660268625.html</t>
   </si>
   <si>
     <t xml:space="preserve">Corner bracket 20x20x20, with T-nuts + M5 bolts</t>
   </si>
   <si>
-    <t xml:space="preserve">Author's BOM: 8.</t>
+    <t xml:space="preserve">Author's BOM: 8. Found: Listing shows a teaser 'from' price; 0.30–0.80 each is typical.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005002491882309</t>
@@ -2898,7 +2901,7 @@
     <t xml:space="preserve">M5 sliding T-nut</t>
   </si>
   <si>
-    <t xml:space="preserve">20-series, 6 mm slot.</t>
+    <t xml:space="preserve">20-series, 6 mm slot. Found: 100-packs run CAD 6–12.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005007883028035</t>
@@ -2910,7 +2913,7 @@
     <t xml:space="preserve">M5 hammer-head T-nut</t>
   </si>
   <si>
-    <t xml:space="preserve">Drop-in type for adding parts after assembly.</t>
+    <t xml:space="preserve">Drop-in type for adding parts after assembly. Found: 100-packs run CAD 8–15.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 32814359094</t>
@@ -2922,13 +2925,19 @@
     <t xml:space="preserve">M4 sliding T-nut</t>
   </si>
   <si>
+    <t xml:space="preserve">Found: 50-packs run CAD 3–6.</t>
+  </si>
+  <si>
     <t xml:space="preserve">M4 hammer-head T-nut</t>
   </si>
   <si>
+    <t xml:space="preserve">Found: 50-packs run CAD 4–8.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Socket-head bolt kit (author's list)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pick the sizes from the list; 304 DIN912. Or an assorted M4/M5 kit on Amazon.ca.</t>
+    <t xml:space="preserve">Pick the sizes from the list; 304 DIN912. Or an assorted M4/M5 kit on Amazon.ca. Found: Full set per the author's list from HZYUEGOU 304 DIN912 bags (10,000+ sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 32968483467</t>
@@ -2946,7 +2955,7 @@
     <t xml:space="preserve">Linear rails</t>
   </si>
   <si>
-    <t xml:space="preserve">Y scaled to 750 mm travel: 600 + 400. Buy as a 2-rail + 4-block set.</t>
+    <t xml:space="preserve">Y scaled to 750 mm travel: 600 + 400. Buy as a 2-rail + 4-block set. Found: 2-rail + 4-block 1000 mm sets run CAD 140–190; single rail + 1 block listing from 13.84 (100 mm).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005004825209262</t>
@@ -2958,13 +2967,13 @@
     <t xml:space="preserve">HGR15 linear rail 600 mm + 2 HGH15CA blocks (X)</t>
   </si>
   <si>
-    <t xml:space="preserve">Same listing, 600 mm option.</t>
+    <t xml:space="preserve">Same listing, 600 mm option. Found: Same set listing, 600 mm option.</t>
   </si>
   <si>
     <t xml:space="preserve">HGR15 linear rail 300 mm + 2 HGH15CA blocks (Z)</t>
   </si>
   <si>
-    <t xml:space="preserve">Same listing, 300 mm option; fixed-length alt 1005012673253692.</t>
+    <t xml:space="preserve">Same listing, 300 mm option; fixed-length alt 1005012673253692. Found: Fixed-length: 2 rails + 4 blocks 200–300 mm at 119.93; 300 mm rail + block at 76.99.</t>
   </si>
   <si>
     <t xml:space="preserve">SFU1605 ballscrew 900 mm, flange nut, ends machined (Y)</t>
@@ -2973,7 +2982,7 @@
     <t xml:space="preserve">Ballscrews</t>
   </si>
   <si>
-    <t xml:space="preserve">C7 rolled. Y = 500 + 400. Check critical speed for 900 mm (author's note).</t>
+    <t xml:space="preserve">C7 rolled. Y = 500 + 400. Check critical speed for 900 mm (author's note). Found: 200–1000 mm listing from 16.08 (short length); 600 mm screw alone seen at 56.68.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005007791178337</t>
@@ -2985,10 +2994,13 @@
     <t xml:space="preserve">SFU1605 ballscrew 600 mm, flange nut, ends machined (X)</t>
   </si>
   <si>
+    <t xml:space="preserve">Found: 600 mm C7 screw-only fixed listing 56.68 (4 sold); with nut 45–65.</t>
+  </si>
+  <si>
     <t xml:space="preserve">SFU1605 ballscrew 300 mm, flange nut, ends machined (Z)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixed-length listing with 105 orders.</t>
+    <t xml:space="preserve">Fixed-length listing with 105 orders. Found: Fixed 300 mm with nut: 38.99 (105 sold, 5 stars) and 37.58.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 32995243964</t>
@@ -3003,7 +3015,7 @@
     <t xml:space="preserve">Bearing blocks</t>
   </si>
   <si>
-    <t xml:space="preserve">One pair per printed ballscrew bearing block.</t>
+    <t xml:space="preserve">One pair per printed ballscrew bearing block. Found: MOCHU 7001AC P5 DFA pair 24.99; cheaper pair listing from 10.58.</t>
   </si>
   <si>
     <t xml:space="preserve">pair</t>
@@ -3021,7 +3033,7 @@
     <t xml:space="preserve">6000-2RS bearing (10x26x8)</t>
   </si>
   <si>
-    <t xml:space="preserve">Floating-end bearings.</t>
+    <t xml:space="preserve">Floating-end bearings. Found: 10-pack 20.79 = 2.08 each; NSK 2-pack from 1.44.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005006093979302</t>
@@ -3036,7 +3048,7 @@
     <t xml:space="preserve">M12x1 locknut (ballscrew end)</t>
   </si>
   <si>
-    <t xml:space="preserve">BK12 lock nut listing; M12x1 for the 1605 screw end.</t>
+    <t xml:space="preserve">BK12 lock nut listing; M12x1 for the 1605 screw end. Found: BK/BF locknut listing from 1.73 (500+ sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 4000909595284</t>
@@ -3054,7 +3066,7 @@
     <t xml:space="preserve">Drive</t>
   </si>
   <si>
-    <t xml:space="preserve">Motor shaft 8 mm → screw end 10 mm.</t>
+    <t xml:space="preserve">Motor shaft 8 mm → screw end 10 mm. Found: D19 x L25 jaw coupling listing shows a teaser price; 2.50–4.00 each is typical.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005007121900242</t>
@@ -3099,7 +3111,7 @@
     <t xml:space="preserve">CNC Shield V3 (shield only, no stepsticks)</t>
   </si>
   <si>
-    <t xml:space="preserve">TB6600 step/dir wired to the shield's driver sockets.</t>
+    <t xml:space="preserve">TB6600 step/dir wired to the shield's driver sockets. Found: Shield-only 4–6; shield + driver kit 8.69 (71 sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005006478108991</t>
@@ -3117,7 +3129,7 @@
     <t xml:space="preserve">Switches</t>
   </si>
   <si>
-    <t xml:space="preserve">2 per axis. 5-packs.</t>
+    <t xml:space="preserve">2 per axis. 5-packs. Found: 5-pack endstops 5.35 = 1.07 each; ME-8108 roller 5-pack 21.02 = 4.20 each.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005001599112235</t>
@@ -3132,7 +3144,7 @@
     <t xml:space="preserve">E-stop button, NC</t>
   </si>
   <si>
-    <t xml:space="preserve">22 mm metal, 2NO 2NC, latching.</t>
+    <t xml:space="preserve">22 mm metal, 2NO 2NC, latching. Found: 22 mm metal 2NO/2NC 5.89 (4,000+ sold); 2.48 (3,000+).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005001806206333</t>
@@ -3150,7 +3162,7 @@
     <t xml:space="preserve">Wiring</t>
   </si>
   <si>
-    <t xml:space="preserve">Pick the 4-core 22AWG shielded option. Author used double-shielded; ground the shield at the box only.</t>
+    <t xml:space="preserve">Pick the 4-core 22AWG shielded option. Author used double-shielded; ground the shield at the box only. Found: 24AWG shielded multi-core listing from 1.44/m teaser; 1–2 per m typical.</t>
   </si>
   <si>
     <t xml:space="preserve">m</t>
@@ -3168,7 +3180,7 @@
     <t xml:space="preserve">Shielded 2-wire cable, limit switches</t>
   </si>
   <si>
-    <t xml:space="preserve">Same listing, 2-core 24AWG shielded.</t>
+    <t xml:space="preserve">Same listing, 2-core 24AWG shielded. Found: Same listing, 2-core option.</t>
   </si>
   <si>
     <t xml:space="preserve">C27</t>
@@ -3177,7 +3189,7 @@
     <t xml:space="preserve">Drag chain 10x20 + end mounts</t>
   </si>
   <si>
-    <t xml:space="preserve">Open bridge type, 10x20, 1 m lengths. X and Y runs.</t>
+    <t xml:space="preserve">Open bridge type, 10x20, 1 m lengths. X and Y runs. Found: 10x20 open bridge 1 m 4.45 (1,000+); 3.50 (4,000+).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005001795469984</t>
@@ -3192,7 +3204,7 @@
     <t xml:space="preserve">Terminal blocks, ferrules, USB cable, hookup wire</t>
   </si>
   <si>
-    <t xml:space="preserve">Ratchet ferrule crimper + ferrule kit. Terminal strips and USB cable from Amazon.ca.</t>
+    <t xml:space="preserve">Ratchet ferrule crimper + ferrule kit. Terminal strips and USB cable from Amazon.ca. Found: Ratchet ferrule crimper + ferrule kit 17.39 (10,000+ sold); terminal strips ~10 extra.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005007097035466</t>
@@ -3210,7 +3222,7 @@
     <t xml:space="preserve">Control box</t>
   </si>
   <si>
-    <t xml:space="preserve">Author's metal enclosure + GX16 connectors cost ~US$500; a plywood panel does the job.</t>
+    <t xml:space="preserve">Author's metal enclosure + GX16 connectors cost ~US$500; a plywood panel does the job. Found: Plywood offcut.</t>
   </si>
   <si>
     <t xml:space="preserve">Home Depot</t>
@@ -3225,7 +3237,7 @@
     <t xml:space="preserve">12 V fan + DC-DC converter for the box</t>
   </si>
   <si>
-    <t xml:space="preserve">36 V → 12 V 3 A buck module. Add any 80 mm 12 V fan. Only if the drivers go in a closed box.</t>
+    <t xml:space="preserve">36 V → 12 V 3 A buck module. Add any 80 mm 12 V fan. Only if the drivers go in a closed box. Found: 36→12 V buck 3–6 (5,000+ sold) + 80 mm fan 5–8.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005007181838501</t>
@@ -3240,7 +3252,7 @@
     <t xml:space="preserve">Ethernet CNC controller (grblHAL Teensy 4.1 + breakout) — EMI fix</t>
   </si>
   <si>
-    <t xml:space="preserve">Author could not fully stop USB/EMI false alarms on Arduino+GRBL. Ethernet upgrade path, not needed to start.</t>
+    <t xml:space="preserve">Author could not fully stop USB/EMI false alarms on Arduino+GRBL. Ethernet upgrade path, not needed to start. Found: Teensy 4.1 ~US$32 + grblHAL breakout ~US$40–60.</t>
   </si>
   <si>
     <t xml:space="preserve">grblHAL Teensy 4.1 breakout (PCBWay) + Teensy 4.1 (pjrc.com)</t>
@@ -3261,7 +3273,7 @@
     <t xml:space="preserve">Router</t>
   </si>
   <si>
-    <t xml:space="preserve">New vs used vs 65 mm clone. Bare RT0701C is the one to buy; the CX7 kit (B00HAQMHEO) adds bases you don't need. The printed mount is sized for the 65 mm Makita body; the Craftsman does not fit.</t>
+    <t xml:space="preserve">New vs used vs 65 mm clone. Bare RT0701C is the one to buy; the CX7 kit (B00HAQMHEO) adds bases you don't need. The printed mount is sized for the 65 mm Makita body; the Craftsman does not fit. Found: Used 80–120; new bare RT0701C ~150–170 at Home Depot.ca; Amazon CX7 kit 292.92 is more than you need.</t>
   </si>
   <si>
     <t xml:space="preserve">Amazon B00E7D3V4S (bare tool) / Home Depot.ca</t>
@@ -3276,7 +3288,7 @@
     <t xml:space="preserve">6 mm collet for RT0701C</t>
   </si>
   <si>
-    <t xml:space="preserve">Router ships with the 1/4 in cone (763637-1) only. Buy the genuine 6 mm cone, not a sleeve adapter (adds runout).</t>
+    <t xml:space="preserve">Router ships with the 1/4 in cone (763637-1) only. Buy the genuine 6 mm cone, not a sleeve adapter (adds runout). Found: Genuine Makita 6 mm cone.</t>
   </si>
   <si>
     <t xml:space="preserve">Amazon.ca search; Makita part 763636-3 (verify)</t>
@@ -3294,7 +3306,7 @@
     <t xml:space="preserve">Upgrade</t>
   </si>
   <si>
-    <t xml:space="preserve">2.2 kW ER20 air-cooled 80 mm round + VFD. Water-cooled kit with clamp: 1005003968400625. Author moved to a 2.2 kW VFD spindle for runout; do this before the gearbox adapter plate.</t>
+    <t xml:space="preserve">2.2 kW ER20 air-cooled 80 mm round + VFD. Water-cooled kit with clamp: 1005003968400625. Author moved to a 2.2 kW VFD spindle for runout; do this before the gearbox adapter plate. Found: 2.2 kW ER20 air-cooled + VFD 238.68 (33 sold); water-cooled kit with clamp 266.99 (43 sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005008081995923</t>
@@ -3309,7 +3321,7 @@
     <t xml:space="preserve">80 mm spindle mount (if VFD spindle)</t>
   </si>
   <si>
-    <t xml:space="preserve">80 mm clamp if you'd rather buy it than machine it.</t>
+    <t xml:space="preserve">80 mm clamp if you'd rather buy it than machine it. Found: 80 mm clamp 16.38 (137 sold) to 23.38 (283 sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005009168636967</t>
@@ -3339,7 +3351,7 @@
     <t xml:space="preserve">Files</t>
   </si>
   <si>
-    <t xml:space="preserve">Onshape model is free to view; files are paid.</t>
+    <t xml:space="preserve">Onshape model is free to view; files are paid. Found: Cults3D price not fetched (blocked); the author's other projects sell for US$10–25.</t>
   </si>
   <si>
     <t xml:space="preserve">Cults3D</t>
@@ -3360,7 +3372,7 @@
     <t xml:space="preserve">Workholding</t>
   </si>
   <si>
-    <t xml:space="preserve">Surface it with the machine once running.</t>
+    <t xml:space="preserve">Surface it with the machine once running. Found: Half sheet / offcut 25–35; full 4x8 3/4 in MDF 45–60 at Home Depot.</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.homedepot.ca/search?q=mdf%203%2F4</t>
@@ -3372,7 +3384,7 @@
     <t xml:space="preserve">Threaded inserts M6 (or T-track) for hold-downs</t>
   </si>
   <si>
-    <t xml:space="preserve">M6 hex-drive wood inserts, 100-pack.</t>
+    <t xml:space="preserve">M6 hex-drive wood inserts, 100-pack. Found: M6 hex-drive wood inserts 100-pack 10.85 (766 sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005011942750737</t>
@@ -3387,7 +3399,7 @@
     <t xml:space="preserve">Clamps / hold-down set</t>
   </si>
   <si>
-    <t xml:space="preserve">Arc press-plate clamps. Print the first set; machine aluminum ones later.</t>
+    <t xml:space="preserve">Arc press-plate clamps. Print the first set; machine aluminum ones later. Found: Arc press-plate clamps 0.70 each (314 sold); set of 4–6 with bolts 10–25.</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005005244930679</t>
@@ -3408,7 +3420,7 @@
     <t xml:space="preserve">Cutters</t>
   </si>
   <si>
-    <t xml:space="preserve">Roughing + profiling the flanges and adapter.</t>
+    <t xml:space="preserve">Roughing + profiling the flanges and adapter. Found: Single-flute 6 mm 5.55 (10,000+ sold); Dreanique 6 mm shank 17.09 (1,000+).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005001948417279</t>
@@ -3423,7 +3435,7 @@
     <t xml:space="preserve">Single-flute carbide endmill, 3 mm or 1/8 in</t>
   </si>
   <si>
-    <t xml:space="preserve">Small features, bung holes.</t>
+    <t xml:space="preserve">Small features, bung holes. Found: Same listing, 3–4 mm sizes; DLC-coated 8.19 (308 sold).</t>
   </si>
   <si>
     <t xml:space="preserve">C43</t>
@@ -3435,7 +3447,7 @@
     <t xml:space="preserve">Setup</t>
   </si>
   <si>
-    <t xml:space="preserve">0.01 mm indicator with flexible magnetic base. Tramming, squareness, collet runout. Mark Have if you own one.</t>
+    <t xml:space="preserve">0.01 mm indicator with flexible magnetic base. Tramming, squareness, collet runout. Mark Have if you own one. Found: 0.01 mm indicator set with flexible base 19.46 (1,000+, 4.9); magnetic stand set 22.79 (2,000+).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005007169855682</t>
@@ -3450,6 +3462,9 @@
     <t xml:space="preserve">Z touch plate / probe</t>
   </si>
   <si>
+    <t xml:space="preserve">Found: Z touch plate 5.39 (1,000+) to 7.79.</t>
+  </si>
+  <si>
     <t xml:space="preserve">AliExpress 1005008660120770</t>
   </si>
   <si>
@@ -3462,7 +3477,7 @@
     <t xml:space="preserve">Air blast or mist setup (isopropyl / WD-40) for aluminum</t>
   </si>
   <si>
-    <t xml:space="preserve">Pneumatic mist sprayer, magnetic base. Stops chip welding on the single-flute cutters.</t>
+    <t xml:space="preserve">Pneumatic mist sprayer, magnetic base. Stops chip welding on the single-flute cutters. Found: Pneumatic mist sprayer with magnetic base 11.78 (1,000+ sold).</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress 1005008490356061</t>
@@ -3483,7 +3498,7 @@
     <t xml:space="preserve">Consumables</t>
   </si>
   <si>
-    <t xml:space="preserve">NLGI 2 lithium grease for rails and screws; zip ties and heat shrink from the same order.</t>
+    <t xml:space="preserve">NLGI 2 lithium grease for rails and screws; zip ties and heat shrink from the same order. Found: Lithium grease 8–12 + zip ties / heat shrink.</t>
   </si>
   <si>
     <t xml:space="preserve">Amazon.ca / Canadian Tire</t>
@@ -3853,7 +3868,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3970,14 +3985,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFBE5E5"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5214,15 +5221,15 @@
       </c>
       <c r="C70" s="12" t="n">
         <f aca="false">SUM(CNC!$U$5:$U$50)</f>
-        <v>349.98</v>
+        <v>1252.25</v>
       </c>
       <c r="D70" s="12" t="n">
         <f aca="false">SUM(CNC!$V$5:$V$50)</f>
-        <v>349.98</v>
+        <v>1900.05</v>
       </c>
       <c r="E70" s="12" t="n">
         <f aca="false">SUM(CNC!$I$5:$I$50)</f>
-        <v>349.98</v>
+        <v>1576.15</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5248,15 +5255,15 @@
       </c>
       <c r="C72" s="12" t="n">
         <f aca="false">C70-C71</f>
-        <v>0</v>
+        <v>902.27</v>
       </c>
       <c r="D72" s="12" t="n">
         <f aca="false">D70-D71</f>
-        <v>0</v>
+        <v>1550.07</v>
       </c>
       <c r="E72" s="12" t="n">
         <f aca="false">E70-E71</f>
-        <v>0</v>
+        <v>1226.17</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5265,15 +5272,15 @@
       </c>
       <c r="C73" s="12" t="n">
         <f aca="false">C72*$C$10</f>
-        <v>0</v>
+        <v>225.5675</v>
       </c>
       <c r="D73" s="12" t="n">
         <f aca="false">D72*$C$10</f>
-        <v>0</v>
+        <v>387.5175</v>
       </c>
       <c r="E73" s="12" t="n">
         <f aca="false">E72*$C$10</f>
-        <v>0</v>
+        <v>306.5425</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5282,15 +5289,15 @@
       </c>
       <c r="C74" s="12" t="n">
         <f aca="false">C70+C73</f>
-        <v>349.98</v>
+        <v>1477.8175</v>
       </c>
       <c r="D74" s="12" t="n">
         <f aca="false">D70+D73</f>
-        <v>349.98</v>
+        <v>2287.5675</v>
       </c>
       <c r="E74" s="12" t="n">
         <f aca="false">E70+E73</f>
-        <v>349.98</v>
+        <v>1882.6925</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5331,7 +5338,7 @@
       </c>
       <c r="C80" s="3" t="n">
         <f aca="false">COUNTIFS(CNC!$K$5:$K$50,"Y",CNC!$F$5:$F$50,"&lt;&gt;Y",CNC!$H$5:$H$50,"",CNC!$D$5:$D$50,"",CNC!$E$5:$E$50,"")</f>
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22699,20 +22706,20 @@
   <dimension ref="A1:X51"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="12" min="12" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="23" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="12" min="12" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="23" min="13" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22961,8 +22968,12 @@
       <c r="C7" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
+      <c r="D7" s="21" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="F7" s="20" t="s">
         <v>101</v>
       </c>
@@ -22972,7 +22983,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="23" t="n">
         <f aca="false">IF(AND($K7="Y",$F7&lt;&gt;"Y",OR($T7="",$T7=Summary!$C$11)),$C7*IF($H7&lt;&gt;"",$H7,($D7+$E7)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P7,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>13.59</v>
       </c>
       <c r="J7" s="20" t="s">
         <v>102</v>
@@ -23007,17 +23018,17 @@
       <c r="T7" s="18"/>
       <c r="U7" s="25" t="n">
         <f aca="false">IF(AND($K7="Y",$F7&lt;&gt;"Y",OR($T7="",$T7=Summary!$C$11)),$C7*IF($H7&lt;&gt;"",$H7,$D7)*INDEX(Summary!$C$6:$C$8,MATCH($P7,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>9.18</v>
       </c>
       <c r="V7" s="25" t="n">
         <f aca="false">IF(AND($K7="Y",$F7&lt;&gt;"Y",OR($T7="",$T7=Summary!$C$11)),$C7*IF($H7&lt;&gt;"",$H7,$E7)*INDEX(Summary!$C$6:$C$8,MATCH($P7,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="W7" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X7" s="26" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23025,13 +23036,17 @@
         <v>783</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="C8" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
+      <c r="D8" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>0.8</v>
+      </c>
       <c r="F8" s="20" t="s">
         <v>101</v>
       </c>
@@ -23041,7 +23056,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="23" t="n">
         <f aca="false">IF(AND($K8="Y",$F8&lt;&gt;"Y",OR($T8="",$T8=Summary!$C$11)),$C8*IF($H8&lt;&gt;"",$H8,($D8+$E8)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P8,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>4.4</v>
       </c>
       <c r="J8" s="20" t="s">
         <v>102</v>
@@ -23056,7 +23071,7 @@
         <v>856</v>
       </c>
       <c r="N8" s="19" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="O8" s="18" t="s">
         <v>106</v>
@@ -23068,7 +23083,7 @@
         <v>44</v>
       </c>
       <c r="R8" s="24" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="S8" s="18" t="s">
         <v>922</v>
@@ -23076,17 +23091,17 @@
       <c r="T8" s="18"/>
       <c r="U8" s="25" t="n">
         <f aca="false">IF(AND($K8="Y",$F8&lt;&gt;"Y",OR($T8="",$T8=Summary!$C$11)),$C8*IF($H8&lt;&gt;"",$H8,$D8)*INDEX(Summary!$C$6:$C$8,MATCH($P8,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="V8" s="25" t="n">
         <f aca="false">IF(AND($K8="Y",$F8&lt;&gt;"Y",OR($T8="",$T8=Summary!$C$11)),$C8*IF($H8&lt;&gt;"",$H8,$E8)*INDEX(Summary!$C$6:$C$8,MATCH($P8,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6.4</v>
       </c>
       <c r="W8" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X8" s="26" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23094,13 +23109,17 @@
         <v>787</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="C9" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
+      <c r="D9" s="21" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>0.12</v>
+      </c>
       <c r="F9" s="20" t="s">
         <v>101</v>
       </c>
@@ -23110,7 +23129,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="23" t="n">
         <f aca="false">IF(AND($K9="Y",$F9&lt;&gt;"Y",OR($T9="",$T9=Summary!$C$11)),$C9*IF($H9&lt;&gt;"",$H9,($D9+$E9)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P9,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J9" s="20" t="s">
         <v>102</v>
@@ -23125,7 +23144,7 @@
         <v>856</v>
       </c>
       <c r="N9" s="19" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="O9" s="18" t="s">
         <v>106</v>
@@ -23137,7 +23156,7 @@
         <v>44</v>
       </c>
       <c r="R9" s="24" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="S9" s="18" t="s">
         <v>922</v>
@@ -23145,17 +23164,17 @@
       <c r="T9" s="18"/>
       <c r="U9" s="25" t="n">
         <f aca="false">IF(AND($K9="Y",$F9&lt;&gt;"Y",OR($T9="",$T9=Summary!$C$11)),$C9*IF($H9&lt;&gt;"",$H9,$D9)*INDEX(Summary!$C$6:$C$8,MATCH($P9,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V9" s="25" t="n">
         <f aca="false">IF(AND($K9="Y",$F9&lt;&gt;"Y",OR($T9="",$T9=Summary!$C$11)),$C9*IF($H9&lt;&gt;"",$H9,$E9)*INDEX(Summary!$C$6:$C$8,MATCH($P9,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="W9" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X9" s="26" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23163,13 +23182,17 @@
         <v>789</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="C10" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
+      <c r="D10" s="21" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0.15</v>
+      </c>
       <c r="F10" s="20" t="s">
         <v>101</v>
       </c>
@@ -23179,7 +23202,7 @@
       <c r="H10" s="22"/>
       <c r="I10" s="23" t="n">
         <f aca="false">IF(AND($K10="Y",$F10&lt;&gt;"Y",OR($T10="",$T10=Summary!$C$11)),$C10*IF($H10&lt;&gt;"",$H10,($D10+$E10)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P10,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="J10" s="20" t="s">
         <v>102</v>
@@ -23194,7 +23217,7 @@
         <v>856</v>
       </c>
       <c r="N10" s="19" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="O10" s="18" t="s">
         <v>106</v>
@@ -23206,7 +23229,7 @@
         <v>44</v>
       </c>
       <c r="R10" s="24" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="S10" s="18" t="s">
         <v>922</v>
@@ -23214,17 +23237,17 @@
       <c r="T10" s="18"/>
       <c r="U10" s="25" t="n">
         <f aca="false">IF(AND($K10="Y",$F10&lt;&gt;"Y",OR($T10="",$T10=Summary!$C$11)),$C10*IF($H10&lt;&gt;"",$H10,$D10)*INDEX(Summary!$C$6:$C$8,MATCH($P10,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="V10" s="25" t="n">
         <f aca="false">IF(AND($K10="Y",$F10&lt;&gt;"Y",OR($T10="",$T10=Summary!$C$11)),$C10*IF($H10&lt;&gt;"",$H10,$E10)*INDEX(Summary!$C$6:$C$8,MATCH($P10,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="W10" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X10" s="26" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23232,13 +23255,17 @@
         <v>791</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="C11" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
+      <c r="D11" s="21" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>0.12</v>
+      </c>
       <c r="F11" s="20" t="s">
         <v>101</v>
       </c>
@@ -23248,7 +23275,7 @@
       <c r="H11" s="22"/>
       <c r="I11" s="23" t="n">
         <f aca="false">IF(AND($K11="Y",$F11&lt;&gt;"Y",OR($T11="",$T11=Summary!$C$11)),$C11*IF($H11&lt;&gt;"",$H11,($D11+$E11)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P11,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="J11" s="20" t="s">
         <v>102</v>
@@ -23262,7 +23289,9 @@
       <c r="M11" s="24" t="s">
         <v>856</v>
       </c>
-      <c r="N11" s="19"/>
+      <c r="N11" s="19" t="s">
+        <v>946</v>
+      </c>
       <c r="O11" s="18" t="s">
         <v>106</v>
       </c>
@@ -23273,7 +23302,7 @@
         <v>44</v>
       </c>
       <c r="R11" s="24" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="S11" s="18" t="s">
         <v>922</v>
@@ -23281,17 +23310,17 @@
       <c r="T11" s="18"/>
       <c r="U11" s="25" t="n">
         <f aca="false">IF(AND($K11="Y",$F11&lt;&gt;"Y",OR($T11="",$T11=Summary!$C$11)),$C11*IF($H11&lt;&gt;"",$H11,$D11)*INDEX(Summary!$C$6:$C$8,MATCH($P11,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V11" s="25" t="n">
         <f aca="false">IF(AND($K11="Y",$F11&lt;&gt;"Y",OR($T11="",$T11=Summary!$C$11)),$C11*IF($H11&lt;&gt;"",$H11,$E11)*INDEX(Summary!$C$6:$C$8,MATCH($P11,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W11" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X11" s="26" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23299,13 +23328,17 @@
         <v>793</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="C12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
+      <c r="D12" s="21" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0.15</v>
+      </c>
       <c r="F12" s="20" t="s">
         <v>101</v>
       </c>
@@ -23315,7 +23348,7 @@
       <c r="H12" s="22"/>
       <c r="I12" s="23" t="n">
         <f aca="false">IF(AND($K12="Y",$F12&lt;&gt;"Y",OR($T12="",$T12=Summary!$C$11)),$C12*IF($H12&lt;&gt;"",$H12,($D12+$E12)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P12,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="J12" s="20" t="s">
         <v>102</v>
@@ -23329,7 +23362,9 @@
       <c r="M12" s="24" t="s">
         <v>856</v>
       </c>
-      <c r="N12" s="19"/>
+      <c r="N12" s="19" t="s">
+        <v>948</v>
+      </c>
       <c r="O12" s="18" t="s">
         <v>106</v>
       </c>
@@ -23340,7 +23375,7 @@
         <v>44</v>
       </c>
       <c r="R12" s="24" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="S12" s="18" t="s">
         <v>922</v>
@@ -23348,17 +23383,17 @@
       <c r="T12" s="18"/>
       <c r="U12" s="25" t="n">
         <f aca="false">IF(AND($K12="Y",$F12&lt;&gt;"Y",OR($T12="",$T12=Summary!$C$11)),$C12*IF($H12&lt;&gt;"",$H12,$D12)*INDEX(Summary!$C$6:$C$8,MATCH($P12,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V12" s="25" t="n">
         <f aca="false">IF(AND($K12="Y",$F12&lt;&gt;"Y",OR($T12="",$T12=Summary!$C$11)),$C12*IF($H12&lt;&gt;"",$H12,$E12)*INDEX(Summary!$C$6:$C$8,MATCH($P12,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="W12" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X12" s="26" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23366,13 +23401,17 @@
         <v>796</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>946</v>
+        <v>949</v>
       </c>
       <c r="C13" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
+      <c r="D13" s="21" t="n">
+        <v>25</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>45</v>
+      </c>
       <c r="F13" s="20" t="s">
         <v>101</v>
       </c>
@@ -23382,7 +23421,7 @@
       <c r="H13" s="22"/>
       <c r="I13" s="23" t="n">
         <f aca="false">IF(AND($K13="Y",$F13&lt;&gt;"Y",OR($T13="",$T13=Summary!$C$11)),$C13*IF($H13&lt;&gt;"",$H13,($D13+$E13)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P13,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J13" s="20" t="s">
         <v>102</v>
@@ -23397,7 +23436,7 @@
         <v>856</v>
       </c>
       <c r="N13" s="19" t="s">
-        <v>947</v>
+        <v>950</v>
       </c>
       <c r="O13" s="18" t="s">
         <v>160</v>
@@ -23409,7 +23448,7 @@
         <v>44</v>
       </c>
       <c r="R13" s="24" t="s">
-        <v>948</v>
+        <v>951</v>
       </c>
       <c r="S13" s="18" t="s">
         <v>922</v>
@@ -23417,17 +23456,17 @@
       <c r="T13" s="18"/>
       <c r="U13" s="25" t="n">
         <f aca="false">IF(AND($K13="Y",$F13&lt;&gt;"Y",OR($T13="",$T13=Summary!$C$11)),$C13*IF($H13&lt;&gt;"",$H13,$D13)*INDEX(Summary!$C$6:$C$8,MATCH($P13,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="V13" s="25" t="n">
         <f aca="false">IF(AND($K13="Y",$F13&lt;&gt;"Y",OR($T13="",$T13=Summary!$C$11)),$C13*IF($H13&lt;&gt;"",$H13,$E13)*INDEX(Summary!$C$6:$C$8,MATCH($P13,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="W13" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X13" s="26" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23435,13 +23474,17 @@
         <v>798</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>950</v>
+        <v>953</v>
       </c>
       <c r="C14" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
+      <c r="D14" s="21" t="n">
+        <v>70</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>95</v>
+      </c>
       <c r="F14" s="20" t="s">
         <v>101</v>
       </c>
@@ -23451,7 +23494,7 @@
       <c r="H14" s="22"/>
       <c r="I14" s="23" t="n">
         <f aca="false">IF(AND($K14="Y",$F14&lt;&gt;"Y",OR($T14="",$T14=Summary!$C$11)),$C14*IF($H14&lt;&gt;"",$H14,($D14+$E14)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P14,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="J14" s="20" t="s">
         <v>102</v>
@@ -23460,13 +23503,13 @@
         <v>103</v>
       </c>
       <c r="L14" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M14" s="24" t="s">
-        <v>952</v>
+        <v>955</v>
       </c>
       <c r="N14" s="19" t="s">
-        <v>953</v>
+        <v>956</v>
       </c>
       <c r="O14" s="18" t="s">
         <v>106</v>
@@ -23478,7 +23521,7 @@
         <v>44</v>
       </c>
       <c r="R14" s="24" t="s">
-        <v>954</v>
+        <v>957</v>
       </c>
       <c r="S14" s="18" t="s">
         <v>922</v>
@@ -23486,17 +23529,17 @@
       <c r="T14" s="18"/>
       <c r="U14" s="25" t="n">
         <f aca="false">IF(AND($K14="Y",$F14&lt;&gt;"Y",OR($T14="",$T14=Summary!$C$11)),$C14*IF($H14&lt;&gt;"",$H14,$D14)*INDEX(Summary!$C$6:$C$8,MATCH($P14,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="V14" s="25" t="n">
         <f aca="false">IF(AND($K14="Y",$F14&lt;&gt;"Y",OR($T14="",$T14=Summary!$C$11)),$C14*IF($H14&lt;&gt;"",$H14,$E14)*INDEX(Summary!$C$6:$C$8,MATCH($P14,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>190</v>
       </c>
       <c r="W14" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X14" s="26" t="s">
-        <v>955</v>
+        <v>958</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23504,13 +23547,17 @@
         <v>802</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>956</v>
+        <v>959</v>
       </c>
       <c r="C15" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
+      <c r="D15" s="21" t="n">
+        <v>45</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>65</v>
+      </c>
       <c r="F15" s="20" t="s">
         <v>101</v>
       </c>
@@ -23520,7 +23567,7 @@
       <c r="H15" s="22"/>
       <c r="I15" s="23" t="n">
         <f aca="false">IF(AND($K15="Y",$F15&lt;&gt;"Y",OR($T15="",$T15=Summary!$C$11)),$C15*IF($H15&lt;&gt;"",$H15,($D15+$E15)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P15,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="J15" s="20" t="s">
         <v>102</v>
@@ -23529,13 +23576,13 @@
         <v>103</v>
       </c>
       <c r="L15" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M15" s="24" t="s">
-        <v>952</v>
+        <v>955</v>
       </c>
       <c r="N15" s="19" t="s">
-        <v>957</v>
+        <v>960</v>
       </c>
       <c r="O15" s="18" t="s">
         <v>106</v>
@@ -23547,7 +23594,7 @@
         <v>44</v>
       </c>
       <c r="R15" s="24" t="s">
-        <v>954</v>
+        <v>957</v>
       </c>
       <c r="S15" s="18" t="s">
         <v>922</v>
@@ -23555,17 +23602,17 @@
       <c r="T15" s="18"/>
       <c r="U15" s="25" t="n">
         <f aca="false">IF(AND($K15="Y",$F15&lt;&gt;"Y",OR($T15="",$T15=Summary!$C$11)),$C15*IF($H15&lt;&gt;"",$H15,$D15)*INDEX(Summary!$C$6:$C$8,MATCH($P15,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="V15" s="25" t="n">
         <f aca="false">IF(AND($K15="Y",$F15&lt;&gt;"Y",OR($T15="",$T15=Summary!$C$11)),$C15*IF($H15&lt;&gt;"",$H15,$E15)*INDEX(Summary!$C$6:$C$8,MATCH($P15,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="W15" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X15" s="26" t="s">
-        <v>955</v>
+        <v>958</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23573,13 +23620,17 @@
         <v>806</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>958</v>
+        <v>961</v>
       </c>
       <c r="C16" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
+      <c r="D16" s="21" t="n">
+        <v>35</v>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>60</v>
+      </c>
       <c r="F16" s="20" t="s">
         <v>101</v>
       </c>
@@ -23589,7 +23640,7 @@
       <c r="H16" s="22"/>
       <c r="I16" s="23" t="n">
         <f aca="false">IF(AND($K16="Y",$F16&lt;&gt;"Y",OR($T16="",$T16=Summary!$C$11)),$C16*IF($H16&lt;&gt;"",$H16,($D16+$E16)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P16,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="J16" s="20" t="s">
         <v>102</v>
@@ -23598,13 +23649,13 @@
         <v>103</v>
       </c>
       <c r="L16" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M16" s="24" t="s">
-        <v>952</v>
+        <v>955</v>
       </c>
       <c r="N16" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="O16" s="18" t="s">
         <v>106</v>
@@ -23616,7 +23667,7 @@
         <v>44</v>
       </c>
       <c r="R16" s="24" t="s">
-        <v>954</v>
+        <v>957</v>
       </c>
       <c r="S16" s="18" t="s">
         <v>922</v>
@@ -23624,17 +23675,17 @@
       <c r="T16" s="18"/>
       <c r="U16" s="25" t="n">
         <f aca="false">IF(AND($K16="Y",$F16&lt;&gt;"Y",OR($T16="",$T16=Summary!$C$11)),$C16*IF($H16&lt;&gt;"",$H16,$D16)*INDEX(Summary!$C$6:$C$8,MATCH($P16,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="V16" s="25" t="n">
         <f aca="false">IF(AND($K16="Y",$F16&lt;&gt;"Y",OR($T16="",$T16=Summary!$C$11)),$C16*IF($H16&lt;&gt;"",$H16,$E16)*INDEX(Summary!$C$6:$C$8,MATCH($P16,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="W16" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X16" s="26" t="s">
-        <v>955</v>
+        <v>958</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23642,13 +23693,17 @@
         <v>808</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>960</v>
+        <v>963</v>
       </c>
       <c r="C17" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
+      <c r="D17" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>80</v>
+      </c>
       <c r="F17" s="20" t="s">
         <v>101</v>
       </c>
@@ -23658,7 +23713,7 @@
       <c r="H17" s="22"/>
       <c r="I17" s="23" t="n">
         <f aca="false">IF(AND($K17="Y",$F17&lt;&gt;"Y",OR($T17="",$T17=Summary!$C$11)),$C17*IF($H17&lt;&gt;"",$H17,($D17+$E17)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P17,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="J17" s="20" t="s">
         <v>102</v>
@@ -23667,13 +23722,13 @@
         <v>103</v>
       </c>
       <c r="L17" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M17" s="24" t="s">
-        <v>961</v>
+        <v>964</v>
       </c>
       <c r="N17" s="19" t="s">
-        <v>962</v>
+        <v>965</v>
       </c>
       <c r="O17" s="18" t="s">
         <v>106</v>
@@ -23685,7 +23740,7 @@
         <v>44</v>
       </c>
       <c r="R17" s="24" t="s">
-        <v>963</v>
+        <v>966</v>
       </c>
       <c r="S17" s="18" t="s">
         <v>922</v>
@@ -23693,17 +23748,17 @@
       <c r="T17" s="18"/>
       <c r="U17" s="25" t="n">
         <f aca="false">IF(AND($K17="Y",$F17&lt;&gt;"Y",OR($T17="",$T17=Summary!$C$11)),$C17*IF($H17&lt;&gt;"",$H17,$D17)*INDEX(Summary!$C$6:$C$8,MATCH($P17,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="V17" s="25" t="n">
         <f aca="false">IF(AND($K17="Y",$F17&lt;&gt;"Y",OR($T17="",$T17=Summary!$C$11)),$C17*IF($H17&lt;&gt;"",$H17,$E17)*INDEX(Summary!$C$6:$C$8,MATCH($P17,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="W17" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X17" s="26" t="s">
-        <v>964</v>
+        <v>967</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23711,13 +23766,17 @@
         <v>813</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="C18" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
+      <c r="D18" s="21" t="n">
+        <v>45</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>65</v>
+      </c>
       <c r="F18" s="20" t="s">
         <v>101</v>
       </c>
@@ -23727,7 +23786,7 @@
       <c r="H18" s="22"/>
       <c r="I18" s="23" t="n">
         <f aca="false">IF(AND($K18="Y",$F18&lt;&gt;"Y",OR($T18="",$T18=Summary!$C$11)),$C18*IF($H18&lt;&gt;"",$H18,($D18+$E18)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P18,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="J18" s="20" t="s">
         <v>102</v>
@@ -23736,12 +23795,14 @@
         <v>103</v>
       </c>
       <c r="L18" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M18" s="24" t="s">
-        <v>961</v>
-      </c>
-      <c r="N18" s="19"/>
+        <v>964</v>
+      </c>
+      <c r="N18" s="19" t="s">
+        <v>969</v>
+      </c>
       <c r="O18" s="18" t="s">
         <v>106</v>
       </c>
@@ -23752,7 +23813,7 @@
         <v>44</v>
       </c>
       <c r="R18" s="24" t="s">
-        <v>963</v>
+        <v>966</v>
       </c>
       <c r="S18" s="18" t="s">
         <v>922</v>
@@ -23760,17 +23821,17 @@
       <c r="T18" s="18"/>
       <c r="U18" s="25" t="n">
         <f aca="false">IF(AND($K18="Y",$F18&lt;&gt;"Y",OR($T18="",$T18=Summary!$C$11)),$C18*IF($H18&lt;&gt;"",$H18,$D18)*INDEX(Summary!$C$6:$C$8,MATCH($P18,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="V18" s="25" t="n">
         <f aca="false">IF(AND($K18="Y",$F18&lt;&gt;"Y",OR($T18="",$T18=Summary!$C$11)),$C18*IF($H18&lt;&gt;"",$H18,$E18)*INDEX(Summary!$C$6:$C$8,MATCH($P18,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="W18" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X18" s="26" t="s">
-        <v>964</v>
+        <v>967</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23778,13 +23839,17 @@
         <v>816</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
       <c r="C19" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
+      <c r="D19" s="21" t="n">
+        <v>37.58</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>38.99</v>
+      </c>
       <c r="F19" s="20" t="s">
         <v>101</v>
       </c>
@@ -23794,7 +23859,7 @@
       <c r="H19" s="22"/>
       <c r="I19" s="23" t="n">
         <f aca="false">IF(AND($K19="Y",$F19&lt;&gt;"Y",OR($T19="",$T19=Summary!$C$11)),$C19*IF($H19&lt;&gt;"",$H19,($D19+$E19)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P19,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>38.285</v>
       </c>
       <c r="J19" s="20" t="s">
         <v>102</v>
@@ -23803,13 +23868,13 @@
         <v>103</v>
       </c>
       <c r="L19" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M19" s="24" t="s">
-        <v>961</v>
+        <v>964</v>
       </c>
       <c r="N19" s="19" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
       <c r="O19" s="18" t="s">
         <v>106</v>
@@ -23821,7 +23886,7 @@
         <v>44</v>
       </c>
       <c r="R19" s="24" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="S19" s="18" t="s">
         <v>922</v>
@@ -23829,17 +23894,17 @@
       <c r="T19" s="18"/>
       <c r="U19" s="25" t="n">
         <f aca="false">IF(AND($K19="Y",$F19&lt;&gt;"Y",OR($T19="",$T19=Summary!$C$11)),$C19*IF($H19&lt;&gt;"",$H19,$D19)*INDEX(Summary!$C$6:$C$8,MATCH($P19,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>37.58</v>
       </c>
       <c r="V19" s="25" t="n">
         <f aca="false">IF(AND($K19="Y",$F19&lt;&gt;"Y",OR($T19="",$T19=Summary!$C$11)),$C19*IF($H19&lt;&gt;"",$H19,$E19)*INDEX(Summary!$C$6:$C$8,MATCH($P19,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>38.99</v>
       </c>
       <c r="W19" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X19" s="26" t="s">
-        <v>969</v>
+        <v>973</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23847,13 +23912,17 @@
         <v>818</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="C20" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
+      <c r="D20" s="21" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>24.99</v>
+      </c>
       <c r="F20" s="20" t="s">
         <v>101</v>
       </c>
@@ -23863,7 +23932,7 @@
       <c r="H20" s="22"/>
       <c r="I20" s="23" t="n">
         <f aca="false">IF(AND($K20="Y",$F20&lt;&gt;"Y",OR($T20="",$T20=Summary!$C$11)),$C20*IF($H20&lt;&gt;"",$H20,($D20+$E20)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P20,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>71.14</v>
       </c>
       <c r="J20" s="20" t="s">
         <v>102</v>
@@ -23872,16 +23941,16 @@
         <v>103</v>
       </c>
       <c r="L20" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M20" s="24" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="N20" s="19" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="O20" s="18" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="P20" s="20" t="s">
         <v>6</v>
@@ -23890,7 +23959,7 @@
         <v>44</v>
       </c>
       <c r="R20" s="24" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="S20" s="18" t="s">
         <v>922</v>
@@ -23898,31 +23967,35 @@
       <c r="T20" s="18"/>
       <c r="U20" s="25" t="n">
         <f aca="false">IF(AND($K20="Y",$F20&lt;&gt;"Y",OR($T20="",$T20=Summary!$C$11)),$C20*IF($H20&lt;&gt;"",$H20,$D20)*INDEX(Summary!$C$6:$C$8,MATCH($P20,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>42.32</v>
       </c>
       <c r="V20" s="25" t="n">
         <f aca="false">IF(AND($K20="Y",$F20&lt;&gt;"Y",OR($T20="",$T20=Summary!$C$11)),$C20*IF($H20&lt;&gt;"",$H20,$E20)*INDEX(Summary!$C$6:$C$8,MATCH($P20,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>99.96</v>
       </c>
       <c r="W20" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X20" s="26" t="s">
-        <v>975</v>
+        <v>979</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>976</v>
+        <v>980</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>977</v>
+        <v>981</v>
       </c>
       <c r="C21" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
+      <c r="D21" s="21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>2.1</v>
+      </c>
       <c r="F21" s="20" t="s">
         <v>101</v>
       </c>
@@ -23932,7 +24005,7 @@
       <c r="H21" s="22"/>
       <c r="I21" s="23" t="n">
         <f aca="false">IF(AND($K21="Y",$F21&lt;&gt;"Y",OR($T21="",$T21=Summary!$C$11)),$C21*IF($H21&lt;&gt;"",$H21,($D21+$E21)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P21,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="J21" s="20" t="s">
         <v>102</v>
@@ -23941,13 +24014,13 @@
         <v>103</v>
       </c>
       <c r="L21" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M21" s="24" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="N21" s="19" t="s">
-        <v>978</v>
+        <v>982</v>
       </c>
       <c r="O21" s="18" t="s">
         <v>106</v>
@@ -23959,7 +24032,7 @@
         <v>44</v>
       </c>
       <c r="R21" s="24" t="s">
-        <v>979</v>
+        <v>983</v>
       </c>
       <c r="S21" s="18" t="s">
         <v>922</v>
@@ -23967,31 +24040,35 @@
       <c r="T21" s="18"/>
       <c r="U21" s="25" t="n">
         <f aca="false">IF(AND($K21="Y",$F21&lt;&gt;"Y",OR($T21="",$T21=Summary!$C$11)),$C21*IF($H21&lt;&gt;"",$H21,$D21)*INDEX(Summary!$C$6:$C$8,MATCH($P21,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V21" s="25" t="n">
         <f aca="false">IF(AND($K21="Y",$F21&lt;&gt;"Y",OR($T21="",$T21=Summary!$C$11)),$C21*IF($H21&lt;&gt;"",$H21,$E21)*INDEX(Summary!$C$6:$C$8,MATCH($P21,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="W21" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X21" s="26" t="s">
-        <v>980</v>
+        <v>984</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>981</v>
+        <v>985</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="C22" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
+      <c r="D22" s="21" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="F22" s="20" t="s">
         <v>101</v>
       </c>
@@ -24001,7 +24078,7 @@
       <c r="H22" s="22"/>
       <c r="I22" s="23" t="n">
         <f aca="false">IF(AND($K22="Y",$F22&lt;&gt;"Y",OR($T22="",$T22=Summary!$C$11)),$C22*IF($H22&lt;&gt;"",$H22,($D22+$E22)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P22,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>9.46</v>
       </c>
       <c r="J22" s="20" t="s">
         <v>102</v>
@@ -24010,13 +24087,13 @@
         <v>103</v>
       </c>
       <c r="L22" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M22" s="24" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="N22" s="19" t="s">
-        <v>983</v>
+        <v>987</v>
       </c>
       <c r="O22" s="18" t="s">
         <v>106</v>
@@ -24028,7 +24105,7 @@
         <v>44</v>
       </c>
       <c r="R22" s="24" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="S22" s="18" t="s">
         <v>922</v>
@@ -24036,31 +24113,35 @@
       <c r="T22" s="18"/>
       <c r="U22" s="25" t="n">
         <f aca="false">IF(AND($K22="Y",$F22&lt;&gt;"Y",OR($T22="",$T22=Summary!$C$11)),$C22*IF($H22&lt;&gt;"",$H22,$D22)*INDEX(Summary!$C$6:$C$8,MATCH($P22,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6.92</v>
       </c>
       <c r="V22" s="25" t="n">
         <f aca="false">IF(AND($K22="Y",$F22&lt;&gt;"Y",OR($T22="",$T22=Summary!$C$11)),$C22*IF($H22&lt;&gt;"",$H22,$E22)*INDEX(Summary!$C$6:$C$8,MATCH($P22,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="W22" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X22" s="26" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>987</v>
+        <v>991</v>
       </c>
       <c r="C23" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
+      <c r="D23" s="21" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="F23" s="20" t="s">
         <v>101</v>
       </c>
@@ -24070,7 +24151,7 @@
       <c r="H23" s="22"/>
       <c r="I23" s="23" t="n">
         <f aca="false">IF(AND($K23="Y",$F23&lt;&gt;"Y",OR($T23="",$T23=Summary!$C$11)),$C23*IF($H23&lt;&gt;"",$H23,($D23+$E23)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P23,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J23" s="20" t="s">
         <v>102</v>
@@ -24079,13 +24160,13 @@
         <v>103</v>
       </c>
       <c r="L23" s="24" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="M23" s="24" t="s">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="N23" s="19" t="s">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="O23" s="18" t="s">
         <v>106</v>
@@ -24097,7 +24178,7 @@
         <v>44</v>
       </c>
       <c r="R23" s="24" t="s">
-        <v>990</v>
+        <v>994</v>
       </c>
       <c r="S23" s="18" t="s">
         <v>922</v>
@@ -24105,25 +24186,25 @@
       <c r="T23" s="18"/>
       <c r="U23" s="25" t="n">
         <f aca="false">IF(AND($K23="Y",$F23&lt;&gt;"Y",OR($T23="",$T23=Summary!$C$11)),$C23*IF($H23&lt;&gt;"",$H23,$D23)*INDEX(Summary!$C$6:$C$8,MATCH($P23,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V23" s="25" t="n">
         <f aca="false">IF(AND($K23="Y",$F23&lt;&gt;"Y",OR($T23="",$T23=Summary!$C$11)),$C23*IF($H23&lt;&gt;"",$H23,$E23)*INDEX(Summary!$C$6:$C$8,MATCH($P23,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="W23" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X23" s="26" t="s">
-        <v>991</v>
+        <v>995</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>992</v>
+        <v>996</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>993</v>
+        <v>997</v>
       </c>
       <c r="C24" s="20" t="n">
         <v>1</v>
@@ -24150,13 +24231,13 @@
         <v>103</v>
       </c>
       <c r="L24" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M24" s="24" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="N24" s="19" t="s">
-        <v>996</v>
+        <v>1000</v>
       </c>
       <c r="O24" s="18" t="s">
         <v>160</v>
@@ -24168,7 +24249,7 @@
         <v>44</v>
       </c>
       <c r="R24" s="24" t="s">
-        <v>997</v>
+        <v>1001</v>
       </c>
       <c r="S24" s="18" t="s">
         <v>922</v>
@@ -24186,15 +24267,15 @@
         <v>219</v>
       </c>
       <c r="X24" s="26" t="s">
-        <v>998</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="C25" s="20" t="n">
         <v>1</v>
@@ -24219,13 +24300,13 @@
         <v>103</v>
       </c>
       <c r="L25" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M25" s="24" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="N25" s="19" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="O25" s="18" t="s">
         <v>106</v>
@@ -24258,16 +24339,20 @@
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
       <c r="C26" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
+      <c r="D26" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" s="21" t="n">
+        <v>8.69</v>
+      </c>
       <c r="F26" s="20" t="s">
         <v>101</v>
       </c>
@@ -24277,7 +24362,7 @@
       <c r="H26" s="22"/>
       <c r="I26" s="23" t="n">
         <f aca="false">IF(AND($K26="Y",$F26&lt;&gt;"Y",OR($T26="",$T26=Summary!$C$11)),$C26*IF($H26&lt;&gt;"",$H26,($D26+$E26)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P26,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6.345</v>
       </c>
       <c r="J26" s="20" t="s">
         <v>102</v>
@@ -24286,13 +24371,13 @@
         <v>103</v>
       </c>
       <c r="L26" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M26" s="24" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="N26" s="19" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="O26" s="18" t="s">
         <v>106</v>
@@ -24304,7 +24389,7 @@
         <v>44</v>
       </c>
       <c r="R26" s="24" t="s">
-        <v>1005</v>
+        <v>1009</v>
       </c>
       <c r="S26" s="18" t="s">
         <v>922</v>
@@ -24312,31 +24397,35 @@
       <c r="T26" s="18"/>
       <c r="U26" s="25" t="n">
         <f aca="false">IF(AND($K26="Y",$F26&lt;&gt;"Y",OR($T26="",$T26=Summary!$C$11)),$C26*IF($H26&lt;&gt;"",$H26,$D26)*INDEX(Summary!$C$6:$C$8,MATCH($P26,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V26" s="25" t="n">
         <f aca="false">IF(AND($K26="Y",$F26&lt;&gt;"Y",OR($T26="",$T26=Summary!$C$11)),$C26*IF($H26&lt;&gt;"",$H26,$E26)*INDEX(Summary!$C$6:$C$8,MATCH($P26,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>8.69</v>
       </c>
       <c r="W26" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X26" s="26" t="s">
-        <v>1006</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="C27" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
+      <c r="D27" s="21" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E27" s="21" t="n">
+        <v>4.2</v>
+      </c>
       <c r="F27" s="20" t="s">
         <v>101</v>
       </c>
@@ -24346,7 +24435,7 @@
       <c r="H27" s="22"/>
       <c r="I27" s="23" t="n">
         <f aca="false">IF(AND($K27="Y",$F27&lt;&gt;"Y",OR($T27="",$T27=Summary!$C$11)),$C27*IF($H27&lt;&gt;"",$H27,($D27+$E27)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P27,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15.81</v>
       </c>
       <c r="J27" s="20" t="s">
         <v>102</v>
@@ -24355,13 +24444,13 @@
         <v>103</v>
       </c>
       <c r="L27" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M27" s="24" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="N27" s="19" t="s">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="O27" s="18" t="s">
         <v>106</v>
@@ -24373,7 +24462,7 @@
         <v>44</v>
       </c>
       <c r="R27" s="24" t="s">
-        <v>1011</v>
+        <v>1015</v>
       </c>
       <c r="S27" s="18" t="s">
         <v>922</v>
@@ -24381,31 +24470,35 @@
       <c r="T27" s="18"/>
       <c r="U27" s="25" t="n">
         <f aca="false">IF(AND($K27="Y",$F27&lt;&gt;"Y",OR($T27="",$T27=Summary!$C$11)),$C27*IF($H27&lt;&gt;"",$H27,$D27)*INDEX(Summary!$C$6:$C$8,MATCH($P27,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6.42</v>
       </c>
       <c r="V27" s="25" t="n">
         <f aca="false">IF(AND($K27="Y",$F27&lt;&gt;"Y",OR($T27="",$T27=Summary!$C$11)),$C27*IF($H27&lt;&gt;"",$H27,$E27)*INDEX(Summary!$C$6:$C$8,MATCH($P27,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>25.2</v>
       </c>
       <c r="W27" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X27" s="26" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>1013</v>
+        <v>1017</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>1014</v>
+        <v>1018</v>
       </c>
       <c r="C28" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
+      <c r="D28" s="21" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="E28" s="21" t="n">
+        <v>5.89</v>
+      </c>
       <c r="F28" s="20" t="s">
         <v>101</v>
       </c>
@@ -24415,7 +24508,7 @@
       <c r="H28" s="22"/>
       <c r="I28" s="23" t="n">
         <f aca="false">IF(AND($K28="Y",$F28&lt;&gt;"Y",OR($T28="",$T28=Summary!$C$11)),$C28*IF($H28&lt;&gt;"",$H28,($D28+$E28)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P28,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>4.185</v>
       </c>
       <c r="J28" s="20" t="s">
         <v>102</v>
@@ -24424,13 +24517,13 @@
         <v>103</v>
       </c>
       <c r="L28" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M28" s="24" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="N28" s="19" t="s">
-        <v>1015</v>
+        <v>1019</v>
       </c>
       <c r="O28" s="18" t="s">
         <v>106</v>
@@ -24442,7 +24535,7 @@
         <v>44</v>
       </c>
       <c r="R28" s="24" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
       <c r="S28" s="18" t="s">
         <v>922</v>
@@ -24450,31 +24543,35 @@
       <c r="T28" s="18"/>
       <c r="U28" s="25" t="n">
         <f aca="false">IF(AND($K28="Y",$F28&lt;&gt;"Y",OR($T28="",$T28=Summary!$C$11)),$C28*IF($H28&lt;&gt;"",$H28,$D28)*INDEX(Summary!$C$6:$C$8,MATCH($P28,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>2.48</v>
       </c>
       <c r="V28" s="25" t="n">
         <f aca="false">IF(AND($K28="Y",$F28&lt;&gt;"Y",OR($T28="",$T28=Summary!$C$11)),$C28*IF($H28&lt;&gt;"",$H28,$E28)*INDEX(Summary!$C$6:$C$8,MATCH($P28,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>5.89</v>
       </c>
       <c r="W28" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X28" s="26" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>1018</v>
+        <v>1022</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
       <c r="C29" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
+      <c r="D29" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="F29" s="20" t="s">
         <v>101</v>
       </c>
@@ -24484,7 +24581,7 @@
       <c r="H29" s="22"/>
       <c r="I29" s="23" t="n">
         <f aca="false">IF(AND($K29="Y",$F29&lt;&gt;"Y",OR($T29="",$T29=Summary!$C$11)),$C29*IF($H29&lt;&gt;"",$H29,($D29+$E29)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P29,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>22.5</v>
       </c>
       <c r="J29" s="20" t="s">
         <v>102</v>
@@ -24493,16 +24590,16 @@
         <v>103</v>
       </c>
       <c r="L29" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M29" s="24" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="N29" s="19" t="s">
-        <v>1021</v>
+        <v>1025</v>
       </c>
       <c r="O29" s="18" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="P29" s="20" t="s">
         <v>6</v>
@@ -24511,7 +24608,7 @@
         <v>44</v>
       </c>
       <c r="R29" s="24" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
       <c r="S29" s="18" t="s">
         <v>922</v>
@@ -24519,31 +24616,35 @@
       <c r="T29" s="18"/>
       <c r="U29" s="25" t="n">
         <f aca="false">IF(AND($K29="Y",$F29&lt;&gt;"Y",OR($T29="",$T29=Summary!$C$11)),$C29*IF($H29&lt;&gt;"",$H29,$D29)*INDEX(Summary!$C$6:$C$8,MATCH($P29,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="V29" s="25" t="n">
         <f aca="false">IF(AND($K29="Y",$F29&lt;&gt;"Y",OR($T29="",$T29=Summary!$C$11)),$C29*IF($H29&lt;&gt;"",$H29,$E29)*INDEX(Summary!$C$6:$C$8,MATCH($P29,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W29" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X29" s="26" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>1025</v>
+        <v>1029</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="C30" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
+      <c r="D30" s="21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E30" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F30" s="20" t="s">
         <v>101</v>
       </c>
@@ -24553,7 +24654,7 @@
       <c r="H30" s="22"/>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(AND($K30="Y",$F30&lt;&gt;"Y",OR($T30="",$T30=Summary!$C$11)),$C30*IF($H30&lt;&gt;"",$H30,($D30+$E30)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P30,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="J30" s="20" t="s">
         <v>102</v>
@@ -24562,16 +24663,16 @@
         <v>103</v>
       </c>
       <c r="L30" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M30" s="24" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="N30" s="19" t="s">
-        <v>1027</v>
+        <v>1031</v>
       </c>
       <c r="O30" s="18" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="P30" s="20" t="s">
         <v>6</v>
@@ -24580,7 +24681,7 @@
         <v>44</v>
       </c>
       <c r="R30" s="24" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
       <c r="S30" s="18" t="s">
         <v>922</v>
@@ -24588,31 +24689,35 @@
       <c r="T30" s="18"/>
       <c r="U30" s="25" t="n">
         <f aca="false">IF(AND($K30="Y",$F30&lt;&gt;"Y",OR($T30="",$T30=Summary!$C$11)),$C30*IF($H30&lt;&gt;"",$H30,$D30)*INDEX(Summary!$C$6:$C$8,MATCH($P30,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="V30" s="25" t="n">
         <f aca="false">IF(AND($K30="Y",$F30&lt;&gt;"Y",OR($T30="",$T30=Summary!$C$11)),$C30*IF($H30&lt;&gt;"",$H30,$E30)*INDEX(Summary!$C$6:$C$8,MATCH($P30,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="W30" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X30" s="26" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>1029</v>
+        <v>1033</v>
       </c>
       <c r="C31" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
+      <c r="D31" s="21" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E31" s="21" t="n">
+        <v>4.45</v>
+      </c>
       <c r="F31" s="20" t="s">
         <v>101</v>
       </c>
@@ -24622,7 +24727,7 @@
       <c r="H31" s="22"/>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(AND($K31="Y",$F31&lt;&gt;"Y",OR($T31="",$T31=Summary!$C$11)),$C31*IF($H31&lt;&gt;"",$H31,($D31+$E31)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P31,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>7.95</v>
       </c>
       <c r="J31" s="20" t="s">
         <v>102</v>
@@ -24631,16 +24736,16 @@
         <v>103</v>
       </c>
       <c r="L31" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M31" s="24" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="N31" s="19" t="s">
-        <v>1030</v>
+        <v>1034</v>
       </c>
       <c r="O31" s="18" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="P31" s="20" t="s">
         <v>6</v>
@@ -24649,7 +24754,7 @@
         <v>44</v>
       </c>
       <c r="R31" s="24" t="s">
-        <v>1031</v>
+        <v>1035</v>
       </c>
       <c r="S31" s="18" t="s">
         <v>922</v>
@@ -24657,31 +24762,35 @@
       <c r="T31" s="18"/>
       <c r="U31" s="25" t="n">
         <f aca="false">IF(AND($K31="Y",$F31&lt;&gt;"Y",OR($T31="",$T31=Summary!$C$11)),$C31*IF($H31&lt;&gt;"",$H31,$D31)*INDEX(Summary!$C$6:$C$8,MATCH($P31,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="V31" s="25" t="n">
         <f aca="false">IF(AND($K31="Y",$F31&lt;&gt;"Y",OR($T31="",$T31=Summary!$C$11)),$C31*IF($H31&lt;&gt;"",$H31,$E31)*INDEX(Summary!$C$6:$C$8,MATCH($P31,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>8.9</v>
       </c>
       <c r="W31" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X31" s="26" t="s">
-        <v>1032</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>1033</v>
+        <v>1037</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="C32" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
+      <c r="D32" s="21" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="E32" s="21" t="n">
+        <v>30</v>
+      </c>
       <c r="F32" s="20" t="s">
         <v>101</v>
       </c>
@@ -24691,7 +24800,7 @@
       <c r="H32" s="22"/>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(AND($K32="Y",$F32&lt;&gt;"Y",OR($T32="",$T32=Summary!$C$11)),$C32*IF($H32&lt;&gt;"",$H32,($D32+$E32)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P32,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>23.695</v>
       </c>
       <c r="J32" s="20" t="s">
         <v>102</v>
@@ -24700,13 +24809,13 @@
         <v>103</v>
       </c>
       <c r="L32" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M32" s="24" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="N32" s="19" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="O32" s="18" t="s">
         <v>212</v>
@@ -24718,7 +24827,7 @@
         <v>44</v>
       </c>
       <c r="R32" s="24" t="s">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="S32" s="18" t="s">
         <v>922</v>
@@ -24726,31 +24835,35 @@
       <c r="T32" s="18"/>
       <c r="U32" s="25" t="n">
         <f aca="false">IF(AND($K32="Y",$F32&lt;&gt;"Y",OR($T32="",$T32=Summary!$C$11)),$C32*IF($H32&lt;&gt;"",$H32,$D32)*INDEX(Summary!$C$6:$C$8,MATCH($P32,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>17.39</v>
       </c>
       <c r="V32" s="25" t="n">
         <f aca="false">IF(AND($K32="Y",$F32&lt;&gt;"Y",OR($T32="",$T32=Summary!$C$11)),$C32*IF($H32&lt;&gt;"",$H32,$E32)*INDEX(Summary!$C$6:$C$8,MATCH($P32,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W32" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X32" s="26" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>1039</v>
+        <v>1043</v>
       </c>
       <c r="C33" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
+      <c r="D33" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="21" t="n">
+        <v>15</v>
+      </c>
       <c r="F33" s="20" t="s">
         <v>101</v>
       </c>
@@ -24760,7 +24873,7 @@
       <c r="H33" s="22"/>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(AND($K33="Y",$F33&lt;&gt;"Y",OR($T33="",$T33=Summary!$C$11)),$C33*IF($H33&lt;&gt;"",$H33,($D33+$E33)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P33,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="J33" s="20" t="s">
         <v>126</v>
@@ -24769,13 +24882,13 @@
         <v>103</v>
       </c>
       <c r="L33" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M33" s="24" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="N33" s="19" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="O33" s="18" t="s">
         <v>106</v>
@@ -24787,7 +24900,7 @@
         <v>45</v>
       </c>
       <c r="R33" s="24" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="S33" s="18" t="s">
         <v>922</v>
@@ -24799,27 +24912,31 @@
       </c>
       <c r="V33" s="25" t="n">
         <f aca="false">IF(AND($K33="Y",$F33&lt;&gt;"Y",OR($T33="",$T33=Summary!$C$11)),$C33*IF($H33&lt;&gt;"",$H33,$E33)*INDEX(Summary!$C$6:$C$8,MATCH($P33,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="W33" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X33" s="26" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>1044</v>
+        <v>1048</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>1045</v>
+        <v>1049</v>
       </c>
       <c r="C34" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
+      <c r="D34" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E34" s="21" t="n">
+        <v>14</v>
+      </c>
       <c r="F34" s="20" t="s">
         <v>101</v>
       </c>
@@ -24838,13 +24955,13 @@
         <v>101</v>
       </c>
       <c r="L34" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M34" s="24" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="N34" s="19" t="s">
-        <v>1046</v>
+        <v>1050</v>
       </c>
       <c r="O34" s="18" t="s">
         <v>106</v>
@@ -24856,7 +24973,7 @@
         <v>44</v>
       </c>
       <c r="R34" s="24" t="s">
-        <v>1047</v>
+        <v>1051</v>
       </c>
       <c r="S34" s="18" t="s">
         <v>922</v>
@@ -24871,24 +24988,28 @@
         <v>0</v>
       </c>
       <c r="W34" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X34" s="26" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="C35" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
+      <c r="D35" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <v>140</v>
+      </c>
       <c r="F35" s="20" t="s">
         <v>101</v>
       </c>
@@ -24907,13 +25028,13 @@
         <v>101</v>
       </c>
       <c r="L35" s="24" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="M35" s="24" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="N35" s="19" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="O35" s="18" t="s">
         <v>106</v>
@@ -24925,7 +25046,7 @@
         <v>44</v>
       </c>
       <c r="R35" s="24" t="s">
-        <v>1052</v>
+        <v>1056</v>
       </c>
       <c r="S35" s="18" t="s">
         <v>922</v>
@@ -24940,24 +25061,28 @@
         <v>0</v>
       </c>
       <c r="W35" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X35" s="26" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>1055</v>
+        <v>1059</v>
       </c>
       <c r="C36" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
+      <c r="D36" s="21" t="n">
+        <v>80</v>
+      </c>
+      <c r="E36" s="21" t="n">
+        <v>170</v>
+      </c>
       <c r="F36" s="20" t="s">
         <v>101</v>
       </c>
@@ -24967,7 +25092,7 @@
       <c r="H36" s="22"/>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(AND($K36="Y",$F36&lt;&gt;"Y",OR($T36="",$T36=Summary!$C$11)),$C36*IF($H36&lt;&gt;"",$H36,($D36+$E36)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P36,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="J36" s="20" t="s">
         <v>157</v>
@@ -24976,13 +25101,13 @@
         <v>103</v>
       </c>
       <c r="L36" s="24" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="M36" s="24" t="s">
-        <v>1057</v>
+        <v>1061</v>
       </c>
       <c r="N36" s="19" t="s">
-        <v>1058</v>
+        <v>1062</v>
       </c>
       <c r="O36" s="18" t="s">
         <v>106</v>
@@ -24994,7 +25119,7 @@
         <v>44</v>
       </c>
       <c r="R36" s="24" t="s">
-        <v>1059</v>
+        <v>1063</v>
       </c>
       <c r="S36" s="18" t="s">
         <v>922</v>
@@ -25002,31 +25127,35 @@
       <c r="T36" s="18"/>
       <c r="U36" s="25" t="n">
         <f aca="false">IF(AND($K36="Y",$F36&lt;&gt;"Y",OR($T36="",$T36=Summary!$C$11)),$C36*IF($H36&lt;&gt;"",$H36,$D36)*INDEX(Summary!$C$6:$C$8,MATCH($P36,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="V36" s="25" t="n">
         <f aca="false">IF(AND($K36="Y",$F36&lt;&gt;"Y",OR($T36="",$T36=Summary!$C$11)),$C36*IF($H36&lt;&gt;"",$H36,$E36)*INDEX(Summary!$C$6:$C$8,MATCH($P36,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="W36" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X36" s="26" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>1061</v>
+        <v>1065</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>1062</v>
+        <v>1066</v>
       </c>
       <c r="C37" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="21"/>
-      <c r="E37" s="21"/>
+      <c r="D37" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E37" s="21" t="n">
+        <v>35</v>
+      </c>
       <c r="F37" s="20" t="s">
         <v>101</v>
       </c>
@@ -25036,7 +25165,7 @@
       <c r="H37" s="22"/>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(AND($K37="Y",$F37&lt;&gt;"Y",OR($T37="",$T37=Summary!$C$11)),$C37*IF($H37&lt;&gt;"",$H37,($D37+$E37)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P37,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>27.5</v>
       </c>
       <c r="J37" s="20" t="s">
         <v>102</v>
@@ -25045,13 +25174,13 @@
         <v>103</v>
       </c>
       <c r="L37" s="24" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="M37" s="24" t="s">
-        <v>1057</v>
+        <v>1061</v>
       </c>
       <c r="N37" s="19" t="s">
-        <v>1063</v>
+        <v>1067</v>
       </c>
       <c r="O37" s="18" t="s">
         <v>106</v>
@@ -25063,7 +25192,7 @@
         <v>44</v>
       </c>
       <c r="R37" s="24" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
       <c r="S37" s="18" t="s">
         <v>922</v>
@@ -25071,31 +25200,35 @@
       <c r="T37" s="18"/>
       <c r="U37" s="25" t="n">
         <f aca="false">IF(AND($K37="Y",$F37&lt;&gt;"Y",OR($T37="",$T37=Summary!$C$11)),$C37*IF($H37&lt;&gt;"",$H37,$D37)*INDEX(Summary!$C$6:$C$8,MATCH($P37,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="V37" s="25" t="n">
         <f aca="false">IF(AND($K37="Y",$F37&lt;&gt;"Y",OR($T37="",$T37=Summary!$C$11)),$C37*IF($H37&lt;&gt;"",$H37,$E37)*INDEX(Summary!$C$6:$C$8,MATCH($P37,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W37" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X37" s="26" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>1066</v>
+        <v>1070</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>1067</v>
+        <v>1071</v>
       </c>
       <c r="C38" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
+      <c r="D38" s="21" t="n">
+        <v>238.68</v>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>266.99</v>
+      </c>
       <c r="F38" s="20" t="s">
         <v>101</v>
       </c>
@@ -25114,13 +25247,13 @@
         <v>101</v>
       </c>
       <c r="L38" s="24" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="M38" s="24" t="s">
-        <v>1068</v>
+        <v>1072</v>
       </c>
       <c r="N38" s="19" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
       <c r="O38" s="18" t="s">
         <v>106</v>
@@ -25132,7 +25265,7 @@
         <v>44</v>
       </c>
       <c r="R38" s="24" t="s">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="S38" s="18" t="s">
         <v>922</v>
@@ -25147,24 +25280,28 @@
         <v>0</v>
       </c>
       <c r="W38" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X38" s="26" t="s">
-        <v>1071</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>1073</v>
+        <v>1077</v>
       </c>
       <c r="C39" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
+      <c r="D39" s="21" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="E39" s="21" t="n">
+        <v>23.38</v>
+      </c>
       <c r="F39" s="20" t="s">
         <v>101</v>
       </c>
@@ -25183,13 +25320,13 @@
         <v>101</v>
       </c>
       <c r="L39" s="24" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="M39" s="24" t="s">
-        <v>1068</v>
+        <v>1072</v>
       </c>
       <c r="N39" s="19" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
       <c r="O39" s="18" t="s">
         <v>106</v>
@@ -25201,7 +25338,7 @@
         <v>45</v>
       </c>
       <c r="R39" s="24" t="s">
-        <v>1075</v>
+        <v>1079</v>
       </c>
       <c r="S39" s="18" t="s">
         <v>922</v>
@@ -25216,18 +25353,18 @@
         <v>0</v>
       </c>
       <c r="W39" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X39" s="26" t="s">
-        <v>1076</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>1077</v>
+        <v>1081</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>1078</v>
+        <v>1082</v>
       </c>
       <c r="C40" s="20" t="n">
         <v>3</v>
@@ -25252,13 +25389,13 @@
         <v>103</v>
       </c>
       <c r="L40" s="24" t="s">
-        <v>1079</v>
+        <v>1083</v>
       </c>
       <c r="M40" s="24" t="s">
         <v>867</v>
       </c>
       <c r="N40" s="19" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="O40" s="18" t="s">
         <v>868</v>
@@ -25291,16 +25428,20 @@
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>1081</v>
+        <v>1085</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>1082</v>
+        <v>1086</v>
       </c>
       <c r="C41" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
+      <c r="D41" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E41" s="21" t="n">
+        <v>35</v>
+      </c>
       <c r="F41" s="20" t="s">
         <v>101</v>
       </c>
@@ -25310,7 +25451,7 @@
       <c r="H41" s="22"/>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(AND($K41="Y",$F41&lt;&gt;"Y",OR($T41="",$T41=Summary!$C$11)),$C41*IF($H41&lt;&gt;"",$H41,($D41+$E41)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P41,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J41" s="20" t="s">
         <v>102</v>
@@ -25319,13 +25460,13 @@
         <v>103</v>
       </c>
       <c r="L41" s="24" t="s">
-        <v>1079</v>
+        <v>1083</v>
       </c>
       <c r="M41" s="24" t="s">
-        <v>1083</v>
+        <v>1087</v>
       </c>
       <c r="N41" s="19" t="s">
-        <v>1084</v>
+        <v>1088</v>
       </c>
       <c r="O41" s="18" t="s">
         <v>106</v>
@@ -25337,7 +25478,7 @@
         <v>44</v>
       </c>
       <c r="R41" s="24" t="s">
-        <v>1085</v>
+        <v>1089</v>
       </c>
       <c r="S41" s="18" t="s">
         <v>922</v>
@@ -25345,31 +25486,35 @@
       <c r="T41" s="18"/>
       <c r="U41" s="25" t="n">
         <f aca="false">IF(AND($K41="Y",$F41&lt;&gt;"Y",OR($T41="",$T41=Summary!$C$11)),$C41*IF($H41&lt;&gt;"",$H41,$D41)*INDEX(Summary!$C$6:$C$8,MATCH($P41,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="V41" s="25" t="n">
         <f aca="false">IF(AND($K41="Y",$F41&lt;&gt;"Y",OR($T41="",$T41=Summary!$C$11)),$C41*IF($H41&lt;&gt;"",$H41,$E41)*INDEX(Summary!$C$6:$C$8,MATCH($P41,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W41" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X41" s="26" t="s">
-        <v>1086</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="18" t="s">
-        <v>1087</v>
+        <v>1091</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>1088</v>
+        <v>1092</v>
       </c>
       <c r="C42" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D42" s="21"/>
-      <c r="E42" s="21"/>
+      <c r="D42" s="21" t="n">
+        <v>25</v>
+      </c>
+      <c r="E42" s="21" t="n">
+        <v>60</v>
+      </c>
       <c r="F42" s="20" t="s">
         <v>101</v>
       </c>
@@ -25379,7 +25524,7 @@
       <c r="H42" s="22"/>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(AND($K42="Y",$F42&lt;&gt;"Y",OR($T42="",$T42=Summary!$C$11)),$C42*IF($H42&lt;&gt;"",$H42,($D42+$E42)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P42,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>42.5</v>
       </c>
       <c r="J42" s="20" t="s">
         <v>102</v>
@@ -25388,13 +25533,13 @@
         <v>103</v>
       </c>
       <c r="L42" s="24" t="s">
-        <v>1089</v>
+        <v>1093</v>
       </c>
       <c r="M42" s="24" t="s">
-        <v>1090</v>
+        <v>1094</v>
       </c>
       <c r="N42" s="19" t="s">
-        <v>1091</v>
+        <v>1095</v>
       </c>
       <c r="O42" s="18" t="s">
         <v>106</v>
@@ -25406,7 +25551,7 @@
         <v>44</v>
       </c>
       <c r="R42" s="24" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="S42" s="18" t="s">
         <v>922</v>
@@ -25414,31 +25559,35 @@
       <c r="T42" s="18"/>
       <c r="U42" s="25" t="n">
         <f aca="false">IF(AND($K42="Y",$F42&lt;&gt;"Y",OR($T42="",$T42=Summary!$C$11)),$C42*IF($H42&lt;&gt;"",$H42,$D42)*INDEX(Summary!$C$6:$C$8,MATCH($P42,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="V42" s="25" t="n">
         <f aca="false">IF(AND($K42="Y",$F42&lt;&gt;"Y",OR($T42="",$T42=Summary!$C$11)),$C42*IF($H42&lt;&gt;"",$H42,$E42)*INDEX(Summary!$C$6:$C$8,MATCH($P42,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="W42" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X42" s="26" t="s">
-        <v>1092</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
-        <v>1093</v>
+        <v>1097</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>1094</v>
+        <v>1098</v>
       </c>
       <c r="C43" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D43" s="21"/>
-      <c r="E43" s="21"/>
+      <c r="D43" s="21" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="E43" s="21" t="n">
+        <v>15</v>
+      </c>
       <c r="F43" s="20" t="s">
         <v>101</v>
       </c>
@@ -25448,7 +25597,7 @@
       <c r="H43" s="22"/>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(AND($K43="Y",$F43&lt;&gt;"Y",OR($T43="",$T43=Summary!$C$11)),$C43*IF($H43&lt;&gt;"",$H43,($D43+$E43)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P43,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>12.925</v>
       </c>
       <c r="J43" s="20" t="s">
         <v>102</v>
@@ -25457,13 +25606,13 @@
         <v>103</v>
       </c>
       <c r="L43" s="24" t="s">
-        <v>1089</v>
+        <v>1093</v>
       </c>
       <c r="M43" s="24" t="s">
-        <v>1090</v>
+        <v>1094</v>
       </c>
       <c r="N43" s="19" t="s">
-        <v>1095</v>
+        <v>1099</v>
       </c>
       <c r="O43" s="18" t="s">
         <v>212</v>
@@ -25475,7 +25624,7 @@
         <v>44</v>
       </c>
       <c r="R43" s="24" t="s">
-        <v>1096</v>
+        <v>1100</v>
       </c>
       <c r="S43" s="18" t="s">
         <v>922</v>
@@ -25483,31 +25632,35 @@
       <c r="T43" s="18"/>
       <c r="U43" s="25" t="n">
         <f aca="false">IF(AND($K43="Y",$F43&lt;&gt;"Y",OR($T43="",$T43=Summary!$C$11)),$C43*IF($H43&lt;&gt;"",$H43,$D43)*INDEX(Summary!$C$6:$C$8,MATCH($P43,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>10.85</v>
       </c>
       <c r="V43" s="25" t="n">
         <f aca="false">IF(AND($K43="Y",$F43&lt;&gt;"Y",OR($T43="",$T43=Summary!$C$11)),$C43*IF($H43&lt;&gt;"",$H43,$E43)*INDEX(Summary!$C$6:$C$8,MATCH($P43,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="W43" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X43" s="26" t="s">
-        <v>1097</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>1098</v>
+        <v>1102</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>1099</v>
+        <v>1103</v>
       </c>
       <c r="C44" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="21"/>
-      <c r="E44" s="21"/>
+      <c r="D44" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E44" s="21" t="n">
+        <v>25</v>
+      </c>
       <c r="F44" s="20" t="s">
         <v>101</v>
       </c>
@@ -25517,7 +25670,7 @@
       <c r="H44" s="22"/>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(AND($K44="Y",$F44&lt;&gt;"Y",OR($T44="",$T44=Summary!$C$11)),$C44*IF($H44&lt;&gt;"",$H44,($D44+$E44)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P44,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>17.5</v>
       </c>
       <c r="J44" s="20" t="s">
         <v>102</v>
@@ -25526,13 +25679,13 @@
         <v>103</v>
       </c>
       <c r="L44" s="24" t="s">
-        <v>1089</v>
+        <v>1093</v>
       </c>
       <c r="M44" s="24" t="s">
-        <v>1090</v>
+        <v>1094</v>
       </c>
       <c r="N44" s="19" t="s">
-        <v>1100</v>
+        <v>1104</v>
       </c>
       <c r="O44" s="18" t="s">
         <v>140</v>
@@ -25544,7 +25697,7 @@
         <v>45</v>
       </c>
       <c r="R44" s="24" t="s">
-        <v>1101</v>
+        <v>1105</v>
       </c>
       <c r="S44" s="18" t="s">
         <v>922</v>
@@ -25552,31 +25705,35 @@
       <c r="T44" s="18"/>
       <c r="U44" s="25" t="n">
         <f aca="false">IF(AND($K44="Y",$F44&lt;&gt;"Y",OR($T44="",$T44=Summary!$C$11)),$C44*IF($H44&lt;&gt;"",$H44,$D44)*INDEX(Summary!$C$6:$C$8,MATCH($P44,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V44" s="25" t="n">
         <f aca="false">IF(AND($K44="Y",$F44&lt;&gt;"Y",OR($T44="",$T44=Summary!$C$11)),$C44*IF($H44&lt;&gt;"",$H44,$E44)*INDEX(Summary!$C$6:$C$8,MATCH($P44,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="W44" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X44" s="26" t="s">
-        <v>1102</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
-        <v>1103</v>
+        <v>1107</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>1104</v>
+        <v>1108</v>
       </c>
       <c r="C45" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
+      <c r="D45" s="21" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="E45" s="21" t="n">
+        <v>17.09</v>
+      </c>
       <c r="F45" s="20" t="s">
         <v>101</v>
       </c>
@@ -25586,7 +25743,7 @@
       <c r="H45" s="22"/>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(AND($K45="Y",$F45&lt;&gt;"Y",OR($T45="",$T45=Summary!$C$11)),$C45*IF($H45&lt;&gt;"",$H45,($D45+$E45)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P45,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>22.64</v>
       </c>
       <c r="J45" s="20" t="s">
         <v>102</v>
@@ -25595,13 +25752,13 @@
         <v>103</v>
       </c>
       <c r="L45" s="24" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="M45" s="24" t="s">
-        <v>1106</v>
+        <v>1110</v>
       </c>
       <c r="N45" s="19" t="s">
-        <v>1107</v>
+        <v>1111</v>
       </c>
       <c r="O45" s="18" t="s">
         <v>106</v>
@@ -25613,7 +25770,7 @@
         <v>44</v>
       </c>
       <c r="R45" s="24" t="s">
-        <v>1108</v>
+        <v>1112</v>
       </c>
       <c r="S45" s="18" t="s">
         <v>922</v>
@@ -25621,31 +25778,35 @@
       <c r="T45" s="18"/>
       <c r="U45" s="25" t="n">
         <f aca="false">IF(AND($K45="Y",$F45&lt;&gt;"Y",OR($T45="",$T45=Summary!$C$11)),$C45*IF($H45&lt;&gt;"",$H45,$D45)*INDEX(Summary!$C$6:$C$8,MATCH($P45,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>11.1</v>
       </c>
       <c r="V45" s="25" t="n">
         <f aca="false">IF(AND($K45="Y",$F45&lt;&gt;"Y",OR($T45="",$T45=Summary!$C$11)),$C45*IF($H45&lt;&gt;"",$H45,$E45)*INDEX(Summary!$C$6:$C$8,MATCH($P45,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>34.18</v>
       </c>
       <c r="W45" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X45" s="26" t="s">
-        <v>1109</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>1110</v>
+        <v>1114</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>1111</v>
+        <v>1115</v>
       </c>
       <c r="C46" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
+      <c r="D46" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" s="21" t="n">
+        <v>8.19</v>
+      </c>
       <c r="F46" s="20" t="s">
         <v>101</v>
       </c>
@@ -25655,7 +25816,7 @@
       <c r="H46" s="22"/>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(AND($K46="Y",$F46&lt;&gt;"Y",OR($T46="",$T46=Summary!$C$11)),$C46*IF($H46&lt;&gt;"",$H46,($D46+$E46)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P46,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>12.19</v>
       </c>
       <c r="J46" s="20" t="s">
         <v>102</v>
@@ -25664,13 +25825,13 @@
         <v>103</v>
       </c>
       <c r="L46" s="24" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="M46" s="24" t="s">
-        <v>1106</v>
+        <v>1110</v>
       </c>
       <c r="N46" s="19" t="s">
-        <v>1112</v>
+        <v>1116</v>
       </c>
       <c r="O46" s="18" t="s">
         <v>106</v>
@@ -25682,7 +25843,7 @@
         <v>44</v>
       </c>
       <c r="R46" s="24" t="s">
-        <v>1108</v>
+        <v>1112</v>
       </c>
       <c r="S46" s="18" t="s">
         <v>922</v>
@@ -25690,31 +25851,35 @@
       <c r="T46" s="18"/>
       <c r="U46" s="25" t="n">
         <f aca="false">IF(AND($K46="Y",$F46&lt;&gt;"Y",OR($T46="",$T46=Summary!$C$11)),$C46*IF($H46&lt;&gt;"",$H46,$D46)*INDEX(Summary!$C$6:$C$8,MATCH($P46,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="V46" s="25" t="n">
         <f aca="false">IF(AND($K46="Y",$F46&lt;&gt;"Y",OR($T46="",$T46=Summary!$C$11)),$C46*IF($H46&lt;&gt;"",$H46,$E46)*INDEX(Summary!$C$6:$C$8,MATCH($P46,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>16.38</v>
       </c>
       <c r="W46" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X46" s="26" t="s">
-        <v>1109</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="s">
-        <v>1113</v>
+        <v>1117</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>1114</v>
+        <v>1118</v>
       </c>
       <c r="C47" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D47" s="21"/>
-      <c r="E47" s="21"/>
+      <c r="D47" s="21" t="n">
+        <v>19.46</v>
+      </c>
+      <c r="E47" s="21" t="n">
+        <v>22.79</v>
+      </c>
       <c r="F47" s="20" t="s">
         <v>101</v>
       </c>
@@ -25724,7 +25889,7 @@
       <c r="H47" s="22"/>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(AND($K47="Y",$F47&lt;&gt;"Y",OR($T47="",$T47=Summary!$C$11)),$C47*IF($H47&lt;&gt;"",$H47,($D47+$E47)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P47,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>21.125</v>
       </c>
       <c r="J47" s="20" t="s">
         <v>157</v>
@@ -25733,13 +25898,13 @@
         <v>103</v>
       </c>
       <c r="L47" s="24" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="M47" s="24" t="s">
-        <v>1115</v>
+        <v>1119</v>
       </c>
       <c r="N47" s="19" t="s">
-        <v>1116</v>
+        <v>1120</v>
       </c>
       <c r="O47" s="18" t="s">
         <v>106</v>
@@ -25751,7 +25916,7 @@
         <v>44</v>
       </c>
       <c r="R47" s="24" t="s">
-        <v>1117</v>
+        <v>1121</v>
       </c>
       <c r="S47" s="18" t="s">
         <v>922</v>
@@ -25759,31 +25924,35 @@
       <c r="T47" s="18"/>
       <c r="U47" s="25" t="n">
         <f aca="false">IF(AND($K47="Y",$F47&lt;&gt;"Y",OR($T47="",$T47=Summary!$C$11)),$C47*IF($H47&lt;&gt;"",$H47,$D47)*INDEX(Summary!$C$6:$C$8,MATCH($P47,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>19.46</v>
       </c>
       <c r="V47" s="25" t="n">
         <f aca="false">IF(AND($K47="Y",$F47&lt;&gt;"Y",OR($T47="",$T47=Summary!$C$11)),$C47*IF($H47&lt;&gt;"",$H47,$E47)*INDEX(Summary!$C$6:$C$8,MATCH($P47,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>22.79</v>
       </c>
       <c r="W47" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X47" s="26" t="s">
-        <v>1118</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="s">
-        <v>1119</v>
+        <v>1123</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>1120</v>
+        <v>1124</v>
       </c>
       <c r="C48" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
+      <c r="D48" s="21" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="E48" s="21" t="n">
+        <v>7.79</v>
+      </c>
       <c r="F48" s="20" t="s">
         <v>101</v>
       </c>
@@ -25793,7 +25962,7 @@
       <c r="H48" s="22"/>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(AND($K48="Y",$F48&lt;&gt;"Y",OR($T48="",$T48=Summary!$C$11)),$C48*IF($H48&lt;&gt;"",$H48,($D48+$E48)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P48,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>6.59</v>
       </c>
       <c r="J48" s="20" t="s">
         <v>126</v>
@@ -25802,12 +25971,14 @@
         <v>103</v>
       </c>
       <c r="L48" s="24" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="M48" s="24" t="s">
-        <v>1115</v>
-      </c>
-      <c r="N48" s="19"/>
+        <v>1119</v>
+      </c>
+      <c r="N48" s="19" t="s">
+        <v>1125</v>
+      </c>
       <c r="O48" s="18" t="s">
         <v>106</v>
       </c>
@@ -25818,7 +25989,7 @@
         <v>44</v>
       </c>
       <c r="R48" s="24" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="S48" s="18" t="s">
         <v>922</v>
@@ -25826,31 +25997,35 @@
       <c r="T48" s="18"/>
       <c r="U48" s="25" t="n">
         <f aca="false">IF(AND($K48="Y",$F48&lt;&gt;"Y",OR($T48="",$T48=Summary!$C$11)),$C48*IF($H48&lt;&gt;"",$H48,$D48)*INDEX(Summary!$C$6:$C$8,MATCH($P48,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>5.39</v>
       </c>
       <c r="V48" s="25" t="n">
         <f aca="false">IF(AND($K48="Y",$F48&lt;&gt;"Y",OR($T48="",$T48=Summary!$C$11)),$C48*IF($H48&lt;&gt;"",$H48,$E48)*INDEX(Summary!$C$6:$C$8,MATCH($P48,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>7.79</v>
       </c>
       <c r="W48" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X48" s="26" t="s">
-        <v>1122</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="s">
-        <v>1123</v>
+        <v>1128</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>1124</v>
+        <v>1129</v>
       </c>
       <c r="C49" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D49" s="21"/>
-      <c r="E49" s="21"/>
+      <c r="D49" s="21" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="E49" s="21" t="n">
+        <v>20</v>
+      </c>
       <c r="F49" s="20" t="s">
         <v>101</v>
       </c>
@@ -25860,7 +26035,7 @@
       <c r="H49" s="22"/>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(AND($K49="Y",$F49&lt;&gt;"Y",OR($T49="",$T49=Summary!$C$11)),$C49*IF($H49&lt;&gt;"",$H49,($D49+$E49)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P49,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15.89</v>
       </c>
       <c r="J49" s="20" t="s">
         <v>126</v>
@@ -25869,13 +26044,13 @@
         <v>103</v>
       </c>
       <c r="L49" s="24" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="M49" s="24" t="s">
-        <v>1115</v>
+        <v>1119</v>
       </c>
       <c r="N49" s="19" t="s">
-        <v>1125</v>
+        <v>1130</v>
       </c>
       <c r="O49" s="18" t="s">
         <v>106</v>
@@ -25887,7 +26062,7 @@
         <v>44</v>
       </c>
       <c r="R49" s="24" t="s">
-        <v>1126</v>
+        <v>1131</v>
       </c>
       <c r="S49" s="18" t="s">
         <v>922</v>
@@ -25895,31 +26070,35 @@
       <c r="T49" s="18"/>
       <c r="U49" s="25" t="n">
         <f aca="false">IF(AND($K49="Y",$F49&lt;&gt;"Y",OR($T49="",$T49=Summary!$C$11)),$C49*IF($H49&lt;&gt;"",$H49,$D49)*INDEX(Summary!$C$6:$C$8,MATCH($P49,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="V49" s="25" t="n">
         <f aca="false">IF(AND($K49="Y",$F49&lt;&gt;"Y",OR($T49="",$T49=Summary!$C$11)),$C49*IF($H49&lt;&gt;"",$H49,$E49)*INDEX(Summary!$C$6:$C$8,MATCH($P49,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="W49" s="18" t="s">
-        <v>62</v>
+        <v>931</v>
       </c>
       <c r="X49" s="26" t="s">
-        <v>1127</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="18" t="s">
-        <v>1128</v>
+        <v>1133</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>1129</v>
+        <v>1134</v>
       </c>
       <c r="C50" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D50" s="21"/>
-      <c r="E50" s="21"/>
+      <c r="D50" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E50" s="21" t="n">
+        <v>20</v>
+      </c>
       <c r="F50" s="20" t="s">
         <v>101</v>
       </c>
@@ -25929,7 +26108,7 @@
       <c r="H50" s="22"/>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(AND($K50="Y",$F50&lt;&gt;"Y",OR($T50="",$T50=Summary!$C$11)),$C50*IF($H50&lt;&gt;"",$H50,($D50+$E50)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P50,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J50" s="20" t="s">
         <v>102</v>
@@ -25938,13 +26117,13 @@
         <v>103</v>
       </c>
       <c r="L50" s="24" t="s">
-        <v>1130</v>
+        <v>1135</v>
       </c>
       <c r="M50" s="24" t="s">
-        <v>1131</v>
+        <v>1136</v>
       </c>
       <c r="N50" s="19" t="s">
-        <v>1132</v>
+        <v>1137</v>
       </c>
       <c r="O50" s="18" t="s">
         <v>212</v>
@@ -25956,7 +26135,7 @@
         <v>44</v>
       </c>
       <c r="R50" s="24" t="s">
-        <v>1133</v>
+        <v>1138</v>
       </c>
       <c r="S50" s="18" t="s">
         <v>922</v>
@@ -25964,17 +26143,17 @@
       <c r="T50" s="18"/>
       <c r="U50" s="25" t="n">
         <f aca="false">IF(AND($K50="Y",$F50&lt;&gt;"Y",OR($T50="",$T50=Summary!$C$11)),$C50*IF($H50&lt;&gt;"",$H50,$D50)*INDEX(Summary!$C$6:$C$8,MATCH($P50,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V50" s="25" t="n">
         <f aca="false">IF(AND($K50="Y",$F50&lt;&gt;"Y",OR($T50="",$T50=Summary!$C$11)),$C50*IF($H50&lt;&gt;"",$H50,$E50)*INDEX(Summary!$C$6:$C$8,MATCH($P50,Summary!$B$6:$B$8,0)),0)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="W50" s="18" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="X50" s="26" t="s">
-        <v>1134</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25983,15 +26162,15 @@
       </c>
       <c r="I51" s="14" t="n">
         <f aca="false">SUM(I5:I50)</f>
-        <v>349.98</v>
+        <v>1576.15</v>
       </c>
       <c r="U51" s="14" t="n">
         <f aca="false">SUM(U5:U50)</f>
-        <v>349.98</v>
+        <v>1252.25</v>
       </c>
       <c r="V51" s="14" t="n">
         <f aca="false">SUM(V5:V50)</f>
-        <v>349.98</v>
+        <v>1900.05</v>
       </c>
     </row>
   </sheetData>
@@ -26000,10 +26179,10 @@
     <mergeCell ref="A2:K2"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:X50">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$K5="N"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>AND($T5&lt;&gt;"",$T5&lt;&gt;Summary!$C$11)</formula>
     </cfRule>
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
@@ -26016,7 +26195,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:E50">
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>AND($K5="Y",$F5&lt;&gt;"Y",$H5="",$D5="",$E5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26112,72 +26291,72 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>1135</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>1136</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>1137</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
-        <v>1138</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>1139</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>1140</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>1141</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>1142</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>1143</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>1144</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>1145</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>1146</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>1147</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>1148</v>
+        <v>1153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BOM: say per-unit in the price headers, show cents on the CNC tab, rename Working to Line total / Best estimate
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZTgn2wDHFLcnBAkTFZVua
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -85,12 +85,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4472" uniqueCount="1158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4473" uniqueCount="1159">
   <si>
     <t xml:space="preserve">07K ZN6 Turbo Swap — Cost Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">All prices in CAD (USD × 1.42, GBP × 1.85 at Oct 4, 2026), before HST. Low/High = estimate range. WORKING = your actual price where you've entered one, otherwise the midpoint of the estimate. Have = Y lines count $0.</t>
+    <t xml:space="preserve">All prices in CAD (USD × 1.42, GBP × 1.85 at Oct 4, 2026), before HST. Low/High = estimate range. Best estimate = your actual price where you've entered one, otherwise the midpoint of the estimate range. Have = Y lines count $0.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumptions</t>
@@ -150,7 +150,7 @@
     <t xml:space="preserve">High (CAD)</t>
   </si>
   <si>
-    <t xml:space="preserve">WORKING (CAD)</t>
+    <t xml:space="preserve">Best estimate (CAD)</t>
   </si>
   <si>
     <t xml:space="preserve">Donors</t>
@@ -330,10 +330,10 @@
     <t xml:space="preserve">Qty</t>
   </si>
   <si>
-    <t xml:space="preserve">Est. low</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Est. high</t>
+    <t xml:space="preserve">Est. unit low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Est. unit high</t>
   </si>
   <si>
     <t xml:space="preserve">Have?</t>
@@ -342,10 +342,10 @@
     <t xml:space="preserve">Make?</t>
   </si>
   <si>
-    <t xml:space="preserve">MY cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Working (CAD)</t>
+    <t xml:space="preserve">MY unit cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line total (CAD)</t>
   </si>
   <si>
     <t xml:space="preserve">Status</t>
@@ -378,10 +378,10 @@
     <t xml:space="preserve">Route</t>
   </si>
   <si>
-    <t xml:space="preserve">Ext low (CAD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ext high (CAD)</t>
+    <t xml:space="preserve">Line total low (CAD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line total high (CAD)</t>
   </si>
   <si>
     <t xml:space="preserve">Basis</t>
@@ -2838,7 +2838,7 @@
     <t xml:space="preserve">07K ZN6 — CNC mill BOM (HTMCNC-style, 450 x 750 x 110 mm work area)</t>
   </si>
   <si>
-    <t xml:space="preserve">Same rules as the BOM tab. Est. low/high (D/E) = the prices I found on Oct 4–5, 2026, per unit in CAD, mostly AliExpress listing prices (Basis = Listing) or inferred from them (Basis = Estimate). That is the number to beat: when you find cheaper, type your real price in the blue column H and it overrides the estimate. Decided and bought-price lines: C01, C02, C20. Have: C21, C36. Every line has a candidate listing in the Link column at the far right; columns L–W with the notes are grouped (click the + above them).</t>
+    <t xml:space="preserve">Prices are PER UNIT (each, pack, metre or lot as the Unit column says). Est. unit low / high = the cheapest and dearest price I found for one unit. Line total = Qty × price, using your MY unit cost if you typed one, otherwise the midpoint of low and high. Have = Y makes a line $0; Incl. = N drops it. Example: C03 is 18 brackets at $0.51–$1.00 each, so its line total is 18 × $0.76 = $13.59.</t>
   </si>
   <si>
     <t xml:space="preserve">2040 T-slot extrusion, 1000 mm, black — VEVOR 5-pack</t>
@@ -3559,17 +3559,21 @@
   </si>
   <si>
     <t xml:space="preserve">10. CNC tab — the parts list for the DIY CNC mill (HTMCNC-style, Y scaled to 750 mm). Same columns and colour rules as the BOM tab, plus pink Est. cells = no price decided yet. The Summary has its own CNC block; it is not added to the car's ALL-IN.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11. Every price column is PER UNIT. Line total (CAD) = Qty × unit price. The Summary's 'Best estimate' column is the sum of line totals, using your real price where you've entered one and the midpoint of the estimate range where you haven't.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="0%"/>
     <numFmt numFmtId="167" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="168" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -3754,7 +3758,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3861,6 +3865,30 @@
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -5316,7 +5344,7 @@
         <v>1226.17</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="3" t="s">
         <v>53</v>
       </c>
@@ -5383,7 +5411,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="3" t="s">
         <v>74</v>
       </c>
@@ -5401,7 +5429,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="9" t="s">
         <v>75</v>
       </c>
@@ -22760,12 +22788,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="6"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="12" min="12" style="1" width="15"/>
@@ -22877,18 +22904,18 @@
       <c r="C5" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
       <c r="F5" s="20" t="s">
         <v>103</v>
       </c>
       <c r="G5" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="28" t="n">
         <v>57.99</v>
       </c>
-      <c r="I5" s="23" t="n">
+      <c r="I5" s="29" t="n">
         <f aca="false">IF(AND($K5="Y",$F5&lt;&gt;"Y",OR($T5="",$T5=Summary!$C$11)),$C5*IF($H5&lt;&gt;"",$H5,($D5+$E5)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P5,Summary!$B$6:$B$8,0)),0)</f>
         <v>57.99</v>
       </c>
@@ -22923,11 +22950,11 @@
         <v>924</v>
       </c>
       <c r="T5" s="18"/>
-      <c r="U5" s="25" t="n">
+      <c r="U5" s="30" t="n">
         <f aca="false">IF(AND($K5="Y",$F5&lt;&gt;"Y",OR($T5="",$T5=Summary!$C$11)),$C5*IF($H5&lt;&gt;"",$H5,$D5)*INDEX(Summary!$C$6:$C$8,MATCH($P5,Summary!$B$6:$B$8,0)),0)</f>
         <v>57.99</v>
       </c>
-      <c r="V5" s="25" t="n">
+      <c r="V5" s="30" t="n">
         <f aca="false">IF(AND($K5="Y",$F5&lt;&gt;"Y",OR($T5="",$T5=Summary!$C$11)),$C5*IF($H5&lt;&gt;"",$H5,$E5)*INDEX(Summary!$C$6:$C$8,MATCH($P5,Summary!$B$6:$B$8,0)),0)</f>
         <v>57.99</v>
       </c>
@@ -22948,18 +22975,18 @@
       <c r="C6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
       <c r="F6" s="20" t="s">
         <v>103</v>
       </c>
       <c r="G6" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="28" t="n">
         <v>106.99</v>
       </c>
-      <c r="I6" s="23" t="n">
+      <c r="I6" s="29" t="n">
         <f aca="false">IF(AND($K6="Y",$F6&lt;&gt;"Y",OR($T6="",$T6=Summary!$C$11)),$C6*IF($H6&lt;&gt;"",$H6,($D6+$E6)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P6,Summary!$B$6:$B$8,0)),0)</f>
         <v>106.99</v>
       </c>
@@ -22994,11 +23021,11 @@
         <v>924</v>
       </c>
       <c r="T6" s="18"/>
-      <c r="U6" s="25" t="n">
+      <c r="U6" s="30" t="n">
         <f aca="false">IF(AND($K6="Y",$F6&lt;&gt;"Y",OR($T6="",$T6=Summary!$C$11)),$C6*IF($H6&lt;&gt;"",$H6,$D6)*INDEX(Summary!$C$6:$C$8,MATCH($P6,Summary!$B$6:$B$8,0)),0)</f>
         <v>106.99</v>
       </c>
-      <c r="V6" s="25" t="n">
+      <c r="V6" s="30" t="n">
         <f aca="false">IF(AND($K6="Y",$F6&lt;&gt;"Y",OR($T6="",$T6=Summary!$C$11)),$C6*IF($H6&lt;&gt;"",$H6,$E6)*INDEX(Summary!$C$6:$C$8,MATCH($P6,Summary!$B$6:$B$8,0)),0)</f>
         <v>106.99</v>
       </c>
@@ -23019,10 +23046,10 @@
       <c r="C7" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="27" t="n">
         <v>0.51</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="27" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="20" t="s">
@@ -23031,8 +23058,8 @@
       <c r="G7" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H7" s="22"/>
-      <c r="I7" s="23" t="n">
+      <c r="H7" s="28"/>
+      <c r="I7" s="29" t="n">
         <f aca="false">IF(AND($K7="Y",$F7&lt;&gt;"Y",OR($T7="",$T7=Summary!$C$11)),$C7*IF($H7&lt;&gt;"",$H7,($D7+$E7)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P7,Summary!$B$6:$B$8,0)),0)</f>
         <v>13.59</v>
       </c>
@@ -23067,11 +23094,11 @@
         <v>924</v>
       </c>
       <c r="T7" s="18"/>
-      <c r="U7" s="25" t="n">
+      <c r="U7" s="30" t="n">
         <f aca="false">IF(AND($K7="Y",$F7&lt;&gt;"Y",OR($T7="",$T7=Summary!$C$11)),$C7*IF($H7&lt;&gt;"",$H7,$D7)*INDEX(Summary!$C$6:$C$8,MATCH($P7,Summary!$B$6:$B$8,0)),0)</f>
         <v>9.18</v>
       </c>
-      <c r="V7" s="25" t="n">
+      <c r="V7" s="30" t="n">
         <f aca="false">IF(AND($K7="Y",$F7&lt;&gt;"Y",OR($T7="",$T7=Summary!$C$11)),$C7*IF($H7&lt;&gt;"",$H7,$E7)*INDEX(Summary!$C$6:$C$8,MATCH($P7,Summary!$B$6:$B$8,0)),0)</f>
         <v>18</v>
       </c>
@@ -23092,10 +23119,10 @@
       <c r="C8" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="27" t="n">
         <v>0.3</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="F8" s="20" t="s">
@@ -23104,8 +23131,8 @@
       <c r="G8" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H8" s="22"/>
-      <c r="I8" s="23" t="n">
+      <c r="H8" s="28"/>
+      <c r="I8" s="29" t="n">
         <f aca="false">IF(AND($K8="Y",$F8&lt;&gt;"Y",OR($T8="",$T8=Summary!$C$11)),$C8*IF($H8&lt;&gt;"",$H8,($D8+$E8)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P8,Summary!$B$6:$B$8,0)),0)</f>
         <v>4.4</v>
       </c>
@@ -23140,11 +23167,11 @@
         <v>924</v>
       </c>
       <c r="T8" s="18"/>
-      <c r="U8" s="25" t="n">
+      <c r="U8" s="30" t="n">
         <f aca="false">IF(AND($K8="Y",$F8&lt;&gt;"Y",OR($T8="",$T8=Summary!$C$11)),$C8*IF($H8&lt;&gt;"",$H8,$D8)*INDEX(Summary!$C$6:$C$8,MATCH($P8,Summary!$B$6:$B$8,0)),0)</f>
         <v>2.4</v>
       </c>
-      <c r="V8" s="25" t="n">
+      <c r="V8" s="30" t="n">
         <f aca="false">IF(AND($K8="Y",$F8&lt;&gt;"Y",OR($T8="",$T8=Summary!$C$11)),$C8*IF($H8&lt;&gt;"",$H8,$E8)*INDEX(Summary!$C$6:$C$8,MATCH($P8,Summary!$B$6:$B$8,0)),0)</f>
         <v>6.4</v>
       </c>
@@ -23165,10 +23192,10 @@
       <c r="C9" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="27" t="n">
         <v>0.06</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="27" t="n">
         <v>0.12</v>
       </c>
       <c r="F9" s="20" t="s">
@@ -23177,8 +23204,8 @@
       <c r="G9" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H9" s="22"/>
-      <c r="I9" s="23" t="n">
+      <c r="H9" s="28"/>
+      <c r="I9" s="29" t="n">
         <f aca="false">IF(AND($K9="Y",$F9&lt;&gt;"Y",OR($T9="",$T9=Summary!$C$11)),$C9*IF($H9&lt;&gt;"",$H9,($D9+$E9)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P9,Summary!$B$6:$B$8,0)),0)</f>
         <v>9</v>
       </c>
@@ -23213,11 +23240,11 @@
         <v>924</v>
       </c>
       <c r="T9" s="18"/>
-      <c r="U9" s="25" t="n">
+      <c r="U9" s="30" t="n">
         <f aca="false">IF(AND($K9="Y",$F9&lt;&gt;"Y",OR($T9="",$T9=Summary!$C$11)),$C9*IF($H9&lt;&gt;"",$H9,$D9)*INDEX(Summary!$C$6:$C$8,MATCH($P9,Summary!$B$6:$B$8,0)),0)</f>
         <v>6</v>
       </c>
-      <c r="V9" s="25" t="n">
+      <c r="V9" s="30" t="n">
         <f aca="false">IF(AND($K9="Y",$F9&lt;&gt;"Y",OR($T9="",$T9=Summary!$C$11)),$C9*IF($H9&lt;&gt;"",$H9,$E9)*INDEX(Summary!$C$6:$C$8,MATCH($P9,Summary!$B$6:$B$8,0)),0)</f>
         <v>12</v>
       </c>
@@ -23238,10 +23265,10 @@
       <c r="C10" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="27" t="n">
         <v>0.15</v>
       </c>
       <c r="F10" s="20" t="s">
@@ -23250,8 +23277,8 @@
       <c r="G10" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H10" s="22"/>
-      <c r="I10" s="23" t="n">
+      <c r="H10" s="28"/>
+      <c r="I10" s="29" t="n">
         <f aca="false">IF(AND($K10="Y",$F10&lt;&gt;"Y",OR($T10="",$T10=Summary!$C$11)),$C10*IF($H10&lt;&gt;"",$H10,($D10+$E10)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P10,Summary!$B$6:$B$8,0)),0)</f>
         <v>11.5</v>
       </c>
@@ -23286,11 +23313,11 @@
         <v>924</v>
       </c>
       <c r="T10" s="18"/>
-      <c r="U10" s="25" t="n">
+      <c r="U10" s="30" t="n">
         <f aca="false">IF(AND($K10="Y",$F10&lt;&gt;"Y",OR($T10="",$T10=Summary!$C$11)),$C10*IF($H10&lt;&gt;"",$H10,$D10)*INDEX(Summary!$C$6:$C$8,MATCH($P10,Summary!$B$6:$B$8,0)),0)</f>
         <v>8</v>
       </c>
-      <c r="V10" s="25" t="n">
+      <c r="V10" s="30" t="n">
         <f aca="false">IF(AND($K10="Y",$F10&lt;&gt;"Y",OR($T10="",$T10=Summary!$C$11)),$C10*IF($H10&lt;&gt;"",$H10,$E10)*INDEX(Summary!$C$6:$C$8,MATCH($P10,Summary!$B$6:$B$8,0)),0)</f>
         <v>15</v>
       </c>
@@ -23311,10 +23338,10 @@
       <c r="C11" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="27" t="n">
         <v>0.06</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="27" t="n">
         <v>0.12</v>
       </c>
       <c r="F11" s="20" t="s">
@@ -23323,8 +23350,8 @@
       <c r="G11" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H11" s="22"/>
-      <c r="I11" s="23" t="n">
+      <c r="H11" s="28"/>
+      <c r="I11" s="29" t="n">
         <f aca="false">IF(AND($K11="Y",$F11&lt;&gt;"Y",OR($T11="",$T11=Summary!$C$11)),$C11*IF($H11&lt;&gt;"",$H11,($D11+$E11)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P11,Summary!$B$6:$B$8,0)),0)</f>
         <v>4.5</v>
       </c>
@@ -23359,11 +23386,11 @@
         <v>924</v>
       </c>
       <c r="T11" s="18"/>
-      <c r="U11" s="25" t="n">
+      <c r="U11" s="30" t="n">
         <f aca="false">IF(AND($K11="Y",$F11&lt;&gt;"Y",OR($T11="",$T11=Summary!$C$11)),$C11*IF($H11&lt;&gt;"",$H11,$D11)*INDEX(Summary!$C$6:$C$8,MATCH($P11,Summary!$B$6:$B$8,0)),0)</f>
         <v>3</v>
       </c>
-      <c r="V11" s="25" t="n">
+      <c r="V11" s="30" t="n">
         <f aca="false">IF(AND($K11="Y",$F11&lt;&gt;"Y",OR($T11="",$T11=Summary!$C$11)),$C11*IF($H11&lt;&gt;"",$H11,$E11)*INDEX(Summary!$C$6:$C$8,MATCH($P11,Summary!$B$6:$B$8,0)),0)</f>
         <v>6</v>
       </c>
@@ -23384,10 +23411,10 @@
       <c r="C12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="E12" s="21" t="n">
+      <c r="E12" s="27" t="n">
         <v>0.15</v>
       </c>
       <c r="F12" s="20" t="s">
@@ -23396,8 +23423,8 @@
       <c r="G12" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H12" s="22"/>
-      <c r="I12" s="23" t="n">
+      <c r="H12" s="28"/>
+      <c r="I12" s="29" t="n">
         <f aca="false">IF(AND($K12="Y",$F12&lt;&gt;"Y",OR($T12="",$T12=Summary!$C$11)),$C12*IF($H12&lt;&gt;"",$H12,($D12+$E12)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P12,Summary!$B$6:$B$8,0)),0)</f>
         <v>5.75</v>
       </c>
@@ -23432,11 +23459,11 @@
         <v>924</v>
       </c>
       <c r="T12" s="18"/>
-      <c r="U12" s="25" t="n">
+      <c r="U12" s="30" t="n">
         <f aca="false">IF(AND($K12="Y",$F12&lt;&gt;"Y",OR($T12="",$T12=Summary!$C$11)),$C12*IF($H12&lt;&gt;"",$H12,$D12)*INDEX(Summary!$C$6:$C$8,MATCH($P12,Summary!$B$6:$B$8,0)),0)</f>
         <v>4</v>
       </c>
-      <c r="V12" s="25" t="n">
+      <c r="V12" s="30" t="n">
         <f aca="false">IF(AND($K12="Y",$F12&lt;&gt;"Y",OR($T12="",$T12=Summary!$C$11)),$C12*IF($H12&lt;&gt;"",$H12,$E12)*INDEX(Summary!$C$6:$C$8,MATCH($P12,Summary!$B$6:$B$8,0)),0)</f>
         <v>7.5</v>
       </c>
@@ -23457,10 +23484,10 @@
       <c r="C13" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="E13" s="21" t="n">
+      <c r="E13" s="27" t="n">
         <v>45</v>
       </c>
       <c r="F13" s="20" t="s">
@@ -23469,8 +23496,8 @@
       <c r="G13" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H13" s="22"/>
-      <c r="I13" s="23" t="n">
+      <c r="H13" s="28"/>
+      <c r="I13" s="29" t="n">
         <f aca="false">IF(AND($K13="Y",$F13&lt;&gt;"Y",OR($T13="",$T13=Summary!$C$11)),$C13*IF($H13&lt;&gt;"",$H13,($D13+$E13)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P13,Summary!$B$6:$B$8,0)),0)</f>
         <v>35</v>
       </c>
@@ -23505,11 +23532,11 @@
         <v>924</v>
       </c>
       <c r="T13" s="18"/>
-      <c r="U13" s="25" t="n">
+      <c r="U13" s="30" t="n">
         <f aca="false">IF(AND($K13="Y",$F13&lt;&gt;"Y",OR($T13="",$T13=Summary!$C$11)),$C13*IF($H13&lt;&gt;"",$H13,$D13)*INDEX(Summary!$C$6:$C$8,MATCH($P13,Summary!$B$6:$B$8,0)),0)</f>
         <v>25</v>
       </c>
-      <c r="V13" s="25" t="n">
+      <c r="V13" s="30" t="n">
         <f aca="false">IF(AND($K13="Y",$F13&lt;&gt;"Y",OR($T13="",$T13=Summary!$C$11)),$C13*IF($H13&lt;&gt;"",$H13,$E13)*INDEX(Summary!$C$6:$C$8,MATCH($P13,Summary!$B$6:$B$8,0)),0)</f>
         <v>45</v>
       </c>
@@ -23530,10 +23557,10 @@
       <c r="C14" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="27" t="n">
         <v>70</v>
       </c>
-      <c r="E14" s="21" t="n">
+      <c r="E14" s="27" t="n">
         <v>95</v>
       </c>
       <c r="F14" s="20" t="s">
@@ -23542,8 +23569,8 @@
       <c r="G14" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H14" s="22"/>
-      <c r="I14" s="23" t="n">
+      <c r="H14" s="28"/>
+      <c r="I14" s="29" t="n">
         <f aca="false">IF(AND($K14="Y",$F14&lt;&gt;"Y",OR($T14="",$T14=Summary!$C$11)),$C14*IF($H14&lt;&gt;"",$H14,($D14+$E14)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P14,Summary!$B$6:$B$8,0)),0)</f>
         <v>165</v>
       </c>
@@ -23578,11 +23605,11 @@
         <v>924</v>
       </c>
       <c r="T14" s="18"/>
-      <c r="U14" s="25" t="n">
+      <c r="U14" s="30" t="n">
         <f aca="false">IF(AND($K14="Y",$F14&lt;&gt;"Y",OR($T14="",$T14=Summary!$C$11)),$C14*IF($H14&lt;&gt;"",$H14,$D14)*INDEX(Summary!$C$6:$C$8,MATCH($P14,Summary!$B$6:$B$8,0)),0)</f>
         <v>140</v>
       </c>
-      <c r="V14" s="25" t="n">
+      <c r="V14" s="30" t="n">
         <f aca="false">IF(AND($K14="Y",$F14&lt;&gt;"Y",OR($T14="",$T14=Summary!$C$11)),$C14*IF($H14&lt;&gt;"",$H14,$E14)*INDEX(Summary!$C$6:$C$8,MATCH($P14,Summary!$B$6:$B$8,0)),0)</f>
         <v>190</v>
       </c>
@@ -23603,10 +23630,10 @@
       <c r="C15" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="27" t="n">
         <v>65</v>
       </c>
       <c r="F15" s="20" t="s">
@@ -23615,8 +23642,8 @@
       <c r="G15" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H15" s="22"/>
-      <c r="I15" s="23" t="n">
+      <c r="H15" s="28"/>
+      <c r="I15" s="29" t="n">
         <f aca="false">IF(AND($K15="Y",$F15&lt;&gt;"Y",OR($T15="",$T15=Summary!$C$11)),$C15*IF($H15&lt;&gt;"",$H15,($D15+$E15)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P15,Summary!$B$6:$B$8,0)),0)</f>
         <v>110</v>
       </c>
@@ -23651,11 +23678,11 @@
         <v>924</v>
       </c>
       <c r="T15" s="18"/>
-      <c r="U15" s="25" t="n">
+      <c r="U15" s="30" t="n">
         <f aca="false">IF(AND($K15="Y",$F15&lt;&gt;"Y",OR($T15="",$T15=Summary!$C$11)),$C15*IF($H15&lt;&gt;"",$H15,$D15)*INDEX(Summary!$C$6:$C$8,MATCH($P15,Summary!$B$6:$B$8,0)),0)</f>
         <v>90</v>
       </c>
-      <c r="V15" s="25" t="n">
+      <c r="V15" s="30" t="n">
         <f aca="false">IF(AND($K15="Y",$F15&lt;&gt;"Y",OR($T15="",$T15=Summary!$C$11)),$C15*IF($H15&lt;&gt;"",$H15,$E15)*INDEX(Summary!$C$6:$C$8,MATCH($P15,Summary!$B$6:$B$8,0)),0)</f>
         <v>130</v>
       </c>
@@ -23676,10 +23703,10 @@
       <c r="C16" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="27" t="n">
         <v>35</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="27" t="n">
         <v>60</v>
       </c>
       <c r="F16" s="20" t="s">
@@ -23688,8 +23715,8 @@
       <c r="G16" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H16" s="22"/>
-      <c r="I16" s="23" t="n">
+      <c r="H16" s="28"/>
+      <c r="I16" s="29" t="n">
         <f aca="false">IF(AND($K16="Y",$F16&lt;&gt;"Y",OR($T16="",$T16=Summary!$C$11)),$C16*IF($H16&lt;&gt;"",$H16,($D16+$E16)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P16,Summary!$B$6:$B$8,0)),0)</f>
         <v>95</v>
       </c>
@@ -23724,11 +23751,11 @@
         <v>924</v>
       </c>
       <c r="T16" s="18"/>
-      <c r="U16" s="25" t="n">
+      <c r="U16" s="30" t="n">
         <f aca="false">IF(AND($K16="Y",$F16&lt;&gt;"Y",OR($T16="",$T16=Summary!$C$11)),$C16*IF($H16&lt;&gt;"",$H16,$D16)*INDEX(Summary!$C$6:$C$8,MATCH($P16,Summary!$B$6:$B$8,0)),0)</f>
         <v>70</v>
       </c>
-      <c r="V16" s="25" t="n">
+      <c r="V16" s="30" t="n">
         <f aca="false">IF(AND($K16="Y",$F16&lt;&gt;"Y",OR($T16="",$T16=Summary!$C$11)),$C16*IF($H16&lt;&gt;"",$H16,$E16)*INDEX(Summary!$C$6:$C$8,MATCH($P16,Summary!$B$6:$B$8,0)),0)</f>
         <v>120</v>
       </c>
@@ -23749,10 +23776,10 @@
       <c r="C17" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="27" t="n">
         <v>55</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="27" t="n">
         <v>80</v>
       </c>
       <c r="F17" s="20" t="s">
@@ -23761,8 +23788,8 @@
       <c r="G17" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H17" s="22"/>
-      <c r="I17" s="23" t="n">
+      <c r="H17" s="28"/>
+      <c r="I17" s="29" t="n">
         <f aca="false">IF(AND($K17="Y",$F17&lt;&gt;"Y",OR($T17="",$T17=Summary!$C$11)),$C17*IF($H17&lt;&gt;"",$H17,($D17+$E17)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P17,Summary!$B$6:$B$8,0)),0)</f>
         <v>135</v>
       </c>
@@ -23797,11 +23824,11 @@
         <v>924</v>
       </c>
       <c r="T17" s="18"/>
-      <c r="U17" s="25" t="n">
+      <c r="U17" s="30" t="n">
         <f aca="false">IF(AND($K17="Y",$F17&lt;&gt;"Y",OR($T17="",$T17=Summary!$C$11)),$C17*IF($H17&lt;&gt;"",$H17,$D17)*INDEX(Summary!$C$6:$C$8,MATCH($P17,Summary!$B$6:$B$8,0)),0)</f>
         <v>110</v>
       </c>
-      <c r="V17" s="25" t="n">
+      <c r="V17" s="30" t="n">
         <f aca="false">IF(AND($K17="Y",$F17&lt;&gt;"Y",OR($T17="",$T17=Summary!$C$11)),$C17*IF($H17&lt;&gt;"",$H17,$E17)*INDEX(Summary!$C$6:$C$8,MATCH($P17,Summary!$B$6:$B$8,0)),0)</f>
         <v>160</v>
       </c>
@@ -23822,10 +23849,10 @@
       <c r="C18" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="21" t="n">
+      <c r="D18" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="E18" s="21" t="n">
+      <c r="E18" s="27" t="n">
         <v>65</v>
       </c>
       <c r="F18" s="20" t="s">
@@ -23834,8 +23861,8 @@
       <c r="G18" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H18" s="22"/>
-      <c r="I18" s="23" t="n">
+      <c r="H18" s="28"/>
+      <c r="I18" s="29" t="n">
         <f aca="false">IF(AND($K18="Y",$F18&lt;&gt;"Y",OR($T18="",$T18=Summary!$C$11)),$C18*IF($H18&lt;&gt;"",$H18,($D18+$E18)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P18,Summary!$B$6:$B$8,0)),0)</f>
         <v>55</v>
       </c>
@@ -23870,11 +23897,11 @@
         <v>924</v>
       </c>
       <c r="T18" s="18"/>
-      <c r="U18" s="25" t="n">
+      <c r="U18" s="30" t="n">
         <f aca="false">IF(AND($K18="Y",$F18&lt;&gt;"Y",OR($T18="",$T18=Summary!$C$11)),$C18*IF($H18&lt;&gt;"",$H18,$D18)*INDEX(Summary!$C$6:$C$8,MATCH($P18,Summary!$B$6:$B$8,0)),0)</f>
         <v>45</v>
       </c>
-      <c r="V18" s="25" t="n">
+      <c r="V18" s="30" t="n">
         <f aca="false">IF(AND($K18="Y",$F18&lt;&gt;"Y",OR($T18="",$T18=Summary!$C$11)),$C18*IF($H18&lt;&gt;"",$H18,$E18)*INDEX(Summary!$C$6:$C$8,MATCH($P18,Summary!$B$6:$B$8,0)),0)</f>
         <v>65</v>
       </c>
@@ -23895,10 +23922,10 @@
       <c r="C19" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="21" t="n">
+      <c r="D19" s="27" t="n">
         <v>37.58</v>
       </c>
-      <c r="E19" s="21" t="n">
+      <c r="E19" s="27" t="n">
         <v>38.99</v>
       </c>
       <c r="F19" s="20" t="s">
@@ -23907,8 +23934,8 @@
       <c r="G19" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H19" s="22"/>
-      <c r="I19" s="23" t="n">
+      <c r="H19" s="28"/>
+      <c r="I19" s="29" t="n">
         <f aca="false">IF(AND($K19="Y",$F19&lt;&gt;"Y",OR($T19="",$T19=Summary!$C$11)),$C19*IF($H19&lt;&gt;"",$H19,($D19+$E19)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P19,Summary!$B$6:$B$8,0)),0)</f>
         <v>38.285</v>
       </c>
@@ -23943,11 +23970,11 @@
         <v>924</v>
       </c>
       <c r="T19" s="18"/>
-      <c r="U19" s="25" t="n">
+      <c r="U19" s="30" t="n">
         <f aca="false">IF(AND($K19="Y",$F19&lt;&gt;"Y",OR($T19="",$T19=Summary!$C$11)),$C19*IF($H19&lt;&gt;"",$H19,$D19)*INDEX(Summary!$C$6:$C$8,MATCH($P19,Summary!$B$6:$B$8,0)),0)</f>
         <v>37.58</v>
       </c>
-      <c r="V19" s="25" t="n">
+      <c r="V19" s="30" t="n">
         <f aca="false">IF(AND($K19="Y",$F19&lt;&gt;"Y",OR($T19="",$T19=Summary!$C$11)),$C19*IF($H19&lt;&gt;"",$H19,$E19)*INDEX(Summary!$C$6:$C$8,MATCH($P19,Summary!$B$6:$B$8,0)),0)</f>
         <v>38.99</v>
       </c>
@@ -23968,10 +23995,10 @@
       <c r="C20" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="21" t="n">
+      <c r="D20" s="27" t="n">
         <v>10.58</v>
       </c>
-      <c r="E20" s="21" t="n">
+      <c r="E20" s="27" t="n">
         <v>24.99</v>
       </c>
       <c r="F20" s="20" t="s">
@@ -23980,8 +24007,8 @@
       <c r="G20" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H20" s="22"/>
-      <c r="I20" s="23" t="n">
+      <c r="H20" s="28"/>
+      <c r="I20" s="29" t="n">
         <f aca="false">IF(AND($K20="Y",$F20&lt;&gt;"Y",OR($T20="",$T20=Summary!$C$11)),$C20*IF($H20&lt;&gt;"",$H20,($D20+$E20)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P20,Summary!$B$6:$B$8,0)),0)</f>
         <v>71.14</v>
       </c>
@@ -24016,11 +24043,11 @@
         <v>924</v>
       </c>
       <c r="T20" s="18"/>
-      <c r="U20" s="25" t="n">
+      <c r="U20" s="30" t="n">
         <f aca="false">IF(AND($K20="Y",$F20&lt;&gt;"Y",OR($T20="",$T20=Summary!$C$11)),$C20*IF($H20&lt;&gt;"",$H20,$D20)*INDEX(Summary!$C$6:$C$8,MATCH($P20,Summary!$B$6:$B$8,0)),0)</f>
         <v>42.32</v>
       </c>
-      <c r="V20" s="25" t="n">
+      <c r="V20" s="30" t="n">
         <f aca="false">IF(AND($K20="Y",$F20&lt;&gt;"Y",OR($T20="",$T20=Summary!$C$11)),$C20*IF($H20&lt;&gt;"",$H20,$E20)*INDEX(Summary!$C$6:$C$8,MATCH($P20,Summary!$B$6:$B$8,0)),0)</f>
         <v>99.96</v>
       </c>
@@ -24041,10 +24068,10 @@
       <c r="C21" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="27" t="n">
         <v>1.5</v>
       </c>
-      <c r="E21" s="21" t="n">
+      <c r="E21" s="27" t="n">
         <v>2.1</v>
       </c>
       <c r="F21" s="20" t="s">
@@ -24053,8 +24080,8 @@
       <c r="G21" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H21" s="22"/>
-      <c r="I21" s="23" t="n">
+      <c r="H21" s="28"/>
+      <c r="I21" s="29" t="n">
         <f aca="false">IF(AND($K21="Y",$F21&lt;&gt;"Y",OR($T21="",$T21=Summary!$C$11)),$C21*IF($H21&lt;&gt;"",$H21,($D21+$E21)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P21,Summary!$B$6:$B$8,0)),0)</f>
         <v>7.2</v>
       </c>
@@ -24089,11 +24116,11 @@
         <v>924</v>
       </c>
       <c r="T21" s="18"/>
-      <c r="U21" s="25" t="n">
+      <c r="U21" s="30" t="n">
         <f aca="false">IF(AND($K21="Y",$F21&lt;&gt;"Y",OR($T21="",$T21=Summary!$C$11)),$C21*IF($H21&lt;&gt;"",$H21,$D21)*INDEX(Summary!$C$6:$C$8,MATCH($P21,Summary!$B$6:$B$8,0)),0)</f>
         <v>6</v>
       </c>
-      <c r="V21" s="25" t="n">
+      <c r="V21" s="30" t="n">
         <f aca="false">IF(AND($K21="Y",$F21&lt;&gt;"Y",OR($T21="",$T21=Summary!$C$11)),$C21*IF($H21&lt;&gt;"",$H21,$E21)*INDEX(Summary!$C$6:$C$8,MATCH($P21,Summary!$B$6:$B$8,0)),0)</f>
         <v>8.4</v>
       </c>
@@ -24114,10 +24141,10 @@
       <c r="C22" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="21" t="n">
+      <c r="D22" s="27" t="n">
         <v>1.73</v>
       </c>
-      <c r="E22" s="21" t="n">
+      <c r="E22" s="27" t="n">
         <v>3</v>
       </c>
       <c r="F22" s="20" t="s">
@@ -24126,8 +24153,8 @@
       <c r="G22" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H22" s="22"/>
-      <c r="I22" s="23" t="n">
+      <c r="H22" s="28"/>
+      <c r="I22" s="29" t="n">
         <f aca="false">IF(AND($K22="Y",$F22&lt;&gt;"Y",OR($T22="",$T22=Summary!$C$11)),$C22*IF($H22&lt;&gt;"",$H22,($D22+$E22)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P22,Summary!$B$6:$B$8,0)),0)</f>
         <v>9.46</v>
       </c>
@@ -24162,11 +24189,11 @@
         <v>924</v>
       </c>
       <c r="T22" s="18"/>
-      <c r="U22" s="25" t="n">
+      <c r="U22" s="30" t="n">
         <f aca="false">IF(AND($K22="Y",$F22&lt;&gt;"Y",OR($T22="",$T22=Summary!$C$11)),$C22*IF($H22&lt;&gt;"",$H22,$D22)*INDEX(Summary!$C$6:$C$8,MATCH($P22,Summary!$B$6:$B$8,0)),0)</f>
         <v>6.92</v>
       </c>
-      <c r="V22" s="25" t="n">
+      <c r="V22" s="30" t="n">
         <f aca="false">IF(AND($K22="Y",$F22&lt;&gt;"Y",OR($T22="",$T22=Summary!$C$11)),$C22*IF($H22&lt;&gt;"",$H22,$E22)*INDEX(Summary!$C$6:$C$8,MATCH($P22,Summary!$B$6:$B$8,0)),0)</f>
         <v>12</v>
       </c>
@@ -24187,10 +24214,10 @@
       <c r="C23" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D23" s="21" t="n">
+      <c r="D23" s="27" t="n">
         <v>2.5</v>
       </c>
-      <c r="E23" s="21" t="n">
+      <c r="E23" s="27" t="n">
         <v>4</v>
       </c>
       <c r="F23" s="20" t="s">
@@ -24199,8 +24226,8 @@
       <c r="G23" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H23" s="22"/>
-      <c r="I23" s="23" t="n">
+      <c r="H23" s="28"/>
+      <c r="I23" s="29" t="n">
         <f aca="false">IF(AND($K23="Y",$F23&lt;&gt;"Y",OR($T23="",$T23=Summary!$C$11)),$C23*IF($H23&lt;&gt;"",$H23,($D23+$E23)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P23,Summary!$B$6:$B$8,0)),0)</f>
         <v>13</v>
       </c>
@@ -24235,11 +24262,11 @@
         <v>924</v>
       </c>
       <c r="T23" s="18"/>
-      <c r="U23" s="25" t="n">
+      <c r="U23" s="30" t="n">
         <f aca="false">IF(AND($K23="Y",$F23&lt;&gt;"Y",OR($T23="",$T23=Summary!$C$11)),$C23*IF($H23&lt;&gt;"",$H23,$D23)*INDEX(Summary!$C$6:$C$8,MATCH($P23,Summary!$B$6:$B$8,0)),0)</f>
         <v>10</v>
       </c>
-      <c r="V23" s="25" t="n">
+      <c r="V23" s="30" t="n">
         <f aca="false">IF(AND($K23="Y",$F23&lt;&gt;"Y",OR($T23="",$T23=Summary!$C$11)),$C23*IF($H23&lt;&gt;"",$H23,$E23)*INDEX(Summary!$C$6:$C$8,MATCH($P23,Summary!$B$6:$B$8,0)),0)</f>
         <v>16</v>
       </c>
@@ -24260,18 +24287,18 @@
       <c r="C24" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
       <c r="F24" s="20" t="s">
         <v>103</v>
       </c>
       <c r="G24" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H24" s="22" t="n">
+      <c r="H24" s="28" t="n">
         <v>185</v>
       </c>
-      <c r="I24" s="23" t="n">
+      <c r="I24" s="29" t="n">
         <f aca="false">IF(AND($K24="Y",$F24&lt;&gt;"Y",OR($T24="",$T24=Summary!$C$11)),$C24*IF($H24&lt;&gt;"",$H24,($D24+$E24)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P24,Summary!$B$6:$B$8,0)),0)</f>
         <v>185</v>
       </c>
@@ -24306,11 +24333,11 @@
         <v>924</v>
       </c>
       <c r="T24" s="18"/>
-      <c r="U24" s="25" t="n">
+      <c r="U24" s="30" t="n">
         <f aca="false">IF(AND($K24="Y",$F24&lt;&gt;"Y",OR($T24="",$T24=Summary!$C$11)),$C24*IF($H24&lt;&gt;"",$H24,$D24)*INDEX(Summary!$C$6:$C$8,MATCH($P24,Summary!$B$6:$B$8,0)),0)</f>
         <v>185</v>
       </c>
-      <c r="V24" s="25" t="n">
+      <c r="V24" s="30" t="n">
         <f aca="false">IF(AND($K24="Y",$F24&lt;&gt;"Y",OR($T24="",$T24=Summary!$C$11)),$C24*IF($H24&lt;&gt;"",$H24,$E24)*INDEX(Summary!$C$6:$C$8,MATCH($P24,Summary!$B$6:$B$8,0)),0)</f>
         <v>185</v>
       </c>
@@ -24331,16 +24358,16 @@
       <c r="C25" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
       <c r="F25" s="20" t="s">
         <v>105</v>
       </c>
       <c r="G25" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="22"/>
-      <c r="I25" s="23" t="n">
+      <c r="H25" s="28"/>
+      <c r="I25" s="29" t="n">
         <f aca="false">IF(AND($K25="Y",$F25&lt;&gt;"Y",OR($T25="",$T25=Summary!$C$11)),$C25*IF($H25&lt;&gt;"",$H25,($D25+$E25)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P25,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -24375,11 +24402,11 @@
         <v>924</v>
       </c>
       <c r="T25" s="18"/>
-      <c r="U25" s="25" t="n">
+      <c r="U25" s="30" t="n">
         <f aca="false">IF(AND($K25="Y",$F25&lt;&gt;"Y",OR($T25="",$T25=Summary!$C$11)),$C25*IF($H25&lt;&gt;"",$H25,$D25)*INDEX(Summary!$C$6:$C$8,MATCH($P25,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
-      <c r="V25" s="25" t="n">
+      <c r="V25" s="30" t="n">
         <f aca="false">IF(AND($K25="Y",$F25&lt;&gt;"Y",OR($T25="",$T25=Summary!$C$11)),$C25*IF($H25&lt;&gt;"",$H25,$E25)*INDEX(Summary!$C$6:$C$8,MATCH($P25,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -24398,10 +24425,10 @@
       <c r="C26" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="21" t="n">
+      <c r="D26" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="E26" s="21" t="n">
+      <c r="E26" s="27" t="n">
         <v>8.69</v>
       </c>
       <c r="F26" s="20" t="s">
@@ -24410,8 +24437,8 @@
       <c r="G26" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H26" s="22"/>
-      <c r="I26" s="23" t="n">
+      <c r="H26" s="28"/>
+      <c r="I26" s="29" t="n">
         <f aca="false">IF(AND($K26="Y",$F26&lt;&gt;"Y",OR($T26="",$T26=Summary!$C$11)),$C26*IF($H26&lt;&gt;"",$H26,($D26+$E26)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P26,Summary!$B$6:$B$8,0)),0)</f>
         <v>6.345</v>
       </c>
@@ -24446,11 +24473,11 @@
         <v>924</v>
       </c>
       <c r="T26" s="18"/>
-      <c r="U26" s="25" t="n">
+      <c r="U26" s="30" t="n">
         <f aca="false">IF(AND($K26="Y",$F26&lt;&gt;"Y",OR($T26="",$T26=Summary!$C$11)),$C26*IF($H26&lt;&gt;"",$H26,$D26)*INDEX(Summary!$C$6:$C$8,MATCH($P26,Summary!$B$6:$B$8,0)),0)</f>
         <v>4</v>
       </c>
-      <c r="V26" s="25" t="n">
+      <c r="V26" s="30" t="n">
         <f aca="false">IF(AND($K26="Y",$F26&lt;&gt;"Y",OR($T26="",$T26=Summary!$C$11)),$C26*IF($H26&lt;&gt;"",$H26,$E26)*INDEX(Summary!$C$6:$C$8,MATCH($P26,Summary!$B$6:$B$8,0)),0)</f>
         <v>8.69</v>
       </c>
@@ -24471,10 +24498,10 @@
       <c r="C27" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="D27" s="21" t="n">
+      <c r="D27" s="27" t="n">
         <v>1.07</v>
       </c>
-      <c r="E27" s="21" t="n">
+      <c r="E27" s="27" t="n">
         <v>4.2</v>
       </c>
       <c r="F27" s="20" t="s">
@@ -24483,8 +24510,8 @@
       <c r="G27" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H27" s="22"/>
-      <c r="I27" s="23" t="n">
+      <c r="H27" s="28"/>
+      <c r="I27" s="29" t="n">
         <f aca="false">IF(AND($K27="Y",$F27&lt;&gt;"Y",OR($T27="",$T27=Summary!$C$11)),$C27*IF($H27&lt;&gt;"",$H27,($D27+$E27)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P27,Summary!$B$6:$B$8,0)),0)</f>
         <v>15.81</v>
       </c>
@@ -24519,11 +24546,11 @@
         <v>924</v>
       </c>
       <c r="T27" s="18"/>
-      <c r="U27" s="25" t="n">
+      <c r="U27" s="30" t="n">
         <f aca="false">IF(AND($K27="Y",$F27&lt;&gt;"Y",OR($T27="",$T27=Summary!$C$11)),$C27*IF($H27&lt;&gt;"",$H27,$D27)*INDEX(Summary!$C$6:$C$8,MATCH($P27,Summary!$B$6:$B$8,0)),0)</f>
         <v>6.42</v>
       </c>
-      <c r="V27" s="25" t="n">
+      <c r="V27" s="30" t="n">
         <f aca="false">IF(AND($K27="Y",$F27&lt;&gt;"Y",OR($T27="",$T27=Summary!$C$11)),$C27*IF($H27&lt;&gt;"",$H27,$E27)*INDEX(Summary!$C$6:$C$8,MATCH($P27,Summary!$B$6:$B$8,0)),0)</f>
         <v>25.2</v>
       </c>
@@ -24544,10 +24571,10 @@
       <c r="C28" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="21" t="n">
+      <c r="D28" s="27" t="n">
         <v>2.48</v>
       </c>
-      <c r="E28" s="21" t="n">
+      <c r="E28" s="27" t="n">
         <v>5.89</v>
       </c>
       <c r="F28" s="20" t="s">
@@ -24556,8 +24583,8 @@
       <c r="G28" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H28" s="22"/>
-      <c r="I28" s="23" t="n">
+      <c r="H28" s="28"/>
+      <c r="I28" s="29" t="n">
         <f aca="false">IF(AND($K28="Y",$F28&lt;&gt;"Y",OR($T28="",$T28=Summary!$C$11)),$C28*IF($H28&lt;&gt;"",$H28,($D28+$E28)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P28,Summary!$B$6:$B$8,0)),0)</f>
         <v>4.185</v>
       </c>
@@ -24592,11 +24619,11 @@
         <v>924</v>
       </c>
       <c r="T28" s="18"/>
-      <c r="U28" s="25" t="n">
+      <c r="U28" s="30" t="n">
         <f aca="false">IF(AND($K28="Y",$F28&lt;&gt;"Y",OR($T28="",$T28=Summary!$C$11)),$C28*IF($H28&lt;&gt;"",$H28,$D28)*INDEX(Summary!$C$6:$C$8,MATCH($P28,Summary!$B$6:$B$8,0)),0)</f>
         <v>2.48</v>
       </c>
-      <c r="V28" s="25" t="n">
+      <c r="V28" s="30" t="n">
         <f aca="false">IF(AND($K28="Y",$F28&lt;&gt;"Y",OR($T28="",$T28=Summary!$C$11)),$C28*IF($H28&lt;&gt;"",$H28,$E28)*INDEX(Summary!$C$6:$C$8,MATCH($P28,Summary!$B$6:$B$8,0)),0)</f>
         <v>5.89</v>
       </c>
@@ -24617,10 +24644,10 @@
       <c r="C29" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="D29" s="21" t="n">
+      <c r="D29" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="21" t="n">
+      <c r="E29" s="27" t="n">
         <v>2</v>
       </c>
       <c r="F29" s="20" t="s">
@@ -24629,8 +24656,8 @@
       <c r="G29" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H29" s="22"/>
-      <c r="I29" s="23" t="n">
+      <c r="H29" s="28"/>
+      <c r="I29" s="29" t="n">
         <f aca="false">IF(AND($K29="Y",$F29&lt;&gt;"Y",OR($T29="",$T29=Summary!$C$11)),$C29*IF($H29&lt;&gt;"",$H29,($D29+$E29)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P29,Summary!$B$6:$B$8,0)),0)</f>
         <v>22.5</v>
       </c>
@@ -24665,11 +24692,11 @@
         <v>924</v>
       </c>
       <c r="T29" s="18"/>
-      <c r="U29" s="25" t="n">
+      <c r="U29" s="30" t="n">
         <f aca="false">IF(AND($K29="Y",$F29&lt;&gt;"Y",OR($T29="",$T29=Summary!$C$11)),$C29*IF($H29&lt;&gt;"",$H29,$D29)*INDEX(Summary!$C$6:$C$8,MATCH($P29,Summary!$B$6:$B$8,0)),0)</f>
         <v>15</v>
       </c>
-      <c r="V29" s="25" t="n">
+      <c r="V29" s="30" t="n">
         <f aca="false">IF(AND($K29="Y",$F29&lt;&gt;"Y",OR($T29="",$T29=Summary!$C$11)),$C29*IF($H29&lt;&gt;"",$H29,$E29)*INDEX(Summary!$C$6:$C$8,MATCH($P29,Summary!$B$6:$B$8,0)),0)</f>
         <v>30</v>
       </c>
@@ -24690,10 +24717,10 @@
       <c r="C30" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="D30" s="21" t="n">
+      <c r="D30" s="27" t="n">
         <v>0.8</v>
       </c>
-      <c r="E30" s="21" t="n">
+      <c r="E30" s="27" t="n">
         <v>1.5</v>
       </c>
       <c r="F30" s="20" t="s">
@@ -24702,8 +24729,8 @@
       <c r="G30" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H30" s="22"/>
-      <c r="I30" s="23" t="n">
+      <c r="H30" s="28"/>
+      <c r="I30" s="29" t="n">
         <f aca="false">IF(AND($K30="Y",$F30&lt;&gt;"Y",OR($T30="",$T30=Summary!$C$11)),$C30*IF($H30&lt;&gt;"",$H30,($D30+$E30)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P30,Summary!$B$6:$B$8,0)),0)</f>
         <v>11.5</v>
       </c>
@@ -24738,11 +24765,11 @@
         <v>924</v>
       </c>
       <c r="T30" s="18"/>
-      <c r="U30" s="25" t="n">
+      <c r="U30" s="30" t="n">
         <f aca="false">IF(AND($K30="Y",$F30&lt;&gt;"Y",OR($T30="",$T30=Summary!$C$11)),$C30*IF($H30&lt;&gt;"",$H30,$D30)*INDEX(Summary!$C$6:$C$8,MATCH($P30,Summary!$B$6:$B$8,0)),0)</f>
         <v>8</v>
       </c>
-      <c r="V30" s="25" t="n">
+      <c r="V30" s="30" t="n">
         <f aca="false">IF(AND($K30="Y",$F30&lt;&gt;"Y",OR($T30="",$T30=Summary!$C$11)),$C30*IF($H30&lt;&gt;"",$H30,$E30)*INDEX(Summary!$C$6:$C$8,MATCH($P30,Summary!$B$6:$B$8,0)),0)</f>
         <v>15</v>
       </c>
@@ -24763,10 +24790,10 @@
       <c r="C31" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D31" s="21" t="n">
+      <c r="D31" s="27" t="n">
         <v>3.5</v>
       </c>
-      <c r="E31" s="21" t="n">
+      <c r="E31" s="27" t="n">
         <v>4.45</v>
       </c>
       <c r="F31" s="20" t="s">
@@ -24775,8 +24802,8 @@
       <c r="G31" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H31" s="22"/>
-      <c r="I31" s="23" t="n">
+      <c r="H31" s="28"/>
+      <c r="I31" s="29" t="n">
         <f aca="false">IF(AND($K31="Y",$F31&lt;&gt;"Y",OR($T31="",$T31=Summary!$C$11)),$C31*IF($H31&lt;&gt;"",$H31,($D31+$E31)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P31,Summary!$B$6:$B$8,0)),0)</f>
         <v>7.95</v>
       </c>
@@ -24811,11 +24838,11 @@
         <v>924</v>
       </c>
       <c r="T31" s="18"/>
-      <c r="U31" s="25" t="n">
+      <c r="U31" s="30" t="n">
         <f aca="false">IF(AND($K31="Y",$F31&lt;&gt;"Y",OR($T31="",$T31=Summary!$C$11)),$C31*IF($H31&lt;&gt;"",$H31,$D31)*INDEX(Summary!$C$6:$C$8,MATCH($P31,Summary!$B$6:$B$8,0)),0)</f>
         <v>7</v>
       </c>
-      <c r="V31" s="25" t="n">
+      <c r="V31" s="30" t="n">
         <f aca="false">IF(AND($K31="Y",$F31&lt;&gt;"Y",OR($T31="",$T31=Summary!$C$11)),$C31*IF($H31&lt;&gt;"",$H31,$E31)*INDEX(Summary!$C$6:$C$8,MATCH($P31,Summary!$B$6:$B$8,0)),0)</f>
         <v>8.9</v>
       </c>
@@ -24836,10 +24863,10 @@
       <c r="C32" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="21" t="n">
+      <c r="D32" s="27" t="n">
         <v>17.39</v>
       </c>
-      <c r="E32" s="21" t="n">
+      <c r="E32" s="27" t="n">
         <v>30</v>
       </c>
       <c r="F32" s="20" t="s">
@@ -24848,8 +24875,8 @@
       <c r="G32" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H32" s="22"/>
-      <c r="I32" s="23" t="n">
+      <c r="H32" s="28"/>
+      <c r="I32" s="29" t="n">
         <f aca="false">IF(AND($K32="Y",$F32&lt;&gt;"Y",OR($T32="",$T32=Summary!$C$11)),$C32*IF($H32&lt;&gt;"",$H32,($D32+$E32)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P32,Summary!$B$6:$B$8,0)),0)</f>
         <v>23.695</v>
       </c>
@@ -24884,11 +24911,11 @@
         <v>924</v>
       </c>
       <c r="T32" s="18"/>
-      <c r="U32" s="25" t="n">
+      <c r="U32" s="30" t="n">
         <f aca="false">IF(AND($K32="Y",$F32&lt;&gt;"Y",OR($T32="",$T32=Summary!$C$11)),$C32*IF($H32&lt;&gt;"",$H32,$D32)*INDEX(Summary!$C$6:$C$8,MATCH($P32,Summary!$B$6:$B$8,0)),0)</f>
         <v>17.39</v>
       </c>
-      <c r="V32" s="25" t="n">
+      <c r="V32" s="30" t="n">
         <f aca="false">IF(AND($K32="Y",$F32&lt;&gt;"Y",OR($T32="",$T32=Summary!$C$11)),$C32*IF($H32&lt;&gt;"",$H32,$E32)*INDEX(Summary!$C$6:$C$8,MATCH($P32,Summary!$B$6:$B$8,0)),0)</f>
         <v>30</v>
       </c>
@@ -24909,10 +24936,10 @@
       <c r="C33" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="21" t="n">
+      <c r="D33" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E33" s="21" t="n">
+      <c r="E33" s="27" t="n">
         <v>15</v>
       </c>
       <c r="F33" s="20" t="s">
@@ -24921,8 +24948,8 @@
       <c r="G33" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H33" s="22"/>
-      <c r="I33" s="23" t="n">
+      <c r="H33" s="28"/>
+      <c r="I33" s="29" t="n">
         <f aca="false">IF(AND($K33="Y",$F33&lt;&gt;"Y",OR($T33="",$T33=Summary!$C$11)),$C33*IF($H33&lt;&gt;"",$H33,($D33+$E33)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P33,Summary!$B$6:$B$8,0)),0)</f>
         <v>7.5</v>
       </c>
@@ -24957,11 +24984,11 @@
         <v>924</v>
       </c>
       <c r="T33" s="18"/>
-      <c r="U33" s="25" t="n">
+      <c r="U33" s="30" t="n">
         <f aca="false">IF(AND($K33="Y",$F33&lt;&gt;"Y",OR($T33="",$T33=Summary!$C$11)),$C33*IF($H33&lt;&gt;"",$H33,$D33)*INDEX(Summary!$C$6:$C$8,MATCH($P33,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
-      <c r="V33" s="25" t="n">
+      <c r="V33" s="30" t="n">
         <f aca="false">IF(AND($K33="Y",$F33&lt;&gt;"Y",OR($T33="",$T33=Summary!$C$11)),$C33*IF($H33&lt;&gt;"",$H33,$E33)*INDEX(Summary!$C$6:$C$8,MATCH($P33,Summary!$B$6:$B$8,0)),0)</f>
         <v>15</v>
       </c>
@@ -24982,10 +25009,10 @@
       <c r="C34" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D34" s="21" t="n">
+      <c r="D34" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="E34" s="21" t="n">
+      <c r="E34" s="27" t="n">
         <v>14</v>
       </c>
       <c r="F34" s="20" t="s">
@@ -24994,8 +25021,8 @@
       <c r="G34" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H34" s="22"/>
-      <c r="I34" s="23" t="n">
+      <c r="H34" s="28"/>
+      <c r="I34" s="29" t="n">
         <f aca="false">IF(AND($K34="Y",$F34&lt;&gt;"Y",OR($T34="",$T34=Summary!$C$11)),$C34*IF($H34&lt;&gt;"",$H34,($D34+$E34)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P34,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25030,11 +25057,11 @@
         <v>924</v>
       </c>
       <c r="T34" s="18"/>
-      <c r="U34" s="25" t="n">
+      <c r="U34" s="30" t="n">
         <f aca="false">IF(AND($K34="Y",$F34&lt;&gt;"Y",OR($T34="",$T34=Summary!$C$11)),$C34*IF($H34&lt;&gt;"",$H34,$D34)*INDEX(Summary!$C$6:$C$8,MATCH($P34,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
-      <c r="V34" s="25" t="n">
+      <c r="V34" s="30" t="n">
         <f aca="false">IF(AND($K34="Y",$F34&lt;&gt;"Y",OR($T34="",$T34=Summary!$C$11)),$C34*IF($H34&lt;&gt;"",$H34,$E34)*INDEX(Summary!$C$6:$C$8,MATCH($P34,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25055,10 +25082,10 @@
       <c r="C35" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="21" t="n">
+      <c r="D35" s="27" t="n">
         <v>100</v>
       </c>
-      <c r="E35" s="21" t="n">
+      <c r="E35" s="27" t="n">
         <v>140</v>
       </c>
       <c r="F35" s="20" t="s">
@@ -25067,8 +25094,8 @@
       <c r="G35" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H35" s="22"/>
-      <c r="I35" s="23" t="n">
+      <c r="H35" s="28"/>
+      <c r="I35" s="29" t="n">
         <f aca="false">IF(AND($K35="Y",$F35&lt;&gt;"Y",OR($T35="",$T35=Summary!$C$11)),$C35*IF($H35&lt;&gt;"",$H35,($D35+$E35)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P35,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25103,11 +25130,11 @@
         <v>924</v>
       </c>
       <c r="T35" s="18"/>
-      <c r="U35" s="25" t="n">
+      <c r="U35" s="30" t="n">
         <f aca="false">IF(AND($K35="Y",$F35&lt;&gt;"Y",OR($T35="",$T35=Summary!$C$11)),$C35*IF($H35&lt;&gt;"",$H35,$D35)*INDEX(Summary!$C$6:$C$8,MATCH($P35,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
-      <c r="V35" s="25" t="n">
+      <c r="V35" s="30" t="n">
         <f aca="false">IF(AND($K35="Y",$F35&lt;&gt;"Y",OR($T35="",$T35=Summary!$C$11)),$C35*IF($H35&lt;&gt;"",$H35,$E35)*INDEX(Summary!$C$6:$C$8,MATCH($P35,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25128,10 +25155,10 @@
       <c r="C36" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D36" s="21" t="n">
+      <c r="D36" s="27" t="n">
         <v>80</v>
       </c>
-      <c r="E36" s="21" t="n">
+      <c r="E36" s="27" t="n">
         <v>170</v>
       </c>
       <c r="F36" s="20" t="s">
@@ -25140,8 +25167,8 @@
       <c r="G36" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H36" s="22"/>
-      <c r="I36" s="23" t="n">
+      <c r="H36" s="28"/>
+      <c r="I36" s="29" t="n">
         <f aca="false">IF(AND($K36="Y",$F36&lt;&gt;"Y",OR($T36="",$T36=Summary!$C$11)),$C36*IF($H36&lt;&gt;"",$H36,($D36+$E36)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P36,Summary!$B$6:$B$8,0)),0)</f>
         <v>125</v>
       </c>
@@ -25176,11 +25203,11 @@
         <v>924</v>
       </c>
       <c r="T36" s="18"/>
-      <c r="U36" s="25" t="n">
+      <c r="U36" s="30" t="n">
         <f aca="false">IF(AND($K36="Y",$F36&lt;&gt;"Y",OR($T36="",$T36=Summary!$C$11)),$C36*IF($H36&lt;&gt;"",$H36,$D36)*INDEX(Summary!$C$6:$C$8,MATCH($P36,Summary!$B$6:$B$8,0)),0)</f>
         <v>80</v>
       </c>
-      <c r="V36" s="25" t="n">
+      <c r="V36" s="30" t="n">
         <f aca="false">IF(AND($K36="Y",$F36&lt;&gt;"Y",OR($T36="",$T36=Summary!$C$11)),$C36*IF($H36&lt;&gt;"",$H36,$E36)*INDEX(Summary!$C$6:$C$8,MATCH($P36,Summary!$B$6:$B$8,0)),0)</f>
         <v>170</v>
       </c>
@@ -25201,10 +25228,10 @@
       <c r="C37" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="21" t="n">
+      <c r="D37" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E37" s="21" t="n">
+      <c r="E37" s="27" t="n">
         <v>35</v>
       </c>
       <c r="F37" s="20" t="s">
@@ -25213,8 +25240,8 @@
       <c r="G37" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H37" s="22"/>
-      <c r="I37" s="23" t="n">
+      <c r="H37" s="28"/>
+      <c r="I37" s="29" t="n">
         <f aca="false">IF(AND($K37="Y",$F37&lt;&gt;"Y",OR($T37="",$T37=Summary!$C$11)),$C37*IF($H37&lt;&gt;"",$H37,($D37+$E37)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P37,Summary!$B$6:$B$8,0)),0)</f>
         <v>27.5</v>
       </c>
@@ -25249,11 +25276,11 @@
         <v>924</v>
       </c>
       <c r="T37" s="18"/>
-      <c r="U37" s="25" t="n">
+      <c r="U37" s="30" t="n">
         <f aca="false">IF(AND($K37="Y",$F37&lt;&gt;"Y",OR($T37="",$T37=Summary!$C$11)),$C37*IF($H37&lt;&gt;"",$H37,$D37)*INDEX(Summary!$C$6:$C$8,MATCH($P37,Summary!$B$6:$B$8,0)),0)</f>
         <v>20</v>
       </c>
-      <c r="V37" s="25" t="n">
+      <c r="V37" s="30" t="n">
         <f aca="false">IF(AND($K37="Y",$F37&lt;&gt;"Y",OR($T37="",$T37=Summary!$C$11)),$C37*IF($H37&lt;&gt;"",$H37,$E37)*INDEX(Summary!$C$6:$C$8,MATCH($P37,Summary!$B$6:$B$8,0)),0)</f>
         <v>35</v>
       </c>
@@ -25274,10 +25301,10 @@
       <c r="C38" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D38" s="21" t="n">
+      <c r="D38" s="27" t="n">
         <v>238.68</v>
       </c>
-      <c r="E38" s="21" t="n">
+      <c r="E38" s="27" t="n">
         <v>266.99</v>
       </c>
       <c r="F38" s="20" t="s">
@@ -25286,8 +25313,8 @@
       <c r="G38" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H38" s="22"/>
-      <c r="I38" s="23" t="n">
+      <c r="H38" s="28"/>
+      <c r="I38" s="29" t="n">
         <f aca="false">IF(AND($K38="Y",$F38&lt;&gt;"Y",OR($T38="",$T38=Summary!$C$11)),$C38*IF($H38&lt;&gt;"",$H38,($D38+$E38)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P38,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25322,11 +25349,11 @@
         <v>924</v>
       </c>
       <c r="T38" s="18"/>
-      <c r="U38" s="25" t="n">
+      <c r="U38" s="30" t="n">
         <f aca="false">IF(AND($K38="Y",$F38&lt;&gt;"Y",OR($T38="",$T38=Summary!$C$11)),$C38*IF($H38&lt;&gt;"",$H38,$D38)*INDEX(Summary!$C$6:$C$8,MATCH($P38,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
-      <c r="V38" s="25" t="n">
+      <c r="V38" s="30" t="n">
         <f aca="false">IF(AND($K38="Y",$F38&lt;&gt;"Y",OR($T38="",$T38=Summary!$C$11)),$C38*IF($H38&lt;&gt;"",$H38,$E38)*INDEX(Summary!$C$6:$C$8,MATCH($P38,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25347,10 +25374,10 @@
       <c r="C39" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="21" t="n">
+      <c r="D39" s="27" t="n">
         <v>16.38</v>
       </c>
-      <c r="E39" s="21" t="n">
+      <c r="E39" s="27" t="n">
         <v>23.38</v>
       </c>
       <c r="F39" s="20" t="s">
@@ -25359,8 +25386,8 @@
       <c r="G39" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H39" s="22"/>
-      <c r="I39" s="23" t="n">
+      <c r="H39" s="28"/>
+      <c r="I39" s="29" t="n">
         <f aca="false">IF(AND($K39="Y",$F39&lt;&gt;"Y",OR($T39="",$T39=Summary!$C$11)),$C39*IF($H39&lt;&gt;"",$H39,($D39+$E39)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P39,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25395,11 +25422,11 @@
         <v>924</v>
       </c>
       <c r="T39" s="18"/>
-      <c r="U39" s="25" t="n">
+      <c r="U39" s="30" t="n">
         <f aca="false">IF(AND($K39="Y",$F39&lt;&gt;"Y",OR($T39="",$T39=Summary!$C$11)),$C39*IF($H39&lt;&gt;"",$H39,$D39)*INDEX(Summary!$C$6:$C$8,MATCH($P39,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
-      <c r="V39" s="25" t="n">
+      <c r="V39" s="30" t="n">
         <f aca="false">IF(AND($K39="Y",$F39&lt;&gt;"Y",OR($T39="",$T39=Summary!$C$11)),$C39*IF($H39&lt;&gt;"",$H39,$E39)*INDEX(Summary!$C$6:$C$8,MATCH($P39,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25420,16 +25447,16 @@
       <c r="C40" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
       <c r="F40" s="20" t="s">
         <v>105</v>
       </c>
       <c r="G40" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H40" s="22"/>
-      <c r="I40" s="23" t="n">
+      <c r="H40" s="28"/>
+      <c r="I40" s="29" t="n">
         <f aca="false">IF(AND($K40="Y",$F40&lt;&gt;"Y",OR($T40="",$T40=Summary!$C$11)),$C40*IF($H40&lt;&gt;"",$H40,($D40+$E40)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P40,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25464,11 +25491,11 @@
         <v>924</v>
       </c>
       <c r="T40" s="18"/>
-      <c r="U40" s="25" t="n">
+      <c r="U40" s="30" t="n">
         <f aca="false">IF(AND($K40="Y",$F40&lt;&gt;"Y",OR($T40="",$T40=Summary!$C$11)),$C40*IF($H40&lt;&gt;"",$H40,$D40)*INDEX(Summary!$C$6:$C$8,MATCH($P40,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
-      <c r="V40" s="25" t="n">
+      <c r="V40" s="30" t="n">
         <f aca="false">IF(AND($K40="Y",$F40&lt;&gt;"Y",OR($T40="",$T40=Summary!$C$11)),$C40*IF($H40&lt;&gt;"",$H40,$E40)*INDEX(Summary!$C$6:$C$8,MATCH($P40,Summary!$B$6:$B$8,0)),0)</f>
         <v>0</v>
       </c>
@@ -25487,10 +25514,10 @@
       <c r="C41" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="21" t="n">
+      <c r="D41" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="E41" s="21" t="n">
+      <c r="E41" s="27" t="n">
         <v>35</v>
       </c>
       <c r="F41" s="20" t="s">
@@ -25499,8 +25526,8 @@
       <c r="G41" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H41" s="22"/>
-      <c r="I41" s="23" t="n">
+      <c r="H41" s="28"/>
+      <c r="I41" s="29" t="n">
         <f aca="false">IF(AND($K41="Y",$F41&lt;&gt;"Y",OR($T41="",$T41=Summary!$C$11)),$C41*IF($H41&lt;&gt;"",$H41,($D41+$E41)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P41,Summary!$B$6:$B$8,0)),0)</f>
         <v>25</v>
       </c>
@@ -25535,11 +25562,11 @@
         <v>924</v>
       </c>
       <c r="T41" s="18"/>
-      <c r="U41" s="25" t="n">
+      <c r="U41" s="30" t="n">
         <f aca="false">IF(AND($K41="Y",$F41&lt;&gt;"Y",OR($T41="",$T41=Summary!$C$11)),$C41*IF($H41&lt;&gt;"",$H41,$D41)*INDEX(Summary!$C$6:$C$8,MATCH($P41,Summary!$B$6:$B$8,0)),0)</f>
         <v>15</v>
       </c>
-      <c r="V41" s="25" t="n">
+      <c r="V41" s="30" t="n">
         <f aca="false">IF(AND($K41="Y",$F41&lt;&gt;"Y",OR($T41="",$T41=Summary!$C$11)),$C41*IF($H41&lt;&gt;"",$H41,$E41)*INDEX(Summary!$C$6:$C$8,MATCH($P41,Summary!$B$6:$B$8,0)),0)</f>
         <v>35</v>
       </c>
@@ -25560,10 +25587,10 @@
       <c r="C42" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D42" s="21" t="n">
+      <c r="D42" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="E42" s="21" t="n">
+      <c r="E42" s="27" t="n">
         <v>60</v>
       </c>
       <c r="F42" s="20" t="s">
@@ -25572,8 +25599,8 @@
       <c r="G42" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H42" s="22"/>
-      <c r="I42" s="23" t="n">
+      <c r="H42" s="28"/>
+      <c r="I42" s="29" t="n">
         <f aca="false">IF(AND($K42="Y",$F42&lt;&gt;"Y",OR($T42="",$T42=Summary!$C$11)),$C42*IF($H42&lt;&gt;"",$H42,($D42+$E42)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P42,Summary!$B$6:$B$8,0)),0)</f>
         <v>42.5</v>
       </c>
@@ -25608,11 +25635,11 @@
         <v>924</v>
       </c>
       <c r="T42" s="18"/>
-      <c r="U42" s="25" t="n">
+      <c r="U42" s="30" t="n">
         <f aca="false">IF(AND($K42="Y",$F42&lt;&gt;"Y",OR($T42="",$T42=Summary!$C$11)),$C42*IF($H42&lt;&gt;"",$H42,$D42)*INDEX(Summary!$C$6:$C$8,MATCH($P42,Summary!$B$6:$B$8,0)),0)</f>
         <v>25</v>
       </c>
-      <c r="V42" s="25" t="n">
+      <c r="V42" s="30" t="n">
         <f aca="false">IF(AND($K42="Y",$F42&lt;&gt;"Y",OR($T42="",$T42=Summary!$C$11)),$C42*IF($H42&lt;&gt;"",$H42,$E42)*INDEX(Summary!$C$6:$C$8,MATCH($P42,Summary!$B$6:$B$8,0)),0)</f>
         <v>60</v>
       </c>
@@ -25633,10 +25660,10 @@
       <c r="C43" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D43" s="21" t="n">
+      <c r="D43" s="27" t="n">
         <v>10.85</v>
       </c>
-      <c r="E43" s="21" t="n">
+      <c r="E43" s="27" t="n">
         <v>15</v>
       </c>
       <c r="F43" s="20" t="s">
@@ -25645,8 +25672,8 @@
       <c r="G43" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H43" s="22"/>
-      <c r="I43" s="23" t="n">
+      <c r="H43" s="28"/>
+      <c r="I43" s="29" t="n">
         <f aca="false">IF(AND($K43="Y",$F43&lt;&gt;"Y",OR($T43="",$T43=Summary!$C$11)),$C43*IF($H43&lt;&gt;"",$H43,($D43+$E43)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P43,Summary!$B$6:$B$8,0)),0)</f>
         <v>12.925</v>
       </c>
@@ -25681,11 +25708,11 @@
         <v>924</v>
       </c>
       <c r="T43" s="18"/>
-      <c r="U43" s="25" t="n">
+      <c r="U43" s="30" t="n">
         <f aca="false">IF(AND($K43="Y",$F43&lt;&gt;"Y",OR($T43="",$T43=Summary!$C$11)),$C43*IF($H43&lt;&gt;"",$H43,$D43)*INDEX(Summary!$C$6:$C$8,MATCH($P43,Summary!$B$6:$B$8,0)),0)</f>
         <v>10.85</v>
       </c>
-      <c r="V43" s="25" t="n">
+      <c r="V43" s="30" t="n">
         <f aca="false">IF(AND($K43="Y",$F43&lt;&gt;"Y",OR($T43="",$T43=Summary!$C$11)),$C43*IF($H43&lt;&gt;"",$H43,$E43)*INDEX(Summary!$C$6:$C$8,MATCH($P43,Summary!$B$6:$B$8,0)),0)</f>
         <v>15</v>
       </c>
@@ -25706,10 +25733,10 @@
       <c r="C44" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="21" t="n">
+      <c r="D44" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="E44" s="21" t="n">
+      <c r="E44" s="27" t="n">
         <v>25</v>
       </c>
       <c r="F44" s="20" t="s">
@@ -25718,8 +25745,8 @@
       <c r="G44" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H44" s="22"/>
-      <c r="I44" s="23" t="n">
+      <c r="H44" s="28"/>
+      <c r="I44" s="29" t="n">
         <f aca="false">IF(AND($K44="Y",$F44&lt;&gt;"Y",OR($T44="",$T44=Summary!$C$11)),$C44*IF($H44&lt;&gt;"",$H44,($D44+$E44)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P44,Summary!$B$6:$B$8,0)),0)</f>
         <v>17.5</v>
       </c>
@@ -25754,11 +25781,11 @@
         <v>924</v>
       </c>
       <c r="T44" s="18"/>
-      <c r="U44" s="25" t="n">
+      <c r="U44" s="30" t="n">
         <f aca="false">IF(AND($K44="Y",$F44&lt;&gt;"Y",OR($T44="",$T44=Summary!$C$11)),$C44*IF($H44&lt;&gt;"",$H44,$D44)*INDEX(Summary!$C$6:$C$8,MATCH($P44,Summary!$B$6:$B$8,0)),0)</f>
         <v>10</v>
       </c>
-      <c r="V44" s="25" t="n">
+      <c r="V44" s="30" t="n">
         <f aca="false">IF(AND($K44="Y",$F44&lt;&gt;"Y",OR($T44="",$T44=Summary!$C$11)),$C44*IF($H44&lt;&gt;"",$H44,$E44)*INDEX(Summary!$C$6:$C$8,MATCH($P44,Summary!$B$6:$B$8,0)),0)</f>
         <v>25</v>
       </c>
@@ -25779,10 +25806,10 @@
       <c r="C45" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D45" s="21" t="n">
+      <c r="D45" s="27" t="n">
         <v>5.55</v>
       </c>
-      <c r="E45" s="21" t="n">
+      <c r="E45" s="27" t="n">
         <v>17.09</v>
       </c>
       <c r="F45" s="20" t="s">
@@ -25791,8 +25818,8 @@
       <c r="G45" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H45" s="22"/>
-      <c r="I45" s="23" t="n">
+      <c r="H45" s="28"/>
+      <c r="I45" s="29" t="n">
         <f aca="false">IF(AND($K45="Y",$F45&lt;&gt;"Y",OR($T45="",$T45=Summary!$C$11)),$C45*IF($H45&lt;&gt;"",$H45,($D45+$E45)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P45,Summary!$B$6:$B$8,0)),0)</f>
         <v>22.64</v>
       </c>
@@ -25827,11 +25854,11 @@
         <v>924</v>
       </c>
       <c r="T45" s="18"/>
-      <c r="U45" s="25" t="n">
+      <c r="U45" s="30" t="n">
         <f aca="false">IF(AND($K45="Y",$F45&lt;&gt;"Y",OR($T45="",$T45=Summary!$C$11)),$C45*IF($H45&lt;&gt;"",$H45,$D45)*INDEX(Summary!$C$6:$C$8,MATCH($P45,Summary!$B$6:$B$8,0)),0)</f>
         <v>11.1</v>
       </c>
-      <c r="V45" s="25" t="n">
+      <c r="V45" s="30" t="n">
         <f aca="false">IF(AND($K45="Y",$F45&lt;&gt;"Y",OR($T45="",$T45=Summary!$C$11)),$C45*IF($H45&lt;&gt;"",$H45,$E45)*INDEX(Summary!$C$6:$C$8,MATCH($P45,Summary!$B$6:$B$8,0)),0)</f>
         <v>34.18</v>
       </c>
@@ -25852,10 +25879,10 @@
       <c r="C46" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D46" s="21" t="n">
+      <c r="D46" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="E46" s="21" t="n">
+      <c r="E46" s="27" t="n">
         <v>8.19</v>
       </c>
       <c r="F46" s="20" t="s">
@@ -25864,8 +25891,8 @@
       <c r="G46" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H46" s="22"/>
-      <c r="I46" s="23" t="n">
+      <c r="H46" s="28"/>
+      <c r="I46" s="29" t="n">
         <f aca="false">IF(AND($K46="Y",$F46&lt;&gt;"Y",OR($T46="",$T46=Summary!$C$11)),$C46*IF($H46&lt;&gt;"",$H46,($D46+$E46)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P46,Summary!$B$6:$B$8,0)),0)</f>
         <v>12.19</v>
       </c>
@@ -25900,11 +25927,11 @@
         <v>924</v>
       </c>
       <c r="T46" s="18"/>
-      <c r="U46" s="25" t="n">
+      <c r="U46" s="30" t="n">
         <f aca="false">IF(AND($K46="Y",$F46&lt;&gt;"Y",OR($T46="",$T46=Summary!$C$11)),$C46*IF($H46&lt;&gt;"",$H46,$D46)*INDEX(Summary!$C$6:$C$8,MATCH($P46,Summary!$B$6:$B$8,0)),0)</f>
         <v>8</v>
       </c>
-      <c r="V46" s="25" t="n">
+      <c r="V46" s="30" t="n">
         <f aca="false">IF(AND($K46="Y",$F46&lt;&gt;"Y",OR($T46="",$T46=Summary!$C$11)),$C46*IF($H46&lt;&gt;"",$H46,$E46)*INDEX(Summary!$C$6:$C$8,MATCH($P46,Summary!$B$6:$B$8,0)),0)</f>
         <v>16.38</v>
       </c>
@@ -25925,10 +25952,10 @@
       <c r="C47" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D47" s="21" t="n">
+      <c r="D47" s="27" t="n">
         <v>19.46</v>
       </c>
-      <c r="E47" s="21" t="n">
+      <c r="E47" s="27" t="n">
         <v>22.79</v>
       </c>
       <c r="F47" s="20" t="s">
@@ -25937,8 +25964,8 @@
       <c r="G47" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H47" s="22"/>
-      <c r="I47" s="23" t="n">
+      <c r="H47" s="28"/>
+      <c r="I47" s="29" t="n">
         <f aca="false">IF(AND($K47="Y",$F47&lt;&gt;"Y",OR($T47="",$T47=Summary!$C$11)),$C47*IF($H47&lt;&gt;"",$H47,($D47+$E47)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P47,Summary!$B$6:$B$8,0)),0)</f>
         <v>21.125</v>
       </c>
@@ -25973,11 +26000,11 @@
         <v>924</v>
       </c>
       <c r="T47" s="18"/>
-      <c r="U47" s="25" t="n">
+      <c r="U47" s="30" t="n">
         <f aca="false">IF(AND($K47="Y",$F47&lt;&gt;"Y",OR($T47="",$T47=Summary!$C$11)),$C47*IF($H47&lt;&gt;"",$H47,$D47)*INDEX(Summary!$C$6:$C$8,MATCH($P47,Summary!$B$6:$B$8,0)),0)</f>
         <v>19.46</v>
       </c>
-      <c r="V47" s="25" t="n">
+      <c r="V47" s="30" t="n">
         <f aca="false">IF(AND($K47="Y",$F47&lt;&gt;"Y",OR($T47="",$T47=Summary!$C$11)),$C47*IF($H47&lt;&gt;"",$H47,$E47)*INDEX(Summary!$C$6:$C$8,MATCH($P47,Summary!$B$6:$B$8,0)),0)</f>
         <v>22.79</v>
       </c>
@@ -25998,10 +26025,10 @@
       <c r="C48" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="21" t="n">
+      <c r="D48" s="27" t="n">
         <v>5.39</v>
       </c>
-      <c r="E48" s="21" t="n">
+      <c r="E48" s="27" t="n">
         <v>7.79</v>
       </c>
       <c r="F48" s="20" t="s">
@@ -26010,8 +26037,8 @@
       <c r="G48" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H48" s="22"/>
-      <c r="I48" s="23" t="n">
+      <c r="H48" s="28"/>
+      <c r="I48" s="29" t="n">
         <f aca="false">IF(AND($K48="Y",$F48&lt;&gt;"Y",OR($T48="",$T48=Summary!$C$11)),$C48*IF($H48&lt;&gt;"",$H48,($D48+$E48)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P48,Summary!$B$6:$B$8,0)),0)</f>
         <v>6.59</v>
       </c>
@@ -26046,11 +26073,11 @@
         <v>924</v>
       </c>
       <c r="T48" s="18"/>
-      <c r="U48" s="25" t="n">
+      <c r="U48" s="30" t="n">
         <f aca="false">IF(AND($K48="Y",$F48&lt;&gt;"Y",OR($T48="",$T48=Summary!$C$11)),$C48*IF($H48&lt;&gt;"",$H48,$D48)*INDEX(Summary!$C$6:$C$8,MATCH($P48,Summary!$B$6:$B$8,0)),0)</f>
         <v>5.39</v>
       </c>
-      <c r="V48" s="25" t="n">
+      <c r="V48" s="30" t="n">
         <f aca="false">IF(AND($K48="Y",$F48&lt;&gt;"Y",OR($T48="",$T48=Summary!$C$11)),$C48*IF($H48&lt;&gt;"",$H48,$E48)*INDEX(Summary!$C$6:$C$8,MATCH($P48,Summary!$B$6:$B$8,0)),0)</f>
         <v>7.79</v>
       </c>
@@ -26071,10 +26098,10 @@
       <c r="C49" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D49" s="21" t="n">
+      <c r="D49" s="27" t="n">
         <v>11.78</v>
       </c>
-      <c r="E49" s="21" t="n">
+      <c r="E49" s="27" t="n">
         <v>20</v>
       </c>
       <c r="F49" s="20" t="s">
@@ -26083,8 +26110,8 @@
       <c r="G49" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H49" s="22"/>
-      <c r="I49" s="23" t="n">
+      <c r="H49" s="28"/>
+      <c r="I49" s="29" t="n">
         <f aca="false">IF(AND($K49="Y",$F49&lt;&gt;"Y",OR($T49="",$T49=Summary!$C$11)),$C49*IF($H49&lt;&gt;"",$H49,($D49+$E49)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P49,Summary!$B$6:$B$8,0)),0)</f>
         <v>15.89</v>
       </c>
@@ -26119,11 +26146,11 @@
         <v>924</v>
       </c>
       <c r="T49" s="18"/>
-      <c r="U49" s="25" t="n">
+      <c r="U49" s="30" t="n">
         <f aca="false">IF(AND($K49="Y",$F49&lt;&gt;"Y",OR($T49="",$T49=Summary!$C$11)),$C49*IF($H49&lt;&gt;"",$H49,$D49)*INDEX(Summary!$C$6:$C$8,MATCH($P49,Summary!$B$6:$B$8,0)),0)</f>
         <v>11.78</v>
       </c>
-      <c r="V49" s="25" t="n">
+      <c r="V49" s="30" t="n">
         <f aca="false">IF(AND($K49="Y",$F49&lt;&gt;"Y",OR($T49="",$T49=Summary!$C$11)),$C49*IF($H49&lt;&gt;"",$H49,$E49)*INDEX(Summary!$C$6:$C$8,MATCH($P49,Summary!$B$6:$B$8,0)),0)</f>
         <v>20</v>
       </c>
@@ -26144,10 +26171,10 @@
       <c r="C50" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D50" s="21" t="n">
+      <c r="D50" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="E50" s="21" t="n">
+      <c r="E50" s="27" t="n">
         <v>20</v>
       </c>
       <c r="F50" s="20" t="s">
@@ -26156,8 +26183,8 @@
       <c r="G50" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H50" s="22"/>
-      <c r="I50" s="23" t="n">
+      <c r="H50" s="28"/>
+      <c r="I50" s="29" t="n">
         <f aca="false">IF(AND($K50="Y",$F50&lt;&gt;"Y",OR($T50="",$T50=Summary!$C$11)),$C50*IF($H50&lt;&gt;"",$H50,($D50+$E50)/2)*INDEX(Summary!$C$6:$C$8,MATCH($P50,Summary!$B$6:$B$8,0)),0)</f>
         <v>15</v>
       </c>
@@ -26192,11 +26219,11 @@
         <v>924</v>
       </c>
       <c r="T50" s="18"/>
-      <c r="U50" s="25" t="n">
+      <c r="U50" s="30" t="n">
         <f aca="false">IF(AND($K50="Y",$F50&lt;&gt;"Y",OR($T50="",$T50=Summary!$C$11)),$C50*IF($H50&lt;&gt;"",$H50,$D50)*INDEX(Summary!$C$6:$C$8,MATCH($P50,Summary!$B$6:$B$8,0)),0)</f>
         <v>10</v>
       </c>
-      <c r="V50" s="25" t="n">
+      <c r="V50" s="30" t="n">
         <f aca="false">IF(AND($K50="Y",$F50&lt;&gt;"Y",OR($T50="",$T50=Summary!$C$11)),$C50*IF($H50&lt;&gt;"",$H50,$E50)*INDEX(Summary!$C$6:$C$8,MATCH($P50,Summary!$B$6:$B$8,0)),0)</f>
         <v>20</v>
       </c>
@@ -26208,58 +26235,64 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H51" s="14" t="s">
+      <c r="D51" s="31"/>
+      <c r="E51" s="31"/>
+      <c r="H51" s="32" t="s">
         <v>915</v>
       </c>
-      <c r="I51" s="14" t="n">
+      <c r="I51" s="32" t="n">
         <f aca="false">SUM(I5:I50)</f>
         <v>1576.15</v>
       </c>
-      <c r="U51" s="14" t="n">
+      <c r="U51" s="32" t="n">
         <f aca="false">SUM(U5:U50)</f>
         <v>1252.25</v>
       </c>
-      <c r="V51" s="14" t="n">
+      <c r="V51" s="32" t="n">
         <f aca="false">SUM(V5:V50)</f>
         <v>1900.05</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H52" s="14" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D52" s="31"/>
+      <c r="E52" s="31"/>
+      <c r="H52" s="32" t="s">
         <v>1142</v>
       </c>
-      <c r="I52" s="14" t="n">
+      <c r="I52" s="32" t="n">
         <f aca="false">SUMIFS($I$5:$I$50,$J$5:$J$50,"Ordered")+SUMIFS($I$5:$I$50,$J$5:$J$50,"Done")</f>
         <v>0</v>
       </c>
-      <c r="U52" s="14" t="n">
+      <c r="U52" s="32" t="n">
         <f aca="false">SUMIFS($U$5:$U$50,$J$5:$J$50,"Ordered")+SUMIFS($U$5:$U$50,$J$5:$J$50,"Done")</f>
         <v>0</v>
       </c>
-      <c r="V52" s="14" t="n">
+      <c r="V52" s="32" t="n">
         <f aca="false">SUMIFS($V$5:$V$50,$J$5:$J$50,"Ordered")+SUMIFS($V$5:$V$50,$J$5:$J$50,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H53" s="14" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D53" s="31"/>
+      <c r="E53" s="31"/>
+      <c r="H53" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="I53" s="14" t="n">
+      <c r="I53" s="32" t="n">
         <f aca="false">I51-I52</f>
         <v>1576.15</v>
       </c>
-      <c r="U53" s="14" t="n">
+      <c r="U53" s="32" t="n">
         <f aca="false">U51-U52</f>
         <v>1252.25</v>
       </c>
-      <c r="V53" s="14" t="n">
+      <c r="V53" s="32" t="n">
         <f aca="false">V51-V52</f>
         <v>1900.05</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H54" s="27" t="s">
+    <row r="54" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H54" s="33" t="s">
         <v>1143</v>
       </c>
     </row>
@@ -26373,80 +26406,85 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="120"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="34" t="s">
         <v>1144</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="35" t="s">
         <v>1145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="35" t="s">
         <v>1146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="35" t="s">
         <v>1147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="35" t="s">
         <v>1148</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="35" t="s">
         <v>1149</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="35" t="s">
         <v>1150</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="35" t="s">
         <v>1151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="35" t="s">
         <v>1152</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="35" t="s">
         <v>1153</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="35" t="s">
         <v>1154</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="35" t="s">
         <v>1155</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="35" t="s">
         <v>1156</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="35" t="s">
         <v>1157</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="35" t="s">
+        <v>1158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>